<commit_message>
fix: refine the script
</commit_message>
<xml_diff>
--- a/data/data_check.xlsx
+++ b/data/data_check.xlsx
@@ -481,7 +481,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>2.218580917471212e-05</v>
+        <v>2.33323678683125e-05</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -502,7 +502,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>6.011528859745077e-06</v>
+        <v>6.312111608355086e-06</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -670,7 +670,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1.893864070117199e-07</v>
+        <v>1.988557273623059e-07</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>4.508780194689376e-06</v>
+        <v>4.734219204423844e-06</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -733,7 +733,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>2.621574400000946e-09</v>
+        <v>2.752653120002561e-09</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>2.621574400000946e-09</v>
+        <v>2.752653120002561e-09</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -775,7 +775,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>3.705304e-08</v>
+        <v>3.8905692e-08</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -796,7 +796,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>3.860012e-08</v>
+        <v>4.053012599999999e-08</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -817,7 +817,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>1.850354454027954e-06</v>
+        <v>1.942872176729352e-06</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -838,7 +838,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>3.700714064832671e-06</v>
+        <v>3.885749768074305e-06</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -859,7 +859,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>5.697425788785309e-08</v>
+        <v>5.982297078224262e-08</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -880,7 +880,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>9.384630480482782e-07</v>
+        <v>9.853862004506921e-07</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -901,7 +901,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>5.909863229730671e-06</v>
+        <v>6.205356391217296e-06</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -943,7 +943,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1.188252400000429e-09</v>
+        <v>1.247665020001161e-09</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -964,7 +964,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>5.773670851704256e-06</v>
+        <v>6.062354394289275e-06</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -1111,7 +1111,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>1.603413951999687e-05</v>
+        <v>1.683584649599671e-05</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -1132,7 +1132,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>3.34871568872747e-06</v>
+        <v>3.516151473163842e-06</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -1174,7 +1174,7 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>1.807489258702972e-05</v>
+        <v>1.897863721638121e-05</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -1195,7 +1195,7 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2.75472467514908e-05</v>
+        <v>2.892460908906534e-05</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -1216,7 +1216,7 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>1.163185918410117e-05</v>
+        <v>1.221345214330662e-05</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -1237,7 +1237,7 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>1.063300312592874e-05</v>
+        <v>1.116465328222518e-05</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -1258,7 +1258,7 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>7.795228182469171e-07</v>
+        <v>8.184989591592644e-07</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -1321,7 +1321,7 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>2.109331291314072e-07</v>
+        <v>2.214797855879776e-07</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -1342,7 +1342,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>1.593375502998286e-05</v>
+        <v>1.673044278148147e-05</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -1384,7 +1384,7 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>6.029479999999999e-13</v>
+        <v>0</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -1405,7 +1405,7 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>6.029479999999999e-13</v>
+        <v>0</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -1426,7 +1426,7 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>4.708531953782044e-06</v>
+        <v>4.943958551470577e-06</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -1468,7 +1468,7 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>2.662927018438403e-07</v>
+        <v>2.796073369360002e-07</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -1510,7 +1510,7 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>7.524426916933714e-06</v>
+        <v>7.900648262780398e-06</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
@@ -1573,7 +1573,7 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>6.605547600002385e-08</v>
+        <v>6.935824980006454e-08</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
@@ -1615,7 +1615,7 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>2.777148240000224e-09</v>
+        <v>2.916005652000083e-09</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
@@ -1636,7 +1636,7 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>6.298536400000508e-10</v>
+        <v>6.613463220000188e-10</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -1678,7 +1678,7 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>6.297095791402802e-07</v>
+        <v>6.611950580972941e-07</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -1762,7 +1762,7 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>1.070980506584029e-08</v>
+        <v>1.124529531913871e-08</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
@@ -1825,7 +1825,7 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>2.381633079165146e-06</v>
+        <v>2.500714733122825e-06</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -1846,7 +1846,7 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>3.007360369784271e-07</v>
+        <v>3.157728388273485e-07</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
@@ -1930,7 +1930,7 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>1.306282425137837e-06</v>
+        <v>1.371596546394728e-06</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
@@ -1951,7 +1951,7 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>5.544367200002002e-11</v>
+        <v>5.821585560005417e-11</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -1972,7 +1972,7 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>1.978941200000714e-09</v>
+        <v>2.077888260001933e-09</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
@@ -2014,7 +2014,7 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>8.511936727383683e-06</v>
+        <v>8.937527916772933e-06</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -2056,7 +2056,7 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>3.337824147921561e-05</v>
+        <v>3.504715355317639e-05</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
@@ -2098,7 +2098,7 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>4.25513514733863e-06</v>
+        <v>4.467831327937559e-06</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
@@ -2140,7 +2140,7 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>2.223890060710289e-05</v>
+        <v>2.335084563745807e-05</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
@@ -2161,7 +2161,7 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>4.447780121420578e-05</v>
+        <v>4.670169127491613e-05</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
@@ -2224,7 +2224,7 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>4.975235471094454e-06</v>
+        <v>5.223997244649175e-06</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
@@ -2266,7 +2266,7 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>2.995377288164981e-06</v>
+        <v>3.14514615257323e-06</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
@@ -2287,7 +2287,7 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>3.384903922540733e-07</v>
+        <v>3.554149118667769e-07</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
@@ -2350,7 +2350,7 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>3.447527200001245e-10</v>
+        <v>3.619903560003369e-10</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
@@ -2392,7 +2392,7 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>8.620373475319055e-06</v>
+        <v>9.051392149085006e-06</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
@@ -2434,7 +2434,7 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>1.036931397729375e-05</v>
+        <v>1.088777967615844e-05</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
@@ -2455,7 +2455,7 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>1.837072000000663e-09</v>
+        <v>1.928925600001795e-09</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
@@ -2497,7 +2497,7 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>0.0001613125541996582</v>
+        <v>0.0001696874844344041</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
@@ -2560,7 +2560,7 @@
         </is>
       </c>
       <c r="C102" t="n">
-        <v>3.395025603786138e-06</v>
+        <v>3.564776883974657e-06</v>
       </c>
       <c r="D102" t="inlineStr">
         <is>
@@ -2581,7 +2581,7 @@
         </is>
       </c>
       <c r="C103" t="n">
-        <v>4.810900605697324e-06</v>
+        <v>5.051445635981162e-06</v>
       </c>
       <c r="D103" t="inlineStr">
         <is>
@@ -2602,7 +2602,7 @@
         </is>
       </c>
       <c r="C104" t="n">
-        <v>1.338052384243475e-06</v>
+        <v>1.404955003455651e-06</v>
       </c>
       <c r="D104" t="inlineStr">
         <is>
@@ -2665,7 +2665,7 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>1.846105471635555e-05</v>
+        <v>1.938410745217332e-05</v>
       </c>
       <c r="D107" t="inlineStr">
         <is>
@@ -2833,7 +2833,7 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>1.905786929985865e-05</v>
+        <v>1.996268074118401e-05</v>
       </c>
       <c r="D115" t="inlineStr">
         <is>
@@ -2875,7 +2875,7 @@
         </is>
       </c>
       <c r="C117" t="n">
-        <v>1.096596400000396e-09</v>
+        <v>1.151426220001071e-09</v>
       </c>
       <c r="D117" t="inlineStr">
         <is>
@@ -2938,7 +2938,7 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>4.180594211731081e-06</v>
+        <v>4.389623922317641e-06</v>
       </c>
       <c r="D120" t="inlineStr">
         <is>
@@ -3232,7 +3232,7 @@
         </is>
       </c>
       <c r="C134" t="n">
-        <v>6.958719679756939e-07</v>
+        <v>7.306655663744784e-07</v>
       </c>
       <c r="D134" t="inlineStr">
         <is>
@@ -3253,7 +3253,7 @@
         </is>
       </c>
       <c r="C135" t="n">
-        <v>6.958719679756939e-07</v>
+        <v>7.306655663744784e-07</v>
       </c>
       <c r="D135" t="inlineStr">
         <is>
@@ -3295,7 +3295,7 @@
         </is>
       </c>
       <c r="C137" t="n">
-        <v>6.958719679756939e-07</v>
+        <v>7.306655663744784e-07</v>
       </c>
       <c r="D137" t="inlineStr">
         <is>
@@ -3379,7 +3379,7 @@
         </is>
       </c>
       <c r="C141" t="n">
-        <v>8.938026513385405e-06</v>
+        <v>9.384927839053832e-06</v>
       </c>
       <c r="D141" t="inlineStr">
         <is>
@@ -3400,7 +3400,7 @@
         </is>
       </c>
       <c r="C142" t="n">
-        <v>1.66422961436568e-06</v>
+        <v>1.747441095083807e-06</v>
       </c>
       <c r="D142" t="inlineStr">
         <is>
@@ -3421,7 +3421,7 @@
         </is>
       </c>
       <c r="C143" t="n">
-        <v>4.184460012915083e-06</v>
+        <v>4.393683013560444e-06</v>
       </c>
       <c r="D143" t="inlineStr">
         <is>
@@ -3484,7 +3484,7 @@
         </is>
       </c>
       <c r="C146" t="n">
-        <v>1.534027460434753e-06</v>
+        <v>1.61072883345649e-06</v>
       </c>
       <c r="D146" t="inlineStr">
         <is>
@@ -3505,7 +3505,7 @@
         </is>
       </c>
       <c r="C147" t="n">
-        <v>1.031242667040271e-06</v>
+        <v>1.082804800392285e-06</v>
       </c>
       <c r="D147" t="inlineStr">
         <is>
@@ -3526,7 +3526,7 @@
         </is>
       </c>
       <c r="C148" t="n">
-        <v>2.494689461923612e-06</v>
+        <v>2.619423935019792e-06</v>
       </c>
       <c r="D148" t="inlineStr">
         <is>
@@ -3568,7 +3568,7 @@
         </is>
       </c>
       <c r="C150" t="n">
-        <v>6.855401610385038e-06</v>
+        <v>7.19817169090429e-06</v>
       </c>
       <c r="D150" t="inlineStr">
         <is>
@@ -3610,7 +3610,7 @@
         </is>
       </c>
       <c r="C152" t="n">
-        <v>2.400933276748113e-06</v>
+        <v>2.520979940585519e-06</v>
       </c>
       <c r="D152" t="inlineStr">
         <is>
@@ -3631,7 +3631,7 @@
         </is>
       </c>
       <c r="C153" t="n">
-        <v>2.183378452836867e-06</v>
+        <v>2.29254737547871e-06</v>
       </c>
       <c r="D153" t="inlineStr">
         <is>
@@ -3652,7 +3652,7 @@
         </is>
       </c>
       <c r="C154" t="n">
-        <v>3.794197609809166e-07</v>
+        <v>3.983907490299623e-07</v>
       </c>
       <c r="D154" t="inlineStr">
         <is>
@@ -3673,7 +3673,7 @@
         </is>
       </c>
       <c r="C155" t="n">
-        <v>3.421170071682078e-06</v>
+        <v>3.613247329435897e-06</v>
       </c>
       <c r="D155" t="inlineStr">
         <is>
@@ -3694,7 +3694,7 @@
         </is>
       </c>
       <c r="C156" t="n">
-        <v>2.79559985577732e-05</v>
+        <v>2.9491268463718e-05</v>
       </c>
       <c r="D156" t="inlineStr">
         <is>
@@ -3715,7 +3715,7 @@
         </is>
       </c>
       <c r="C157" t="n">
-        <v>3.035111140021581e-06</v>
+        <v>3.18686669702266e-06</v>
       </c>
       <c r="D157" t="inlineStr">
         <is>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C158" t="n">
-        <v>7.099243650918684e-08</v>
+        <v>7.454205833464618e-08</v>
       </c>
       <c r="D158" t="inlineStr">
         <is>
@@ -3799,7 +3799,7 @@
         </is>
       </c>
       <c r="C161" t="n">
-        <v>4.764597460009487e-06</v>
+        <v>5.002827333009961e-06</v>
       </c>
       <c r="D161" t="inlineStr">
         <is>
@@ -3820,7 +3820,7 @@
         </is>
       </c>
       <c r="C162" t="n">
-        <v>2.442051031251549e-06</v>
+        <v>2.566369345777992e-06</v>
       </c>
       <c r="D162" t="inlineStr">
         <is>
@@ -3841,7 +3841,7 @@
         </is>
       </c>
       <c r="C163" t="n">
-        <v>8.140145615165766e-07</v>
+        <v>8.554538750250497e-07</v>
       </c>
       <c r="D163" t="inlineStr">
         <is>
@@ -3862,7 +3862,7 @@
         </is>
       </c>
       <c r="C164" t="n">
-        <v>8.140145615165766e-07</v>
+        <v>8.554538750250497e-07</v>
       </c>
       <c r="D164" t="inlineStr">
         <is>
@@ -3883,7 +3883,7 @@
         </is>
       </c>
       <c r="C165" t="n">
-        <v>1.628029123033153e-06</v>
+        <v>1.710907750050099e-06</v>
       </c>
       <c r="D165" t="inlineStr">
         <is>
@@ -3925,7 +3925,7 @@
         </is>
       </c>
       <c r="C167" t="n">
-        <v>1.628029123033153e-06</v>
+        <v>1.710907750050099e-06</v>
       </c>
       <c r="D167" t="inlineStr">
         <is>
@@ -3946,7 +3946,7 @@
         </is>
       </c>
       <c r="C168" t="n">
-        <v>2.442051031251549e-06</v>
+        <v>2.566369345777992e-06</v>
       </c>
       <c r="D168" t="inlineStr">
         <is>
@@ -3967,7 +3967,7 @@
         </is>
       </c>
       <c r="C169" t="n">
-        <v>1.628029123033153e-06</v>
+        <v>1.710907750050099e-06</v>
       </c>
       <c r="D169" t="inlineStr">
         <is>
@@ -3988,7 +3988,7 @@
         </is>
       </c>
       <c r="C170" t="n">
-        <v>8.140145615165766e-07</v>
+        <v>8.554538750250497e-07</v>
       </c>
       <c r="D170" t="inlineStr">
         <is>
@@ -4009,7 +4009,7 @@
         </is>
       </c>
       <c r="C171" t="n">
-        <v>1.628029123033153e-06</v>
+        <v>1.710907750050099e-06</v>
       </c>
       <c r="D171" t="inlineStr">
         <is>
@@ -4030,7 +4030,7 @@
         </is>
       </c>
       <c r="C172" t="n">
-        <v>1.628029123033153e-06</v>
+        <v>1.710907750050099e-06</v>
       </c>
       <c r="D172" t="inlineStr">
         <is>
@@ -4051,7 +4051,7 @@
         </is>
       </c>
       <c r="C173" t="n">
-        <v>8.140145615165766e-07</v>
+        <v>8.554538750250497e-07</v>
       </c>
       <c r="D173" t="inlineStr">
         <is>
@@ -4072,7 +4072,7 @@
         </is>
       </c>
       <c r="C174" t="n">
-        <v>8.140145615165766e-07</v>
+        <v>8.554538750250497e-07</v>
       </c>
       <c r="D174" t="inlineStr">
         <is>
@@ -4261,7 +4261,7 @@
         </is>
       </c>
       <c r="C183" t="n">
-        <v>2.226229755432932e-06</v>
+        <v>2.337541243204578e-06</v>
       </c>
       <c r="D183" t="inlineStr">
         <is>
@@ -4303,7 +4303,7 @@
         </is>
       </c>
       <c r="C185" t="n">
-        <v>2.662552557345443e-06</v>
+        <v>2.795680185212714e-06</v>
       </c>
       <c r="D185" t="inlineStr">
         <is>
@@ -4324,7 +4324,7 @@
         </is>
       </c>
       <c r="C186" t="n">
-        <v>2.164231307529159e-06</v>
+        <v>2.272442872905617e-06</v>
       </c>
       <c r="D186" t="inlineStr">
         <is>
@@ -4345,7 +4345,7 @@
         </is>
       </c>
       <c r="C187" t="n">
-        <v>3.897266261386836e-05</v>
+        <v>4.092129574456177e-05</v>
       </c>
       <c r="D187" t="inlineStr">
         <is>
@@ -4408,7 +4408,7 @@
         </is>
       </c>
       <c r="C190" t="n">
-        <v>1.263619970483665e-07</v>
+        <v>1.326800969007848e-07</v>
       </c>
       <c r="D190" t="inlineStr">
         <is>
@@ -4471,7 +4471,7 @@
         </is>
       </c>
       <c r="C193" t="n">
-        <v>1.305176875038369e-06</v>
+        <v>1.370435718790287e-06</v>
       </c>
       <c r="D193" t="inlineStr">
         <is>
@@ -4492,7 +4492,7 @@
         </is>
       </c>
       <c r="C194" t="n">
-        <v>1.305176875038369e-06</v>
+        <v>1.370435718790287e-06</v>
       </c>
       <c r="D194" t="inlineStr">
         <is>
@@ -4744,7 +4744,7 @@
         </is>
       </c>
       <c r="C206" t="n">
-        <v>6.606355335560282e-08</v>
+        <v>6.936673102338296e-08</v>
       </c>
       <c r="D206" t="inlineStr">
         <is>
@@ -4765,7 +4765,7 @@
         </is>
       </c>
       <c r="C207" t="n">
-        <v>2.941093213009567e-05</v>
+        <v>3.088147873659947e-05</v>
       </c>
       <c r="D207" t="inlineStr">
         <is>
@@ -4786,7 +4786,7 @@
         </is>
       </c>
       <c r="C208" t="n">
-        <v>2.699410523594338e-07</v>
+        <v>2.841442224131645e-07</v>
       </c>
       <c r="D208" t="inlineStr">
         <is>
@@ -4870,7 +4870,7 @@
         </is>
       </c>
       <c r="C212" t="n">
-        <v>1.569652e-11</v>
+        <v>0</v>
       </c>
       <c r="D212" t="inlineStr">
         <is>
@@ -4912,7 +4912,7 @@
         </is>
       </c>
       <c r="C214" t="n">
-        <v>1.584020191141963e-07</v>
+        <v>1.663221200699061e-07</v>
       </c>
       <c r="D214" t="inlineStr">
         <is>
@@ -4954,7 +4954,7 @@
         </is>
       </c>
       <c r="C216" t="n">
-        <v>2.127627899462521e-07</v>
+        <v>2.234009294435678e-07</v>
       </c>
       <c r="D216" t="inlineStr">
         <is>
@@ -5017,7 +5017,7 @@
         </is>
       </c>
       <c r="C219" t="n">
-        <v>1.40957751883528e-06</v>
+        <v>1.480056394777044e-06</v>
       </c>
       <c r="D219" t="inlineStr">
         <is>
@@ -5038,7 +5038,7 @@
         </is>
       </c>
       <c r="C220" t="n">
-        <v>1.377681665101807e-07</v>
+        <v>1.446565748356897e-07</v>
       </c>
       <c r="D220" t="inlineStr">
         <is>
@@ -5059,7 +5059,7 @@
         </is>
       </c>
       <c r="C221" t="n">
-        <v>2.8323216e-09</v>
+        <v>2.97393768e-09</v>
       </c>
       <c r="D221" t="inlineStr">
         <is>
@@ -5101,7 +5101,7 @@
         </is>
       </c>
       <c r="C223" t="n">
-        <v>1.862162824001563e-07</v>
+        <v>1.95527096520164e-07</v>
       </c>
       <c r="D223" t="inlineStr">
         <is>
@@ -5122,7 +5122,7 @@
         </is>
       </c>
       <c r="C224" t="n">
-        <v>1.862162824001563e-07</v>
+        <v>1.95527096520164e-07</v>
       </c>
       <c r="D224" t="inlineStr">
         <is>
@@ -5227,7 +5227,7 @@
         </is>
       </c>
       <c r="C229" t="n">
-        <v>0.0002480201757423169</v>
+        <v>0.000259881173288825</v>
       </c>
       <c r="D229" t="inlineStr">
         <is>
@@ -5269,7 +5269,7 @@
         </is>
       </c>
       <c r="C231" t="n">
-        <v>1.175503630891533e-08</v>
+        <v>7.857397788360957e-09</v>
       </c>
       <c r="D231" t="inlineStr">
         <is>
@@ -5353,7 +5353,7 @@
         </is>
       </c>
       <c r="C235" t="n">
-        <v>1.206197895760002e-07</v>
+        <v>1.266507790548001e-07</v>
       </c>
       <c r="D235" t="inlineStr">
         <is>
@@ -5374,7 +5374,7 @@
         </is>
       </c>
       <c r="C236" t="n">
-        <v>8.108910720000655e-12</v>
+        <v>8.514356256000243e-12</v>
       </c>
       <c r="D236" t="inlineStr">
         <is>
@@ -5395,7 +5395,7 @@
         </is>
       </c>
       <c r="C237" t="n">
-        <v>4.775922000000385e-10</v>
+        <v>5.014718100000143e-10</v>
       </c>
       <c r="D237" t="inlineStr">
         <is>
@@ -5416,7 +5416,7 @@
         </is>
       </c>
       <c r="C238" t="n">
-        <v>2.498790147556277e-06</v>
+        <v>2.623729654934091e-06</v>
       </c>
       <c r="D238" t="inlineStr">
         <is>
@@ -5437,7 +5437,7 @@
         </is>
       </c>
       <c r="C239" t="n">
-        <v>1.851899375463689e-05</v>
+        <v>1.944494344236874e-05</v>
       </c>
       <c r="D239" t="inlineStr">
         <is>
@@ -5479,7 +5479,7 @@
         </is>
       </c>
       <c r="C241" t="n">
-        <v>5.471676228433106e-05</v>
+        <v>5.74518214421808e-05</v>
       </c>
       <c r="D241" t="inlineStr">
         <is>
@@ -5500,7 +5500,7 @@
         </is>
       </c>
       <c r="C242" t="n">
-        <v>2.43368878760813e-05</v>
+        <v>2.549913844514835e-05</v>
       </c>
       <c r="D242" t="inlineStr">
         <is>
@@ -5542,7 +5542,7 @@
         </is>
       </c>
       <c r="C244" t="n">
-        <v>3.889294752136462e-06</v>
+        <v>4.083759489743285e-06</v>
       </c>
       <c r="D244" t="inlineStr">
         <is>
@@ -5647,7 +5647,7 @@
         </is>
       </c>
       <c r="C249" t="n">
-        <v>3.8077488e-09</v>
+        <v>0</v>
       </c>
       <c r="D249" t="inlineStr">
         <is>
@@ -5899,7 +5899,7 @@
         </is>
       </c>
       <c r="C261" t="n">
-        <v>2.2751905416523e-10</v>
+        <v>0</v>
       </c>
       <c r="D261" t="inlineStr">
         <is>
@@ -5941,7 +5941,7 @@
         </is>
       </c>
       <c r="C263" t="n">
-        <v>2.229884106371213e-07</v>
+        <v>2.344554461223332e-07</v>
       </c>
       <c r="D263" t="inlineStr">
         <is>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C264" t="n">
-        <v>4.459768212742427e-07</v>
+        <v>4.689108922446664e-07</v>
       </c>
       <c r="D264" t="inlineStr">
         <is>
@@ -5983,7 +5983,7 @@
         </is>
       </c>
       <c r="C265" t="n">
-        <v>2.229884106371213e-07</v>
+        <v>2.344554461223332e-07</v>
       </c>
       <c r="D265" t="inlineStr">
         <is>
@@ -6004,7 +6004,7 @@
         </is>
       </c>
       <c r="C266" t="n">
-        <v>2.229884106371213e-07</v>
+        <v>2.344554461223332e-07</v>
       </c>
       <c r="D266" t="inlineStr">
         <is>
@@ -6025,7 +6025,7 @@
         </is>
       </c>
       <c r="C267" t="n">
-        <v>2.229884106371213e-07</v>
+        <v>2.344554461223332e-07</v>
       </c>
       <c r="D267" t="inlineStr">
         <is>
@@ -6046,7 +6046,7 @@
         </is>
       </c>
       <c r="C268" t="n">
-        <v>2.229884106371213e-07</v>
+        <v>2.344554461223332e-07</v>
       </c>
       <c r="D268" t="inlineStr">
         <is>
@@ -6067,7 +6067,7 @@
         </is>
       </c>
       <c r="C269" t="n">
-        <v>2.229884106371213e-07</v>
+        <v>2.344554461223332e-07</v>
       </c>
       <c r="D269" t="inlineStr">
         <is>
@@ -6088,7 +6088,7 @@
         </is>
       </c>
       <c r="C270" t="n">
-        <v>2.229884106371213e-07</v>
+        <v>2.344554461223332e-07</v>
       </c>
       <c r="D270" t="inlineStr">
         <is>
@@ -6109,7 +6109,7 @@
         </is>
       </c>
       <c r="C271" t="n">
-        <v>2.229884106371213e-07</v>
+        <v>2.344554461223332e-07</v>
       </c>
       <c r="D271" t="inlineStr">
         <is>
@@ -6214,7 +6214,7 @@
         </is>
       </c>
       <c r="C276" t="n">
-        <v>2.173983235343788e-05</v>
+        <v>2.286345697606783e-05</v>
       </c>
       <c r="D276" t="inlineStr">
         <is>
@@ -6235,7 +6235,7 @@
         </is>
       </c>
       <c r="C277" t="n">
-        <v>2.173983235343788e-05</v>
+        <v>2.286345697606783e-05</v>
       </c>
       <c r="D277" t="inlineStr">
         <is>
@@ -6256,7 +6256,7 @@
         </is>
       </c>
       <c r="C278" t="n">
-        <v>2.173983235343788e-05</v>
+        <v>2.286345697606783e-05</v>
       </c>
       <c r="D278" t="inlineStr">
         <is>
@@ -6277,7 +6277,7 @@
         </is>
       </c>
       <c r="C279" t="n">
-        <v>2.173983235343788e-05</v>
+        <v>2.286345697606783e-05</v>
       </c>
       <c r="D279" t="inlineStr">
         <is>
@@ -6298,7 +6298,7 @@
         </is>
       </c>
       <c r="C280" t="n">
-        <v>2.173983235343788e-05</v>
+        <v>2.286345697606783e-05</v>
       </c>
       <c r="D280" t="inlineStr">
         <is>
@@ -6319,7 +6319,7 @@
         </is>
       </c>
       <c r="C281" t="n">
-        <v>2.173983235343788e-05</v>
+        <v>2.286345697606783e-05</v>
       </c>
       <c r="D281" t="inlineStr">
         <is>
@@ -6340,7 +6340,7 @@
         </is>
       </c>
       <c r="C282" t="n">
-        <v>2.173983235343788e-05</v>
+        <v>2.286345697606783e-05</v>
       </c>
       <c r="D282" t="inlineStr">
         <is>
@@ -6361,7 +6361,7 @@
         </is>
       </c>
       <c r="C283" t="n">
-        <v>2.173983235343788e-05</v>
+        <v>2.286345697606783e-05</v>
       </c>
       <c r="D283" t="inlineStr">
         <is>
@@ -6382,7 +6382,7 @@
         </is>
       </c>
       <c r="C284" t="n">
-        <v>2.173983235343788e-05</v>
+        <v>2.286345697606783e-05</v>
       </c>
       <c r="D284" t="inlineStr">
         <is>
@@ -6403,7 +6403,7 @@
         </is>
       </c>
       <c r="C285" t="n">
-        <v>2.780119371548624e-09</v>
+        <v>2.919125340126056e-09</v>
       </c>
       <c r="D285" t="inlineStr">
         <is>
@@ -6445,7 +6445,7 @@
         </is>
       </c>
       <c r="C287" t="n">
-        <v>7.311747325466474e-06</v>
+        <v>7.677334691738655e-06</v>
       </c>
       <c r="D287" t="inlineStr">
         <is>
@@ -6466,7 +6466,7 @@
         </is>
       </c>
       <c r="C288" t="n">
-        <v>7.488545255653111e-09</v>
+        <v>7.862972518134744e-09</v>
       </c>
       <c r="D288" t="inlineStr">
         <is>
@@ -6529,7 +6529,7 @@
         </is>
       </c>
       <c r="C291" t="n">
-        <v>5.735327336492966e-07</v>
+        <v>6.048268733640848e-07</v>
       </c>
       <c r="D291" t="inlineStr">
         <is>
@@ -6550,7 +6550,7 @@
         </is>
       </c>
       <c r="C292" t="n">
-        <v>2.968363725405392e-07</v>
+        <v>3.116781911675662e-07</v>
       </c>
       <c r="D292" t="inlineStr">
         <is>
@@ -6655,7 +6655,7 @@
         </is>
       </c>
       <c r="C297" t="n">
-        <v>5.693161188931681e-06</v>
+        <v>5.977815471427374e-06</v>
       </c>
       <c r="D297" t="inlineStr">
         <is>
@@ -6676,7 +6676,7 @@
         </is>
       </c>
       <c r="C298" t="n">
-        <v>7.551122123600002e-05</v>
+        <v>7.91136465644257e-05</v>
       </c>
       <c r="D298" t="inlineStr">
         <is>
@@ -6697,7 +6697,7 @@
         </is>
       </c>
       <c r="C299" t="n">
-        <v>2.014310667157161e-06</v>
+        <v>2.115026200515019e-06</v>
       </c>
       <c r="D299" t="inlineStr">
         <is>
@@ -6802,7 +6802,7 @@
         </is>
       </c>
       <c r="C304" t="n">
-        <v>1.643284903763787e-06</v>
+        <v>1.725449148951976e-06</v>
       </c>
       <c r="D304" t="inlineStr">
         <is>
@@ -6823,7 +6823,7 @@
         </is>
       </c>
       <c r="C305" t="n">
-        <v>2.767644607442319e-06</v>
+        <v>2.906026837814163e-06</v>
       </c>
       <c r="D305" t="inlineStr">
         <is>
@@ -6865,7 +6865,7 @@
         </is>
       </c>
       <c r="C307" t="n">
-        <v>7.262669579153224e-06</v>
+        <v>7.625803058110884e-06</v>
       </c>
       <c r="D307" t="inlineStr">
         <is>
@@ -6886,7 +6886,7 @@
         </is>
       </c>
       <c r="C308" t="n">
-        <v>2.894766704087832e-06</v>
+        <v>3.039505039292224e-06</v>
       </c>
       <c r="D308" t="inlineStr">
         <is>
@@ -7180,7 +7180,7 @@
         </is>
       </c>
       <c r="C322" t="n">
-        <v>7.501670866161366e-05</v>
+        <v>7.860149751449465e-05</v>
       </c>
       <c r="D322" t="inlineStr">
         <is>
@@ -7327,7 +7327,7 @@
         </is>
       </c>
       <c r="C329" t="n">
-        <v>1.836487896588184e-08</v>
+        <v>1.928312291417596e-08</v>
       </c>
       <c r="D329" t="inlineStr">
         <is>
@@ -7369,7 +7369,7 @@
         </is>
       </c>
       <c r="C331" t="n">
-        <v>1.422292241446131e-06</v>
+        <v>1.493406853518092e-06</v>
       </c>
       <c r="D331" t="inlineStr">
         <is>
@@ -7390,7 +7390,7 @@
         </is>
       </c>
       <c r="C332" t="n">
-        <v>1.732844790367112e-09</v>
+        <v>1.819487029827726e-09</v>
       </c>
       <c r="D332" t="inlineStr">
         <is>
@@ -7411,7 +7411,7 @@
         </is>
       </c>
       <c r="C333" t="n">
-        <v>1.732844790367112e-09</v>
+        <v>1.819487029827726e-09</v>
       </c>
       <c r="D333" t="inlineStr">
         <is>
@@ -7432,7 +7432,7 @@
         </is>
       </c>
       <c r="C334" t="n">
-        <v>3.170870160063953e-06</v>
+        <v>3.351699293248974e-06</v>
       </c>
       <c r="D334" t="inlineStr">
         <is>
@@ -7453,7 +7453,7 @@
         </is>
       </c>
       <c r="C335" t="n">
-        <v>1.732844790367112e-09</v>
+        <v>1.819487029827726e-09</v>
       </c>
       <c r="D335" t="inlineStr">
         <is>
@@ -7474,7 +7474,7 @@
         </is>
       </c>
       <c r="C336" t="n">
-        <v>7.669911353699372e-06</v>
+        <v>8.053406921383617e-06</v>
       </c>
       <c r="D336" t="inlineStr">
         <is>
@@ -7495,7 +7495,7 @@
         </is>
       </c>
       <c r="C337" t="n">
-        <v>7.380269457770806e-10</v>
+        <v>7.74928293041342e-10</v>
       </c>
       <c r="D337" t="inlineStr">
         <is>
@@ -7516,7 +7516,7 @@
         </is>
       </c>
       <c r="C338" t="n">
-        <v>0</v>
+        <v>9.03236146884308e-09</v>
       </c>
       <c r="D338" t="inlineStr">
         <is>
@@ -7537,7 +7537,7 @@
         </is>
       </c>
       <c r="C339" t="n">
-        <v>0</v>
+        <v>9.03236146884308e-09</v>
       </c>
       <c r="D339" t="inlineStr">
         <is>
@@ -7558,7 +7558,7 @@
         </is>
       </c>
       <c r="C340" t="n">
-        <v>7.039979126063309e-06</v>
+        <v>7.391978082366474e-06</v>
       </c>
       <c r="D340" t="inlineStr">
         <is>
@@ -7579,7 +7579,7 @@
         </is>
       </c>
       <c r="C341" t="n">
-        <v>1.759987553225276e-06</v>
+        <v>1.847986930886539e-06</v>
       </c>
       <c r="D341" t="inlineStr">
         <is>
@@ -7642,7 +7642,7 @@
         </is>
       </c>
       <c r="C344" t="n">
-        <v>3.158919239582594e-06</v>
+        <v>3.316865201561724e-06</v>
       </c>
       <c r="D344" t="inlineStr">
         <is>
@@ -7663,7 +7663,7 @@
         </is>
       </c>
       <c r="C345" t="n">
-        <v>2.014827125160911e-06</v>
+        <v>2.115568481418949e-06</v>
       </c>
       <c r="D345" t="inlineStr">
         <is>
@@ -7810,7 +7810,7 @@
         </is>
       </c>
       <c r="C352" t="n">
-        <v>1.209071888219943e-07</v>
+        <v>1.269525482630874e-07</v>
       </c>
       <c r="D352" t="inlineStr">
         <is>
@@ -7831,7 +7831,7 @@
         </is>
       </c>
       <c r="C353" t="n">
-        <v>2.978428e-09</v>
+        <v>3.1273494e-09</v>
       </c>
       <c r="D353" t="inlineStr">
         <is>
@@ -7894,7 +7894,7 @@
         </is>
       </c>
       <c r="C356" t="n">
-        <v>3.998066940864294e-05</v>
+        <v>4.190210775583306e-05</v>
       </c>
       <c r="D356" t="inlineStr">
         <is>
@@ -7978,7 +7978,7 @@
         </is>
       </c>
       <c r="C360" t="n">
-        <v>2.614988329875119e-06</v>
+        <v>2.745737746368875e-06</v>
       </c>
       <c r="D360" t="inlineStr">
         <is>
@@ -7999,7 +7999,7 @@
         </is>
       </c>
       <c r="C361" t="n">
-        <v>3.965849969513516e-06</v>
+        <v>4.164142467989191e-06</v>
       </c>
       <c r="D361" t="inlineStr">
         <is>
@@ -8020,7 +8020,7 @@
         </is>
       </c>
       <c r="C362" t="n">
-        <v>1.800386586534176e-07</v>
+        <v>1.890405915860884e-07</v>
       </c>
       <c r="D362" t="inlineStr">
         <is>
@@ -8041,7 +8041,7 @@
         </is>
       </c>
       <c r="C363" t="n">
-        <v>2.39790985716497e-07</v>
+        <v>2.517805350023218e-07</v>
       </c>
       <c r="D363" t="inlineStr">
         <is>
@@ -8083,7 +8083,7 @@
         </is>
       </c>
       <c r="C365" t="n">
-        <v>4.996620291048433e-08</v>
+        <v>5.246451305600854e-08</v>
       </c>
       <c r="D365" t="inlineStr">
         <is>
@@ -8104,7 +8104,7 @@
         </is>
       </c>
       <c r="C366" t="n">
-        <v>7.807151810813678e-05</v>
+        <v>8.19750940135436e-05</v>
       </c>
       <c r="D366" t="inlineStr">
         <is>
@@ -8188,7 +8188,7 @@
         </is>
       </c>
       <c r="C370" t="n">
-        <v>1.284657547856912e-05</v>
+        <v>1.348890425249758e-05</v>
       </c>
       <c r="D370" t="inlineStr">
         <is>
@@ -8209,7 +8209,7 @@
         </is>
       </c>
       <c r="C371" t="n">
-        <v>4.456117896806678e-07</v>
+        <v>4.678923791647012e-07</v>
       </c>
       <c r="D371" t="inlineStr">
         <is>
@@ -8230,7 +8230,7 @@
         </is>
       </c>
       <c r="C372" t="n">
-        <v>6.234929156648294e-06</v>
+        <v>6.546675614480708e-06</v>
       </c>
       <c r="D372" t="inlineStr">
         <is>
@@ -8251,7 +8251,7 @@
         </is>
       </c>
       <c r="C373" t="n">
-        <v>1.32479717158321e-06</v>
+        <v>1.391037030162371e-06</v>
       </c>
       <c r="D373" t="inlineStr">
         <is>
@@ -8272,7 +8272,7 @@
         </is>
       </c>
       <c r="C374" t="n">
-        <v>5.821591525866918e-05</v>
+        <v>6.112671102160274e-05</v>
       </c>
       <c r="D374" t="inlineStr">
         <is>
@@ -8377,7 +8377,7 @@
         </is>
       </c>
       <c r="C379" t="n">
-        <v>3.004772890305417e-07</v>
+        <v>3.155014686592018e-07</v>
       </c>
       <c r="D379" t="inlineStr">
         <is>
@@ -8503,7 +8503,7 @@
         </is>
       </c>
       <c r="C385" t="n">
-        <v>5.545974888541768e-07</v>
+        <v>5.823194679604853e-07</v>
       </c>
       <c r="D385" t="inlineStr">
         <is>
@@ -8524,7 +8524,7 @@
         </is>
       </c>
       <c r="C386" t="n">
-        <v>1.487369618288663e-06</v>
+        <v>1.561716924777096e-06</v>
       </c>
       <c r="D386" t="inlineStr">
         <is>
@@ -8566,7 +8566,7 @@
         </is>
       </c>
       <c r="C388" t="n">
-        <v>7.801025333571875e-06</v>
+        <v>8.191076600250467e-06</v>
       </c>
       <c r="D388" t="inlineStr">
         <is>
@@ -8587,7 +8587,7 @@
         </is>
       </c>
       <c r="C389" t="n">
-        <v>1.626827382153204e-06</v>
+        <v>1.708168751260864e-06</v>
       </c>
       <c r="D389" t="inlineStr">
         <is>
@@ -8608,7 +8608,7 @@
         </is>
       </c>
       <c r="C390" t="n">
-        <v>8.732114233546061e-06</v>
+        <v>9.168719945223332e-06</v>
       </c>
       <c r="D390" t="inlineStr">
         <is>
@@ -8671,7 +8671,7 @@
         </is>
       </c>
       <c r="C393" t="n">
-        <v>4.714913690314284e-05</v>
+        <v>4.94573017980073e-05</v>
       </c>
       <c r="D393" t="inlineStr">
         <is>
@@ -8713,7 +8713,7 @@
         </is>
       </c>
       <c r="C395" t="n">
-        <v>7.307525760194551e-06</v>
+        <v>7.672902048202971e-06</v>
       </c>
       <c r="D395" t="inlineStr">
         <is>
@@ -8776,7 +8776,7 @@
         </is>
       </c>
       <c r="C398" t="n">
-        <v>9.280146682957589e-06</v>
+        <v>9.464012881355822e-06</v>
       </c>
       <c r="D398" t="inlineStr">
         <is>
@@ -8797,7 +8797,7 @@
         </is>
       </c>
       <c r="C399" t="n">
-        <v>9.280146682957589e-06</v>
+        <v>9.464012881355822e-06</v>
       </c>
       <c r="D399" t="inlineStr">
         <is>
@@ -8860,7 +8860,7 @@
         </is>
       </c>
       <c r="C402" t="n">
-        <v>1.142439481564453e-06</v>
+        <v>1.199561455642676e-06</v>
       </c>
       <c r="D402" t="inlineStr">
         <is>
@@ -8902,7 +8902,7 @@
         </is>
       </c>
       <c r="C404" t="n">
-        <v>7.900572216732767e-06</v>
+        <v>8.295488353790388e-06</v>
       </c>
       <c r="D404" t="inlineStr">
         <is>
@@ -8923,7 +8923,7 @@
         </is>
       </c>
       <c r="C405" t="n">
-        <v>0</v>
+        <v>8.823868704185921e-09</v>
       </c>
       <c r="D405" t="inlineStr">
         <is>
@@ -8944,7 +8944,7 @@
         </is>
       </c>
       <c r="C406" t="n">
-        <v>0</v>
+        <v>8.823868704185921e-09</v>
       </c>
       <c r="D406" t="inlineStr">
         <is>
@@ -8965,7 +8965,7 @@
         </is>
       </c>
       <c r="C407" t="n">
-        <v>1.345208705766142e-06</v>
+        <v>1.412469141054287e-06</v>
       </c>
       <c r="D407" t="inlineStr">
         <is>
@@ -9049,7 +9049,7 @@
         </is>
       </c>
       <c r="C411" t="n">
-        <v>1.820609739388279e-06</v>
+        <v>1.911640226357693e-06</v>
       </c>
       <c r="D411" t="inlineStr">
         <is>
@@ -9091,7 +9091,7 @@
         </is>
       </c>
       <c r="C413" t="n">
-        <v>7.782846001744886e-06</v>
+        <v>8.17198830183213e-06</v>
       </c>
       <c r="D413" t="inlineStr">
         <is>
@@ -9154,7 +9154,7 @@
         </is>
       </c>
       <c r="C416" t="n">
-        <v>2.992617956127918e-05</v>
+        <v>3.142248853933954e-05</v>
       </c>
       <c r="D416" t="inlineStr">
         <is>
@@ -9175,7 +9175,7 @@
         </is>
       </c>
       <c r="C417" t="n">
-        <v>2.819502061715797e-07</v>
+        <v>2.960480122238335e-07</v>
       </c>
       <c r="D417" t="inlineStr">
         <is>
@@ -9196,7 +9196,7 @@
         </is>
       </c>
       <c r="C418" t="n">
-        <v>4.444232131388521e-07</v>
+        <v>4.666443737957946e-07</v>
       </c>
       <c r="D418" t="inlineStr">
         <is>
@@ -9217,7 +9217,7 @@
         </is>
       </c>
       <c r="C419" t="n">
-        <v>1.09734851850746e-06</v>
+        <v>1.152215944432833e-06</v>
       </c>
       <c r="D419" t="inlineStr">
         <is>
@@ -9280,7 +9280,7 @@
         </is>
       </c>
       <c r="C422" t="n">
-        <v>4.872957324980008e-06</v>
+        <v>5.116605191229008e-06</v>
       </c>
       <c r="D422" t="inlineStr">
         <is>
@@ -9322,7 +9322,7 @@
         </is>
       </c>
       <c r="C424" t="n">
-        <v>8.672376800885835e-06</v>
+        <v>9.14549142354481e-06</v>
       </c>
       <c r="D424" t="inlineStr">
         <is>
@@ -9406,7 +9406,7 @@
         </is>
       </c>
       <c r="C428" t="n">
-        <v>3.661621533009997e-06</v>
+        <v>3.652620544906112e-06</v>
       </c>
       <c r="D428" t="inlineStr">
         <is>
@@ -9448,7 +9448,7 @@
         </is>
       </c>
       <c r="C430" t="n">
-        <v>4.418660397187281e-07</v>
+        <v>4.639593417046644e-07</v>
       </c>
       <c r="D430" t="inlineStr">
         <is>
@@ -9469,7 +9469,7 @@
         </is>
       </c>
       <c r="C431" t="n">
-        <v>1.331018322860008e-05</v>
+        <v>1.397569239003009e-05</v>
       </c>
       <c r="D431" t="inlineStr">
         <is>
@@ -9490,7 +9490,7 @@
         </is>
       </c>
       <c r="C432" t="n">
-        <v>2.360851759232435e-06</v>
+        <v>2.478894347194059e-06</v>
       </c>
       <c r="D432" t="inlineStr">
         <is>
@@ -9532,7 +9532,7 @@
         </is>
       </c>
       <c r="C434" t="n">
-        <v>2.858891379788844e-06</v>
+        <v>3.001835948778286e-06</v>
       </c>
       <c r="D434" t="inlineStr">
         <is>
@@ -9595,7 +9595,7 @@
         </is>
       </c>
       <c r="C437" t="n">
-        <v>1.345528239762537e-06</v>
+        <v>1.412785496600663e-06</v>
       </c>
       <c r="D437" t="inlineStr">
         <is>
@@ -9616,7 +9616,7 @@
         </is>
       </c>
       <c r="C438" t="n">
-        <v>8.072015643816016e-05</v>
+        <v>8.475501511532414e-05</v>
       </c>
       <c r="D438" t="inlineStr">
         <is>
@@ -9700,7 +9700,7 @@
         </is>
       </c>
       <c r="C442" t="n">
-        <v>3.680934041245245e-08</v>
+        <v>3.864980743307508e-08</v>
       </c>
       <c r="D442" t="inlineStr">
         <is>
@@ -9721,7 +9721,7 @@
         </is>
       </c>
       <c r="C443" t="n">
-        <v>3.629924318275614e-08</v>
+        <v>3.811420534189395e-08</v>
       </c>
       <c r="D443" t="inlineStr">
         <is>
@@ -9784,7 +9784,7 @@
         </is>
       </c>
       <c r="C446" t="n">
-        <v>1.355076418452953e-07</v>
+        <v>1.422830239375601e-07</v>
       </c>
       <c r="D446" t="inlineStr">
         <is>
@@ -9805,7 +9805,7 @@
         </is>
       </c>
       <c r="C447" t="n">
-        <v>2.899389212727849e-07</v>
+        <v>3.044358673363892e-07</v>
       </c>
       <c r="D447" t="inlineStr">
         <is>
@@ -9952,7 +9952,7 @@
         </is>
       </c>
       <c r="C454" t="n">
-        <v>1.852751663742932e-06</v>
+        <v>1.945389246929855e-06</v>
       </c>
       <c r="D454" t="inlineStr">
         <is>
@@ -9994,7 +9994,7 @@
         </is>
       </c>
       <c r="C456" t="n">
-        <v>0.0001273384022506662</v>
+        <v>0.0001338855933464049</v>
       </c>
       <c r="D456" t="inlineStr">
         <is>
@@ -10120,7 +10120,7 @@
         </is>
       </c>
       <c r="C462" t="n">
-        <v>2.742545993580063e-07</v>
+        <v>2.879673293258735e-07</v>
       </c>
       <c r="D462" t="inlineStr">
         <is>
@@ -10141,7 +10141,7 @@
         </is>
       </c>
       <c r="C463" t="n">
-        <v>3.206900802334428e-05</v>
+        <v>3.367245842450763e-05</v>
       </c>
       <c r="D463" t="inlineStr">
         <is>
@@ -10183,7 +10183,7 @@
         </is>
       </c>
       <c r="C465" t="n">
-        <v>1.638306294649157e-05</v>
+        <v>1.720220600355917e-05</v>
       </c>
       <c r="D465" t="inlineStr">
         <is>
@@ -10246,7 +10246,7 @@
         </is>
       </c>
       <c r="C468" t="n">
-        <v>3.838054602063419e-07</v>
+        <v>4.029957332166645e-07</v>
       </c>
       <c r="D468" t="inlineStr">
         <is>
@@ -10267,7 +10267,7 @@
         </is>
       </c>
       <c r="C469" t="n">
-        <v>1.395494721960478e-07</v>
+        <v>1.465269458058502e-07</v>
       </c>
       <c r="D469" t="inlineStr">
         <is>
@@ -10330,7 +10330,7 @@
         </is>
       </c>
       <c r="C472" t="n">
-        <v>9.595281395776819e-08</v>
+        <v>1.007504546556566e-07</v>
       </c>
       <c r="D472" t="inlineStr">
         <is>
@@ -10372,7 +10372,7 @@
         </is>
       </c>
       <c r="C474" t="n">
-        <v>5.979909392234532e-07</v>
+        <v>6.278904861846259e-07</v>
       </c>
       <c r="D474" t="inlineStr">
         <is>
@@ -10393,7 +10393,7 @@
         </is>
       </c>
       <c r="C475" t="n">
-        <v>1.013999600000366e-08</v>
+        <v>1.064699580000991e-08</v>
       </c>
       <c r="D475" t="inlineStr">
         <is>
@@ -10414,7 +10414,7 @@
         </is>
       </c>
       <c r="C476" t="n">
-        <v>6.21755098336188e-07</v>
+        <v>6.528428532533693e-07</v>
       </c>
       <c r="D476" t="inlineStr">
         <is>
@@ -10435,7 +10435,7 @@
         </is>
       </c>
       <c r="C477" t="n">
-        <v>6.596480800002381e-09</v>
+        <v>6.926304840006445e-09</v>
       </c>
       <c r="D477" t="inlineStr">
         <is>
@@ -10477,7 +10477,7 @@
         </is>
       </c>
       <c r="C479" t="n">
-        <v>2.281281653885253e-06</v>
+        <v>2.395345736579516e-06</v>
       </c>
       <c r="D479" t="inlineStr">
         <is>
@@ -10498,7 +10498,7 @@
         </is>
       </c>
       <c r="C480" t="n">
-        <v>2.281281653885253e-06</v>
+        <v>2.395345736579516e-06</v>
       </c>
       <c r="D480" t="inlineStr">
         <is>
@@ -10540,7 +10540,7 @@
         </is>
       </c>
       <c r="C482" t="n">
-        <v>3.721928010156923e-06</v>
+        <v>3.908024410663865e-06</v>
       </c>
       <c r="D482" t="inlineStr">
         <is>
@@ -10582,7 +10582,7 @@
         </is>
       </c>
       <c r="C484" t="n">
-        <v>5.345255357718277e-05</v>
+        <v>5.612518125604202e-05</v>
       </c>
       <c r="D484" t="inlineStr">
         <is>
@@ -10624,7 +10624,7 @@
         </is>
       </c>
       <c r="C486" t="n">
-        <v>6.824544097322718e-05</v>
+        <v>7.150912307296414e-05</v>
       </c>
       <c r="D486" t="inlineStr">
         <is>
@@ -10666,7 +10666,7 @@
         </is>
       </c>
       <c r="C488" t="n">
-        <v>4.777607206280719e-06</v>
+        <v>5.016487566594755e-06</v>
       </c>
       <c r="D488" t="inlineStr">
         <is>
@@ -10729,7 +10729,7 @@
         </is>
       </c>
       <c r="C491" t="n">
-        <v>1.507200534584629e-05</v>
+        <v>1.582560561313729e-05</v>
       </c>
       <c r="D491" t="inlineStr">
         <is>
@@ -10771,7 +10771,7 @@
         </is>
       </c>
       <c r="C493" t="n">
-        <v>2.287705902808117e-05</v>
+        <v>2.397027449505794e-05</v>
       </c>
       <c r="D493" t="inlineStr">
         <is>
@@ -10813,7 +10813,7 @@
         </is>
       </c>
       <c r="C495" t="n">
-        <v>1.567087247343509e-05</v>
+        <v>1.645441609710684e-05</v>
       </c>
       <c r="D495" t="inlineStr">
         <is>
@@ -10834,7 +10834,7 @@
         </is>
       </c>
       <c r="C496" t="n">
-        <v>1.42103359357549e-06</v>
+        <v>1.492065043198264e-06</v>
       </c>
       <c r="D496" t="inlineStr">
         <is>
@@ -10855,7 +10855,7 @@
         </is>
       </c>
       <c r="C497" t="n">
-        <v>1.349058921891755e-07</v>
+        <v>1.416511867987149e-07</v>
       </c>
       <c r="D497" t="inlineStr">
         <is>
@@ -10876,7 +10876,7 @@
         </is>
       </c>
       <c r="C498" t="n">
-        <v>1.119480000000404e-09</v>
+        <v>1.175454000001094e-09</v>
       </c>
       <c r="D498" t="inlineStr">
         <is>
@@ -10960,7 +10960,7 @@
         </is>
       </c>
       <c r="C502" t="n">
-        <v>5.59561235664154e-07</v>
+        <v>5.875392974472259e-07</v>
       </c>
       <c r="D502" t="inlineStr">
         <is>
@@ -10981,7 +10981,7 @@
         </is>
       </c>
       <c r="C503" t="n">
-        <v>9.193668825783161e-06</v>
+        <v>9.653352267070088e-06</v>
       </c>
       <c r="D503" t="inlineStr">
         <is>
@@ -11002,7 +11002,7 @@
         </is>
       </c>
       <c r="C504" t="n">
-        <v>1.60190148983349e-07</v>
+        <v>1.681996564325014e-07</v>
       </c>
       <c r="D504" t="inlineStr">
         <is>
@@ -11023,7 +11023,7 @@
         </is>
       </c>
       <c r="C505" t="n">
-        <v>1.008899278398689e-05</v>
+        <v>1.059344242318379e-05</v>
       </c>
       <c r="D505" t="inlineStr">
         <is>
@@ -11065,7 +11065,7 @@
         </is>
       </c>
       <c r="C507" t="n">
-        <v>3.375972689484288e-07</v>
+        <v>3.544771323958096e-07</v>
       </c>
       <c r="D507" t="inlineStr">
         <is>
@@ -11107,7 +11107,7 @@
         </is>
       </c>
       <c r="C509" t="n">
-        <v>3.375972689484288e-07</v>
+        <v>3.544771323958096e-07</v>
       </c>
       <c r="D509" t="inlineStr">
         <is>
@@ -11149,7 +11149,7 @@
         </is>
       </c>
       <c r="C511" t="n">
-        <v>2.912338872323109e-06</v>
+        <v>3.057955815939011e-06</v>
       </c>
       <c r="D511" t="inlineStr">
         <is>
@@ -11170,7 +11170,7 @@
         </is>
       </c>
       <c r="C512" t="n">
-        <v>9.592139972410787e-06</v>
+        <v>1.007174697103049e-05</v>
       </c>
       <c r="D512" t="inlineStr">
         <is>
@@ -11233,7 +11233,7 @@
         </is>
       </c>
       <c r="C515" t="n">
-        <v>7.589595237838669e-06</v>
+        <v>7.969074999730602e-06</v>
       </c>
       <c r="D515" t="inlineStr">
         <is>
@@ -11254,7 +11254,7 @@
         </is>
       </c>
       <c r="C516" t="n">
-        <v>3.854069751724866e-06</v>
+        <v>4.046773239311109e-06</v>
       </c>
       <c r="D516" t="inlineStr">
         <is>
@@ -11296,7 +11296,7 @@
         </is>
       </c>
       <c r="C518" t="n">
-        <v>1.004098073418044e-06</v>
+        <v>1.054302977088947e-06</v>
       </c>
       <c r="D518" t="inlineStr">
         <is>
@@ -11317,7 +11317,7 @@
         </is>
       </c>
       <c r="C519" t="n">
-        <v>6.50414e-12</v>
+        <v>0</v>
       </c>
       <c r="D519" t="inlineStr">
         <is>
@@ -11422,7 +11422,7 @@
         </is>
       </c>
       <c r="C524" t="n">
-        <v>1.679185723217527e-05</v>
+        <v>1.743847977761864e-05</v>
       </c>
       <c r="D524" t="inlineStr">
         <is>
@@ -11443,7 +11443,7 @@
         </is>
       </c>
       <c r="C525" t="n">
-        <v>1.583707689161518e-06</v>
+        <v>1.66500352472282e-06</v>
       </c>
       <c r="D525" t="inlineStr">
         <is>
@@ -11464,7 +11464,7 @@
         </is>
       </c>
       <c r="C526" t="n">
-        <v>1.583707689161518e-06</v>
+        <v>1.66500352472282e-06</v>
       </c>
       <c r="D526" t="inlineStr">
         <is>
@@ -11485,7 +11485,7 @@
         </is>
       </c>
       <c r="C527" t="n">
-        <v>1.583707689161518e-06</v>
+        <v>1.66500352472282e-06</v>
       </c>
       <c r="D527" t="inlineStr">
         <is>
@@ -11506,7 +11506,7 @@
         </is>
       </c>
       <c r="C528" t="n">
-        <v>1.583707689161518e-06</v>
+        <v>1.66500352472282e-06</v>
       </c>
       <c r="D528" t="inlineStr">
         <is>
@@ -11548,7 +11548,7 @@
         </is>
       </c>
       <c r="C530" t="n">
-        <v>7.702768088265969e-05</v>
+        <v>8.070423186588362e-05</v>
       </c>
       <c r="D530" t="inlineStr">
         <is>
@@ -11569,7 +11569,7 @@
         </is>
       </c>
       <c r="C531" t="n">
-        <v>1.972236e-10</v>
+        <v>2.070847799999997e-10</v>
       </c>
       <c r="D531" t="inlineStr">
         <is>
@@ -11590,7 +11590,7 @@
         </is>
       </c>
       <c r="C532" t="n">
-        <v>8.60158812975504e-07</v>
+        <v>9.031667536242791e-07</v>
       </c>
       <c r="D532" t="inlineStr">
         <is>
@@ -11611,7 +11611,7 @@
         </is>
       </c>
       <c r="C533" t="n">
-        <v>2.540424e-09</v>
+        <v>2.6674452e-09</v>
       </c>
       <c r="D533" t="inlineStr">
         <is>
@@ -11632,7 +11632,7 @@
         </is>
       </c>
       <c r="C534" t="n">
-        <v>1.508976e-08</v>
+        <v>1.5844248e-08</v>
       </c>
       <c r="D534" t="inlineStr">
         <is>
@@ -11653,7 +11653,7 @@
         </is>
       </c>
       <c r="C535" t="n">
-        <v>3.617769721192275e-08</v>
+        <v>3.798658207251888e-08</v>
       </c>
       <c r="D535" t="inlineStr">
         <is>
@@ -11716,7 +11716,7 @@
         </is>
       </c>
       <c r="C538" t="n">
-        <v>5.333814507989121e-06</v>
+        <v>5.600502645293783e-06</v>
       </c>
       <c r="D538" t="inlineStr">
         <is>
@@ -11758,7 +11758,7 @@
         </is>
       </c>
       <c r="C540" t="n">
-        <v>5.782651879644417e-07</v>
+        <v>6.071779770794277e-07</v>
       </c>
       <c r="D540" t="inlineStr">
         <is>
@@ -11821,7 +11821,7 @@
         </is>
       </c>
       <c r="C543" t="n">
-        <v>8.178785060926369e-06</v>
+        <v>8.587724313972687e-06</v>
       </c>
       <c r="D543" t="inlineStr">
         <is>
@@ -11842,7 +11842,7 @@
         </is>
       </c>
       <c r="C544" t="n">
-        <v>1.399703293416549e-06</v>
+        <v>1.469688458087377e-06</v>
       </c>
       <c r="D544" t="inlineStr">
         <is>
@@ -11989,7 +11989,7 @@
         </is>
       </c>
       <c r="C551" t="n">
-        <v>9.029656865729843e-06</v>
+        <v>9.481139709016335e-06</v>
       </c>
       <c r="D551" t="inlineStr">
         <is>
@@ -12073,7 +12073,7 @@
         </is>
       </c>
       <c r="C555" t="n">
-        <v>1.020528000000368e-10</v>
+        <v>1.071554400000997e-10</v>
       </c>
       <c r="D555" t="inlineStr">
         <is>
@@ -12157,7 +12157,7 @@
         </is>
       </c>
       <c r="C559" t="n">
-        <v>2.052922406067376e-08</v>
+        <v>2.155568526370744e-08</v>
       </c>
       <c r="D559" t="inlineStr">
         <is>
@@ -12178,7 +12178,7 @@
         </is>
       </c>
       <c r="C560" t="n">
-        <v>1.658245374072874e-07</v>
+        <v>1.741157642776518e-07</v>
       </c>
       <c r="D560" t="inlineStr">
         <is>
@@ -12199,7 +12199,7 @@
         </is>
       </c>
       <c r="C561" t="n">
-        <v>4.659951061532284e-07</v>
+        <v>5.051094701391905e-07</v>
       </c>
       <c r="D561" t="inlineStr">
         <is>
@@ -12220,7 +12220,7 @@
         </is>
       </c>
       <c r="C562" t="n">
-        <v>4.659951061532284e-07</v>
+        <v>5.051094701391905e-07</v>
       </c>
       <c r="D562" t="inlineStr">
         <is>
@@ -12241,7 +12241,7 @@
         </is>
       </c>
       <c r="C563" t="n">
-        <v>4.659951061532284e-07</v>
+        <v>5.051094701391905e-07</v>
       </c>
       <c r="D563" t="inlineStr">
         <is>
@@ -12325,7 +12325,7 @@
         </is>
       </c>
       <c r="C567" t="n">
-        <v>3.925001301184434e-06</v>
+        <v>4.121251366243663e-06</v>
       </c>
       <c r="D567" t="inlineStr">
         <is>
@@ -12346,7 +12346,7 @@
         </is>
       </c>
       <c r="C568" t="n">
-        <v>9.592735724668506e-07</v>
+        <v>1.007237251090195e-06</v>
       </c>
       <c r="D568" t="inlineStr">
         <is>
@@ -12367,7 +12367,7 @@
         </is>
       </c>
       <c r="C569" t="n">
-        <v>9.592735724668506e-07</v>
+        <v>1.007237251090195e-06</v>
       </c>
       <c r="D569" t="inlineStr">
         <is>
@@ -12451,7 +12451,7 @@
         </is>
       </c>
       <c r="C573" t="n">
-        <v>4.763361681486404e-06</v>
+        <v>5.001529765560731e-06</v>
       </c>
       <c r="D573" t="inlineStr">
         <is>
@@ -12493,7 +12493,7 @@
         </is>
       </c>
       <c r="C575" t="n">
-        <v>2.871941987803036e-06</v>
+        <v>3.015539087193188e-06</v>
       </c>
       <c r="D575" t="inlineStr">
         <is>
@@ -12535,7 +12535,7 @@
         </is>
       </c>
       <c r="C577" t="n">
-        <v>3.6862848e-08</v>
+        <v>3.87059904e-08</v>
       </c>
       <c r="D577" t="inlineStr">
         <is>
@@ -12598,7 +12598,7 @@
         </is>
       </c>
       <c r="C580" t="n">
-        <v>1.849431119280691e-05</v>
+        <v>1.937706215416395e-05</v>
       </c>
       <c r="D580" t="inlineStr">
         <is>
@@ -12619,7 +12619,7 @@
         </is>
       </c>
       <c r="C581" t="n">
-        <v>2.538001511301743e-05</v>
+        <v>2.664899708156437e-05</v>
       </c>
       <c r="D581" t="inlineStr">
         <is>
@@ -12661,7 +12661,7 @@
         </is>
       </c>
       <c r="C583" t="n">
-        <v>3.349512475927993e-06</v>
+        <v>3.50918139113354e-06</v>
       </c>
       <c r="D583" t="inlineStr">
         <is>
@@ -12682,7 +12682,7 @@
         </is>
       </c>
       <c r="C584" t="n">
-        <v>9.061977711093132e-06</v>
+        <v>9.515076596646934e-06</v>
       </c>
       <c r="D584" t="inlineStr">
         <is>
@@ -12703,7 +12703,7 @@
         </is>
       </c>
       <c r="C585" t="n">
-        <v>2.5380872158825e-07</v>
+        <v>2.664991576676624e-07</v>
       </c>
       <c r="D585" t="inlineStr">
         <is>
@@ -12745,7 +12745,7 @@
         </is>
       </c>
       <c r="C587" t="n">
-        <v>3.236470024254777e-06</v>
+        <v>3.398293525467515e-06</v>
       </c>
       <c r="D587" t="inlineStr">
         <is>
@@ -12829,7 +12829,7 @@
         </is>
       </c>
       <c r="C591" t="n">
-        <v>1.129772859147806e-05</v>
+        <v>1.186261502105199e-05</v>
       </c>
       <c r="D591" t="inlineStr">
         <is>
@@ -12913,7 +12913,7 @@
         </is>
       </c>
       <c r="C595" t="n">
-        <v>5.71072e-12</v>
+        <v>0</v>
       </c>
       <c r="D595" t="inlineStr">
         <is>
@@ -12997,7 +12997,7 @@
         </is>
       </c>
       <c r="C599" t="n">
-        <v>5.298396733055351e-06</v>
+        <v>5.563316569708118e-06</v>
       </c>
       <c r="D599" t="inlineStr">
         <is>
@@ -13144,7 +13144,7 @@
         </is>
       </c>
       <c r="C606" t="n">
-        <v>1.366996320769412e-05</v>
+        <v>1.541795633422876e-05</v>
       </c>
       <c r="D606" t="inlineStr">
         <is>
@@ -13165,7 +13165,7 @@
         </is>
       </c>
       <c r="C607" t="n">
-        <v>9.054249826216743e-06</v>
+        <v>9.506962317527592e-06</v>
       </c>
       <c r="D607" t="inlineStr">
         <is>
@@ -13186,7 +13186,7 @@
         </is>
       </c>
       <c r="C608" t="n">
-        <v>9.054249826216743e-06</v>
+        <v>9.506962317527592e-06</v>
       </c>
       <c r="D608" t="inlineStr">
         <is>
@@ -13354,7 +13354,7 @@
         </is>
       </c>
       <c r="C616" t="n">
-        <v>2.83848279570657e-07</v>
+        <v>2.980406935491901e-07</v>
       </c>
       <c r="D616" t="inlineStr">
         <is>
@@ -13396,7 +13396,7 @@
         </is>
       </c>
       <c r="C618" t="n">
-        <v>3.950217597991484e-09</v>
+        <v>3.330403817508616e-09</v>
       </c>
       <c r="D618" t="inlineStr">
         <is>
@@ -13459,7 +13459,7 @@
         </is>
       </c>
       <c r="C621" t="n">
-        <v>1.566325264370038e-07</v>
+        <v>1.644641527588539e-07</v>
       </c>
       <c r="D621" t="inlineStr">
         <is>
@@ -13480,7 +13480,7 @@
         </is>
       </c>
       <c r="C622" t="n">
-        <v>1.147053599307165e-06</v>
+        <v>1.204406279272527e-06</v>
       </c>
       <c r="D622" t="inlineStr">
         <is>
@@ -13522,7 +13522,7 @@
         </is>
       </c>
       <c r="C624" t="n">
-        <v>1.796528291781682e-06</v>
+        <v>2.460137982377647e-06</v>
       </c>
       <c r="D624" t="inlineStr">
         <is>
@@ -13543,7 +13543,7 @@
         </is>
       </c>
       <c r="C625" t="n">
-        <v>6.821796540229741e-07</v>
+        <v>4.948280078568954e-07</v>
       </c>
       <c r="D625" t="inlineStr">
         <is>
@@ -13648,7 +13648,7 @@
         </is>
       </c>
       <c r="C630" t="n">
-        <v>6.77518841376117e-08</v>
+        <v>5.431140932267017e-08</v>
       </c>
       <c r="D630" t="inlineStr">
         <is>
@@ -13669,7 +13669,7 @@
         </is>
       </c>
       <c r="C631" t="n">
-        <v>1.303459450743497e-06</v>
+        <v>1.263781464514028e-06</v>
       </c>
       <c r="D631" t="inlineStr">
         <is>
@@ -13690,7 +13690,7 @@
         </is>
       </c>
       <c r="C632" t="n">
-        <v>5.569388581310849e-07</v>
+        <v>5.039266493460528e-07</v>
       </c>
       <c r="D632" t="inlineStr">
         <is>
@@ -13711,7 +13711,7 @@
         </is>
       </c>
       <c r="C633" t="n">
-        <v>8.862845409685291e-08</v>
+        <v>9.305987680169555e-08</v>
       </c>
       <c r="D633" t="inlineStr">
         <is>
@@ -13753,7 +13753,7 @@
         </is>
       </c>
       <c r="C635" t="n">
-        <v>5.681316709699577e-07</v>
+        <v>4.271464610655413e-07</v>
       </c>
       <c r="D635" t="inlineStr">
         <is>
@@ -13774,7 +13774,7 @@
         </is>
       </c>
       <c r="C636" t="n">
-        <v>2.360382879658617e-08</v>
+        <v>2.47840202364158e-08</v>
       </c>
       <c r="D636" t="inlineStr">
         <is>
@@ -13795,7 +13795,7 @@
         </is>
       </c>
       <c r="C637" t="n">
-        <v>3.830923194378065e-06</v>
+        <v>3.824660392198851e-06</v>
       </c>
       <c r="D637" t="inlineStr">
         <is>
@@ -14068,7 +14068,7 @@
         </is>
       </c>
       <c r="C650" t="n">
-        <v>0</v>
+        <v>1.297639553658393e-07</v>
       </c>
       <c r="D650" t="inlineStr">
         <is>
@@ -14824,7 +14824,7 @@
         </is>
       </c>
       <c r="C686" t="n">
-        <v>1.146713437933638e-05</v>
+        <v>1.208511016474748e-05</v>
       </c>
       <c r="D686" t="inlineStr">
         <is>
@@ -14887,7 +14887,7 @@
         </is>
       </c>
       <c r="C689" t="n">
-        <v>1.089684072766537e-05</v>
+        <v>1.145385136341727e-05</v>
       </c>
       <c r="D689" t="inlineStr">
         <is>
@@ -14992,7 +14992,7 @@
         </is>
       </c>
       <c r="C694" t="n">
-        <v>3.785170067422894e-06</v>
+        <v>3.974428570793885e-06</v>
       </c>
       <c r="D694" t="inlineStr">
         <is>
@@ -15034,7 +15034,7 @@
         </is>
       </c>
       <c r="C696" t="n">
-        <v>5.563736399718351e-05</v>
+        <v>5.864097385130594e-05</v>
       </c>
       <c r="D696" t="inlineStr">
         <is>
@@ -15265,7 +15265,7 @@
         </is>
       </c>
       <c r="C707" t="n">
-        <v>6.913283494591251e-05</v>
+        <v>7.245530258039204e-05</v>
       </c>
       <c r="D707" t="inlineStr">
         <is>
@@ -15412,7 +15412,7 @@
         </is>
       </c>
       <c r="C714" t="n">
-        <v>8.061766718719799e-06</v>
+        <v>8.464855054655803e-06</v>
       </c>
       <c r="D714" t="inlineStr">
         <is>
@@ -15496,7 +15496,7 @@
         </is>
       </c>
       <c r="C718" t="n">
-        <v>8.43155312e-10</v>
+        <v>8.571183936e-10</v>
       </c>
       <c r="D718" t="inlineStr">
         <is>
@@ -15559,7 +15559,7 @@
         </is>
       </c>
       <c r="C721" t="n">
-        <v>3.7475e-10</v>
+        <v>0</v>
       </c>
       <c r="D721" t="inlineStr">
         <is>
@@ -15643,7 +15643,7 @@
         </is>
       </c>
       <c r="C725" t="n">
-        <v>4.929536592734306e-09</v>
+        <v>5.176013422206758e-09</v>
       </c>
       <c r="D725" t="inlineStr">
         <is>
@@ -15748,7 +15748,7 @@
         </is>
       </c>
       <c r="C730" t="n">
-        <v>3.795920108308879e-08</v>
+        <v>3.985716113724323e-08</v>
       </c>
       <c r="D730" t="inlineStr">
         <is>
@@ -15832,7 +15832,7 @@
         </is>
       </c>
       <c r="C734" t="n">
-        <v>5.021174669852316e-07</v>
+        <v>4.921512027174269e-08</v>
       </c>
       <c r="D734" t="inlineStr">
         <is>
@@ -15874,7 +15874,7 @@
         </is>
       </c>
       <c r="C736" t="n">
-        <v>3.228428605959648e-08</v>
+        <v>3.38985003625763e-08</v>
       </c>
       <c r="D736" t="inlineStr">
         <is>
@@ -15895,7 +15895,7 @@
         </is>
       </c>
       <c r="C737" t="n">
-        <v>2.231995931762132e-05</v>
+        <v>2.343595728350238e-05</v>
       </c>
       <c r="D737" t="inlineStr">
         <is>
@@ -15979,7 +15979,7 @@
         </is>
       </c>
       <c r="C741" t="n">
-        <v>0.0001639271783962479</v>
+        <v>0.0001720108659936563</v>
       </c>
       <c r="D741" t="inlineStr">
         <is>
@@ -16105,7 +16105,7 @@
         </is>
       </c>
       <c r="C747" t="n">
-        <v>3.3766438e-08</v>
+        <v>3.54547599e-08</v>
       </c>
       <c r="D747" t="inlineStr">
         <is>
@@ -16210,7 +16210,7 @@
         </is>
       </c>
       <c r="C752" t="n">
-        <v>2.311945769509503e-06</v>
+        <v>2.427543057984982e-06</v>
       </c>
       <c r="D752" t="inlineStr">
         <is>
@@ -17239,7 +17239,7 @@
         </is>
       </c>
       <c r="C801" t="n">
-        <v>1.627467469032639e-07</v>
+        <v>1.708840842484271e-07</v>
       </c>
       <c r="D801" t="inlineStr">
         <is>
@@ -18709,7 +18709,7 @@
         </is>
       </c>
       <c r="C871" t="n">
-        <v>3.533160555991282e-08</v>
+        <v>3.709818583790847e-08</v>
       </c>
       <c r="D871" t="inlineStr">
         <is>
@@ -18730,7 +18730,7 @@
         </is>
       </c>
       <c r="C872" t="n">
-        <v>4.89485216e-09</v>
+        <v>5.139594767999999e-09</v>
       </c>
       <c r="D872" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix: add the first constraints from compartment annotations
</commit_message>
<xml_diff>
--- a/data/data_check.xlsx
+++ b/data/data_check.xlsx
@@ -481,7 +481,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>2.33323678683125e-05</v>
+        <v>2.649843398175449e-05</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -502,7 +502,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>6.312111608355086e-06</v>
+        <v>1.482276902352393e-06</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -733,7 +733,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>2.752653120002561e-09</v>
+        <v>2.752653119994902e-09</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>2.752653120002561e-09</v>
+        <v>2.752653119994902e-09</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -817,7 +817,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>1.942872176729352e-06</v>
+        <v>1.94287217672935e-06</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -838,7 +838,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>3.885749768074305e-06</v>
+        <v>3.885749768074303e-06</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -901,7 +901,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>6.205356391217296e-06</v>
+        <v>6.205356391217201e-06</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -943,7 +943,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1.247665020001161e-09</v>
+        <v>1.247665019997689e-09</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -964,7 +964,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>6.062354394289275e-06</v>
+        <v>6.062354394289476e-06</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -1216,7 +1216,7 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>1.221345214330662e-05</v>
+        <v>1.221345214330621e-05</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -1258,7 +1258,7 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>8.184989591592644e-07</v>
+        <v>8.184989591592579e-07</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -1342,7 +1342,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>1.673044278148147e-05</v>
+        <v>1.673044278148202e-05</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -1384,7 +1384,7 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>0</v>
+        <v>6.330953999999999e-13</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -1405,7 +1405,7 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>0</v>
+        <v>6.330953999999999e-13</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -1426,7 +1426,7 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>4.943958551470577e-06</v>
+        <v>4.943958551471168e-06</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -1468,7 +1468,7 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>2.796073369360002e-07</v>
+        <v>2.796073369360335e-07</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -1573,7 +1573,7 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>6.935824980006454e-08</v>
+        <v>6.935824979987155e-08</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
@@ -1762,7 +1762,7 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>1.124529531913871e-08</v>
+        <v>1.124529531910742e-08</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
@@ -1825,7 +1825,7 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>2.500714733122825e-06</v>
+        <v>2.500714733124178e-06</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -1846,7 +1846,7 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>3.157728388273485e-07</v>
+        <v>3.167705113852122e-07</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
@@ -1930,7 +1930,7 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>1.371596546394728e-06</v>
+        <v>1.375930054748013e-06</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
@@ -1951,7 +1951,7 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>5.821585560005417e-11</v>
+        <v>5.821585559989219e-11</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -1972,7 +1972,7 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>2.077888260001933e-09</v>
+        <v>2.077888259996152e-09</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
@@ -2014,7 +2014,7 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>8.937527916772933e-06</v>
+        <v>8.939387940576949e-06</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -2056,7 +2056,7 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>3.504715355317639e-05</v>
+        <v>3.504715355317637e-05</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
@@ -2098,7 +2098,7 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>4.467831327937559e-06</v>
+        <v>4.467891904705558e-06</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
@@ -2140,7 +2140,7 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>2.335084563745807e-05</v>
+        <v>2.335084563745803e-05</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
@@ -2161,7 +2161,7 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>4.670169127491613e-05</v>
+        <v>4.670169127491606e-05</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
@@ -2350,7 +2350,7 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>3.619903560003369e-10</v>
+        <v>3.619903559993297e-10</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
@@ -2392,7 +2392,7 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>9.051392149085006e-06</v>
+        <v>9.091859078054608e-06</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
@@ -2434,7 +2434,7 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>1.088777967615844e-05</v>
+        <v>1.093645671937287e-05</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
@@ -2455,7 +2455,7 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>1.928925600001795e-09</v>
+        <v>1.928925599996428e-09</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
@@ -2497,7 +2497,7 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>0.0001696874844344041</v>
+        <v>0.0001699766665603495</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
@@ -2560,7 +2560,7 @@
         </is>
       </c>
       <c r="C102" t="n">
-        <v>3.564776883974657e-06</v>
+        <v>3.564776883976501e-06</v>
       </c>
       <c r="D102" t="inlineStr">
         <is>
@@ -2581,7 +2581,7 @@
         </is>
       </c>
       <c r="C103" t="n">
-        <v>5.051445635981162e-06</v>
+        <v>5.051445635983571e-06</v>
       </c>
       <c r="D103" t="inlineStr">
         <is>
@@ -2602,7 +2602,7 @@
         </is>
       </c>
       <c r="C104" t="n">
-        <v>1.404955003455651e-06</v>
+        <v>1.40495500345564e-06</v>
       </c>
       <c r="D104" t="inlineStr">
         <is>
@@ -2833,7 +2833,7 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>1.996268074118401e-05</v>
+        <v>1.874382950969299e-05</v>
       </c>
       <c r="D115" t="inlineStr">
         <is>
@@ -2875,7 +2875,7 @@
         </is>
       </c>
       <c r="C117" t="n">
-        <v>1.151426220001071e-09</v>
+        <v>1.151426219997868e-09</v>
       </c>
       <c r="D117" t="inlineStr">
         <is>
@@ -2938,7 +2938,7 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>4.389623922317641e-06</v>
+        <v>4.389623922317634e-06</v>
       </c>
       <c r="D120" t="inlineStr">
         <is>
@@ -3379,7 +3379,7 @@
         </is>
       </c>
       <c r="C141" t="n">
-        <v>9.384927839053832e-06</v>
+        <v>9.384927839054706e-06</v>
       </c>
       <c r="D141" t="inlineStr">
         <is>
@@ -3400,7 +3400,7 @@
         </is>
       </c>
       <c r="C142" t="n">
-        <v>1.747441095083807e-06</v>
+        <v>1.74744109508397e-06</v>
       </c>
       <c r="D142" t="inlineStr">
         <is>
@@ -3421,7 +3421,7 @@
         </is>
       </c>
       <c r="C143" t="n">
-        <v>4.393683013560444e-06</v>
+        <v>4.393683013560853e-06</v>
       </c>
       <c r="D143" t="inlineStr">
         <is>
@@ -3631,7 +3631,7 @@
         </is>
       </c>
       <c r="C153" t="n">
-        <v>2.29254737547871e-06</v>
+        <v>2.292547375478711e-06</v>
       </c>
       <c r="D153" t="inlineStr">
         <is>
@@ -3673,7 +3673,7 @@
         </is>
       </c>
       <c r="C155" t="n">
-        <v>3.613247329435897e-06</v>
+        <v>4.434805821719214e-06</v>
       </c>
       <c r="D155" t="inlineStr">
         <is>
@@ -3694,7 +3694,7 @@
         </is>
       </c>
       <c r="C156" t="n">
-        <v>2.9491268463718e-05</v>
+        <v>3.486454734573162e-05</v>
       </c>
       <c r="D156" t="inlineStr">
         <is>
@@ -3820,7 +3820,7 @@
         </is>
       </c>
       <c r="C162" t="n">
-        <v>2.566369345777992e-06</v>
+        <v>2.691099396024619e-06</v>
       </c>
       <c r="D162" t="inlineStr">
         <is>
@@ -3841,7 +3841,7 @@
         </is>
       </c>
       <c r="C163" t="n">
-        <v>8.554538750250497e-07</v>
+        <v>8.970304333606933e-07</v>
       </c>
       <c r="D163" t="inlineStr">
         <is>
@@ -3862,7 +3862,7 @@
         </is>
       </c>
       <c r="C164" t="n">
-        <v>8.554538750250497e-07</v>
+        <v>8.970304333606933e-07</v>
       </c>
       <c r="D164" t="inlineStr">
         <is>
@@ -3883,7 +3883,7 @@
         </is>
       </c>
       <c r="C165" t="n">
-        <v>1.710907750050099e-06</v>
+        <v>1.794060866721387e-06</v>
       </c>
       <c r="D165" t="inlineStr">
         <is>
@@ -3925,7 +3925,7 @@
         </is>
       </c>
       <c r="C167" t="n">
-        <v>1.710907750050099e-06</v>
+        <v>1.794060866721387e-06</v>
       </c>
       <c r="D167" t="inlineStr">
         <is>
@@ -3946,7 +3946,7 @@
         </is>
       </c>
       <c r="C168" t="n">
-        <v>2.566369345777992e-06</v>
+        <v>2.691099396024619e-06</v>
       </c>
       <c r="D168" t="inlineStr">
         <is>
@@ -3967,7 +3967,7 @@
         </is>
       </c>
       <c r="C169" t="n">
-        <v>1.710907750050099e-06</v>
+        <v>1.794060866721387e-06</v>
       </c>
       <c r="D169" t="inlineStr">
         <is>
@@ -3988,7 +3988,7 @@
         </is>
       </c>
       <c r="C170" t="n">
-        <v>8.554538750250497e-07</v>
+        <v>8.970304333606933e-07</v>
       </c>
       <c r="D170" t="inlineStr">
         <is>
@@ -4009,7 +4009,7 @@
         </is>
       </c>
       <c r="C171" t="n">
-        <v>1.710907750050099e-06</v>
+        <v>1.794060866721387e-06</v>
       </c>
       <c r="D171" t="inlineStr">
         <is>
@@ -4030,7 +4030,7 @@
         </is>
       </c>
       <c r="C172" t="n">
-        <v>1.710907750050099e-06</v>
+        <v>1.794060866721387e-06</v>
       </c>
       <c r="D172" t="inlineStr">
         <is>
@@ -4051,7 +4051,7 @@
         </is>
       </c>
       <c r="C173" t="n">
-        <v>8.554538750250497e-07</v>
+        <v>8.970304333606933e-07</v>
       </c>
       <c r="D173" t="inlineStr">
         <is>
@@ -4072,7 +4072,7 @@
         </is>
       </c>
       <c r="C174" t="n">
-        <v>8.554538750250497e-07</v>
+        <v>8.970304333606933e-07</v>
       </c>
       <c r="D174" t="inlineStr">
         <is>
@@ -4471,7 +4471,7 @@
         </is>
       </c>
       <c r="C193" t="n">
-        <v>1.370435718790287e-06</v>
+        <v>1.370435718790288e-06</v>
       </c>
       <c r="D193" t="inlineStr">
         <is>
@@ -4492,7 +4492,7 @@
         </is>
       </c>
       <c r="C194" t="n">
-        <v>1.370435718790287e-06</v>
+        <v>1.370435718790288e-06</v>
       </c>
       <c r="D194" t="inlineStr">
         <is>
@@ -4765,7 +4765,7 @@
         </is>
       </c>
       <c r="C207" t="n">
-        <v>3.088147873659947e-05</v>
+        <v>3.088147873660049e-05</v>
       </c>
       <c r="D207" t="inlineStr">
         <is>
@@ -4786,7 +4786,7 @@
         </is>
       </c>
       <c r="C208" t="n">
-        <v>2.841442224131645e-07</v>
+        <v>2.834381049774056e-07</v>
       </c>
       <c r="D208" t="inlineStr">
         <is>
@@ -4870,7 +4870,7 @@
         </is>
       </c>
       <c r="C212" t="n">
-        <v>0</v>
+        <v>1.6481346e-11</v>
       </c>
       <c r="D212" t="inlineStr">
         <is>
@@ -4954,7 +4954,7 @@
         </is>
       </c>
       <c r="C216" t="n">
-        <v>2.234009294435678e-07</v>
+        <v>0</v>
       </c>
       <c r="D216" t="inlineStr">
         <is>
@@ -5017,7 +5017,7 @@
         </is>
       </c>
       <c r="C219" t="n">
-        <v>1.480056394777044e-06</v>
+        <v>1.707609041973026e-06</v>
       </c>
       <c r="D219" t="inlineStr">
         <is>
@@ -5227,7 +5227,7 @@
         </is>
       </c>
       <c r="C229" t="n">
-        <v>0.000259881173288825</v>
+        <v>0.0002458742248587892</v>
       </c>
       <c r="D229" t="inlineStr">
         <is>
@@ -5269,7 +5269,7 @@
         </is>
       </c>
       <c r="C231" t="n">
-        <v>7.857397788360957e-09</v>
+        <v>1.234278812436112e-08</v>
       </c>
       <c r="D231" t="inlineStr">
         <is>
@@ -5416,7 +5416,7 @@
         </is>
       </c>
       <c r="C238" t="n">
-        <v>2.623729654934091e-06</v>
+        <v>2.623729654934093e-06</v>
       </c>
       <c r="D238" t="inlineStr">
         <is>
@@ -5437,7 +5437,7 @@
         </is>
       </c>
       <c r="C239" t="n">
-        <v>1.944494344236874e-05</v>
+        <v>1.944494344236873e-05</v>
       </c>
       <c r="D239" t="inlineStr">
         <is>
@@ -5479,7 +5479,7 @@
         </is>
       </c>
       <c r="C241" t="n">
-        <v>5.74518214421808e-05</v>
+        <v>5.74526003985476e-05</v>
       </c>
       <c r="D241" t="inlineStr">
         <is>
@@ -5500,7 +5500,7 @@
         </is>
       </c>
       <c r="C242" t="n">
-        <v>2.549913844514835e-05</v>
+        <v>2.47267668291286e-05</v>
       </c>
       <c r="D242" t="inlineStr">
         <is>
@@ -5647,7 +5647,7 @@
         </is>
       </c>
       <c r="C249" t="n">
-        <v>0</v>
+        <v>3.998136239999999e-09</v>
       </c>
       <c r="D249" t="inlineStr">
         <is>
@@ -5899,7 +5899,7 @@
         </is>
       </c>
       <c r="C261" t="n">
-        <v>0</v>
+        <v>2.388950068734915e-10</v>
       </c>
       <c r="D261" t="inlineStr">
         <is>
@@ -5941,7 +5941,7 @@
         </is>
       </c>
       <c r="C263" t="n">
-        <v>2.344554461223332e-07</v>
+        <v>2.341720341564525e-07</v>
       </c>
       <c r="D263" t="inlineStr">
         <is>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C264" t="n">
-        <v>4.689108922446664e-07</v>
+        <v>4.683440683129051e-07</v>
       </c>
       <c r="D264" t="inlineStr">
         <is>
@@ -5983,7 +5983,7 @@
         </is>
       </c>
       <c r="C265" t="n">
-        <v>2.344554461223332e-07</v>
+        <v>2.341720341564525e-07</v>
       </c>
       <c r="D265" t="inlineStr">
         <is>
@@ -6004,7 +6004,7 @@
         </is>
       </c>
       <c r="C266" t="n">
-        <v>2.344554461223332e-07</v>
+        <v>2.341720341564525e-07</v>
       </c>
       <c r="D266" t="inlineStr">
         <is>
@@ -6025,7 +6025,7 @@
         </is>
       </c>
       <c r="C267" t="n">
-        <v>2.344554461223332e-07</v>
+        <v>2.341720341564525e-07</v>
       </c>
       <c r="D267" t="inlineStr">
         <is>
@@ -6046,7 +6046,7 @@
         </is>
       </c>
       <c r="C268" t="n">
-        <v>2.344554461223332e-07</v>
+        <v>2.341720341564525e-07</v>
       </c>
       <c r="D268" t="inlineStr">
         <is>
@@ -6067,7 +6067,7 @@
         </is>
       </c>
       <c r="C269" t="n">
-        <v>2.344554461223332e-07</v>
+        <v>2.341720341564525e-07</v>
       </c>
       <c r="D269" t="inlineStr">
         <is>
@@ -6088,7 +6088,7 @@
         </is>
       </c>
       <c r="C270" t="n">
-        <v>2.344554461223332e-07</v>
+        <v>2.341720341564525e-07</v>
       </c>
       <c r="D270" t="inlineStr">
         <is>
@@ -6109,7 +6109,7 @@
         </is>
       </c>
       <c r="C271" t="n">
-        <v>2.344554461223332e-07</v>
+        <v>2.341720341564525e-07</v>
       </c>
       <c r="D271" t="inlineStr">
         <is>
@@ -6214,7 +6214,7 @@
         </is>
       </c>
       <c r="C276" t="n">
-        <v>2.286345697606783e-05</v>
+        <v>2.603008991344158e-05</v>
       </c>
       <c r="D276" t="inlineStr">
         <is>
@@ -6235,7 +6235,7 @@
         </is>
       </c>
       <c r="C277" t="n">
-        <v>2.286345697606783e-05</v>
+        <v>2.603008991344158e-05</v>
       </c>
       <c r="D277" t="inlineStr">
         <is>
@@ -6256,7 +6256,7 @@
         </is>
       </c>
       <c r="C278" t="n">
-        <v>2.286345697606783e-05</v>
+        <v>2.603008991344158e-05</v>
       </c>
       <c r="D278" t="inlineStr">
         <is>
@@ -6277,7 +6277,7 @@
         </is>
       </c>
       <c r="C279" t="n">
-        <v>2.286345697606783e-05</v>
+        <v>2.603008991344158e-05</v>
       </c>
       <c r="D279" t="inlineStr">
         <is>
@@ -6298,7 +6298,7 @@
         </is>
       </c>
       <c r="C280" t="n">
-        <v>2.286345697606783e-05</v>
+        <v>2.603008991344158e-05</v>
       </c>
       <c r="D280" t="inlineStr">
         <is>
@@ -6319,7 +6319,7 @@
         </is>
       </c>
       <c r="C281" t="n">
-        <v>2.286345697606783e-05</v>
+        <v>2.603008991344158e-05</v>
       </c>
       <c r="D281" t="inlineStr">
         <is>
@@ -6340,7 +6340,7 @@
         </is>
       </c>
       <c r="C282" t="n">
-        <v>2.286345697606783e-05</v>
+        <v>2.603008991344158e-05</v>
       </c>
       <c r="D282" t="inlineStr">
         <is>
@@ -6361,7 +6361,7 @@
         </is>
       </c>
       <c r="C283" t="n">
-        <v>2.286345697606783e-05</v>
+        <v>2.603008991344158e-05</v>
       </c>
       <c r="D283" t="inlineStr">
         <is>
@@ -6382,7 +6382,7 @@
         </is>
       </c>
       <c r="C284" t="n">
-        <v>2.286345697606783e-05</v>
+        <v>2.603008991344158e-05</v>
       </c>
       <c r="D284" t="inlineStr">
         <is>
@@ -6445,7 +6445,7 @@
         </is>
       </c>
       <c r="C287" t="n">
-        <v>7.677334691738655e-06</v>
+        <v>7.664890881874985e-06</v>
       </c>
       <c r="D287" t="inlineStr">
         <is>
@@ -6466,7 +6466,7 @@
         </is>
       </c>
       <c r="C288" t="n">
-        <v>7.862972518134744e-09</v>
+        <v>1.312530472560445e-08</v>
       </c>
       <c r="D288" t="inlineStr">
         <is>
@@ -6529,7 +6529,7 @@
         </is>
       </c>
       <c r="C291" t="n">
-        <v>6.048268733640848e-07</v>
+        <v>6.022093703318908e-07</v>
       </c>
       <c r="D291" t="inlineStr">
         <is>
@@ -6550,7 +6550,7 @@
         </is>
       </c>
       <c r="C292" t="n">
-        <v>3.116781911675662e-07</v>
+        <v>3.116781911675664e-07</v>
       </c>
       <c r="D292" t="inlineStr">
         <is>
@@ -6655,7 +6655,7 @@
         </is>
       </c>
       <c r="C297" t="n">
-        <v>5.977815471427374e-06</v>
+        <v>5.97905953792724e-06</v>
       </c>
       <c r="D297" t="inlineStr">
         <is>
@@ -6676,7 +6676,7 @@
         </is>
       </c>
       <c r="C298" t="n">
-        <v>7.91136465644257e-05</v>
+        <v>7.462120906280369e-05</v>
       </c>
       <c r="D298" t="inlineStr">
         <is>
@@ -6823,7 +6823,7 @@
         </is>
       </c>
       <c r="C305" t="n">
-        <v>2.906026837814163e-06</v>
+        <v>2.906026837814722e-06</v>
       </c>
       <c r="D305" t="inlineStr">
         <is>
@@ -7180,7 +7180,7 @@
         </is>
       </c>
       <c r="C322" t="n">
-        <v>7.860149751449465e-05</v>
+        <v>7.625310897385459e-05</v>
       </c>
       <c r="D322" t="inlineStr">
         <is>
@@ -7327,7 +7327,7 @@
         </is>
       </c>
       <c r="C329" t="n">
-        <v>1.928312291417596e-08</v>
+        <v>1.932032168758395e-08</v>
       </c>
       <c r="D329" t="inlineStr">
         <is>
@@ -7369,7 +7369,7 @@
         </is>
       </c>
       <c r="C331" t="n">
-        <v>1.493406853518092e-06</v>
+        <v>1.4934068535189e-06</v>
       </c>
       <c r="D331" t="inlineStr">
         <is>
@@ -7390,7 +7390,7 @@
         </is>
       </c>
       <c r="C332" t="n">
-        <v>1.819487029827726e-09</v>
+        <v>2.831958989843268e-09</v>
       </c>
       <c r="D332" t="inlineStr">
         <is>
@@ -7411,7 +7411,7 @@
         </is>
       </c>
       <c r="C333" t="n">
-        <v>1.819487029827726e-09</v>
+        <v>2.831958989843268e-09</v>
       </c>
       <c r="D333" t="inlineStr">
         <is>
@@ -7432,7 +7432,7 @@
         </is>
       </c>
       <c r="C334" t="n">
-        <v>3.351699293248974e-06</v>
+        <v>3.331438606717563e-06</v>
       </c>
       <c r="D334" t="inlineStr">
         <is>
@@ -7453,7 +7453,7 @@
         </is>
       </c>
       <c r="C335" t="n">
-        <v>1.819487029827726e-09</v>
+        <v>2.831958989843268e-09</v>
       </c>
       <c r="D335" t="inlineStr">
         <is>
@@ -7474,7 +7474,7 @@
         </is>
       </c>
       <c r="C336" t="n">
-        <v>8.053406921383617e-06</v>
+        <v>8.053406921385313e-06</v>
       </c>
       <c r="D336" t="inlineStr">
         <is>
@@ -7495,7 +7495,7 @@
         </is>
       </c>
       <c r="C337" t="n">
-        <v>7.74928293041342e-10</v>
+        <v>1.206144979318767e-09</v>
       </c>
       <c r="D337" t="inlineStr">
         <is>
@@ -7516,7 +7516,7 @@
         </is>
       </c>
       <c r="C338" t="n">
-        <v>9.03236146884308e-09</v>
+        <v>0</v>
       </c>
       <c r="D338" t="inlineStr">
         <is>
@@ -7537,7 +7537,7 @@
         </is>
       </c>
       <c r="C339" t="n">
-        <v>9.03236146884308e-09</v>
+        <v>0</v>
       </c>
       <c r="D339" t="inlineStr">
         <is>
@@ -7663,7 +7663,7 @@
         </is>
       </c>
       <c r="C345" t="n">
-        <v>2.115568481418949e-06</v>
+        <v>2.115568481418958e-06</v>
       </c>
       <c r="D345" t="inlineStr">
         <is>
@@ -7894,7 +7894,7 @@
         </is>
       </c>
       <c r="C356" t="n">
-        <v>4.190210775583306e-05</v>
+        <v>3.988978407642667e-05</v>
       </c>
       <c r="D356" t="inlineStr">
         <is>
@@ -8251,7 +8251,7 @@
         </is>
       </c>
       <c r="C373" t="n">
-        <v>1.391037030162371e-06</v>
+        <v>1.39103703016237e-06</v>
       </c>
       <c r="D373" t="inlineStr">
         <is>
@@ -8272,7 +8272,7 @@
         </is>
       </c>
       <c r="C374" t="n">
-        <v>6.112671102160274e-05</v>
+        <v>6.112671102160227e-05</v>
       </c>
       <c r="D374" t="inlineStr">
         <is>
@@ -8377,7 +8377,7 @@
         </is>
       </c>
       <c r="C379" t="n">
-        <v>3.155014686592018e-07</v>
+        <v>7.408939649178085e-08</v>
       </c>
       <c r="D379" t="inlineStr">
         <is>
@@ -8503,7 +8503,7 @@
         </is>
       </c>
       <c r="C385" t="n">
-        <v>5.823194679604853e-07</v>
+        <v>5.823273632968851e-07</v>
       </c>
       <c r="D385" t="inlineStr">
         <is>
@@ -8524,7 +8524,7 @@
         </is>
       </c>
       <c r="C386" t="n">
-        <v>1.561716924777096e-06</v>
+        <v>1.561738099203095e-06</v>
       </c>
       <c r="D386" t="inlineStr">
         <is>
@@ -8608,7 +8608,7 @@
         </is>
       </c>
       <c r="C390" t="n">
-        <v>9.168719945223332e-06</v>
+        <v>9.168719945223369e-06</v>
       </c>
       <c r="D390" t="inlineStr">
         <is>
@@ -8671,7 +8671,7 @@
         </is>
       </c>
       <c r="C393" t="n">
-        <v>4.94573017980073e-05</v>
+        <v>0</v>
       </c>
       <c r="D393" t="inlineStr">
         <is>
@@ -8713,7 +8713,7 @@
         </is>
       </c>
       <c r="C395" t="n">
-        <v>7.672902048202971e-06</v>
+        <v>7.672902048206029e-06</v>
       </c>
       <c r="D395" t="inlineStr">
         <is>
@@ -8776,7 +8776,7 @@
         </is>
       </c>
       <c r="C398" t="n">
-        <v>9.464012881355822e-06</v>
+        <v>1.399152629986029e-05</v>
       </c>
       <c r="D398" t="inlineStr">
         <is>
@@ -8797,7 +8797,7 @@
         </is>
       </c>
       <c r="C399" t="n">
-        <v>9.464012881355822e-06</v>
+        <v>1.399152629986029e-05</v>
       </c>
       <c r="D399" t="inlineStr">
         <is>
@@ -8902,7 +8902,7 @@
         </is>
       </c>
       <c r="C404" t="n">
-        <v>8.295488353790388e-06</v>
+        <v>8.295600827569403e-06</v>
       </c>
       <c r="D404" t="inlineStr">
         <is>
@@ -8923,7 +8923,7 @@
         </is>
       </c>
       <c r="C405" t="n">
-        <v>8.823868704185921e-09</v>
+        <v>0</v>
       </c>
       <c r="D405" t="inlineStr">
         <is>
@@ -8944,7 +8944,7 @@
         </is>
       </c>
       <c r="C406" t="n">
-        <v>8.823868704185921e-09</v>
+        <v>0</v>
       </c>
       <c r="D406" t="inlineStr">
         <is>
@@ -8965,7 +8965,7 @@
         </is>
       </c>
       <c r="C407" t="n">
-        <v>1.412469141054287e-06</v>
+        <v>1.412469141054455e-06</v>
       </c>
       <c r="D407" t="inlineStr">
         <is>
@@ -9154,7 +9154,7 @@
         </is>
       </c>
       <c r="C416" t="n">
-        <v>3.142248853933954e-05</v>
+        <v>3.142248853934328e-05</v>
       </c>
       <c r="D416" t="inlineStr">
         <is>
@@ -9175,7 +9175,7 @@
         </is>
       </c>
       <c r="C417" t="n">
-        <v>2.960480122238335e-07</v>
+        <v>6.952112981111937e-08</v>
       </c>
       <c r="D417" t="inlineStr">
         <is>
@@ -9322,7 +9322,7 @@
         </is>
       </c>
       <c r="C424" t="n">
-        <v>9.14549142354481e-06</v>
+        <v>1.054576669368036e-05</v>
       </c>
       <c r="D424" t="inlineStr">
         <is>
@@ -9406,7 +9406,7 @@
         </is>
       </c>
       <c r="C428" t="n">
-        <v>3.652620544906112e-06</v>
+        <v>6.430857242503712e-06</v>
       </c>
       <c r="D428" t="inlineStr">
         <is>
@@ -9490,7 +9490,7 @@
         </is>
       </c>
       <c r="C432" t="n">
-        <v>2.478894347194059e-06</v>
+        <v>2.48996199183861e-06</v>
       </c>
       <c r="D432" t="inlineStr">
         <is>
@@ -9595,7 +9595,7 @@
         </is>
       </c>
       <c r="C437" t="n">
-        <v>1.412785496600663e-06</v>
+        <v>1.412804651750662e-06</v>
       </c>
       <c r="D437" t="inlineStr">
         <is>
@@ -9616,7 +9616,7 @@
         </is>
       </c>
       <c r="C438" t="n">
-        <v>8.475501511532414e-05</v>
+        <v>8.47561642600681e-05</v>
       </c>
       <c r="D438" t="inlineStr">
         <is>
@@ -9805,7 +9805,7 @@
         </is>
       </c>
       <c r="C447" t="n">
-        <v>3.044358673363892e-07</v>
+        <v>3.044358673364254e-07</v>
       </c>
       <c r="D447" t="inlineStr">
         <is>
@@ -9952,7 +9952,7 @@
         </is>
       </c>
       <c r="C454" t="n">
-        <v>1.945389246929855e-06</v>
+        <v>1.945389246930087e-06</v>
       </c>
       <c r="D454" t="inlineStr">
         <is>
@@ -9994,7 +9994,7 @@
         </is>
       </c>
       <c r="C456" t="n">
-        <v>0.0001338855933464049</v>
+        <v>0.0001526247714053364</v>
       </c>
       <c r="D456" t="inlineStr">
         <is>
@@ -10120,7 +10120,7 @@
         </is>
       </c>
       <c r="C462" t="n">
-        <v>2.879673293258735e-07</v>
+        <v>2.879673293259079e-07</v>
       </c>
       <c r="D462" t="inlineStr">
         <is>
@@ -10141,7 +10141,7 @@
         </is>
       </c>
       <c r="C463" t="n">
-        <v>3.367245842450763e-05</v>
+        <v>3.367245842451165e-05</v>
       </c>
       <c r="D463" t="inlineStr">
         <is>
@@ -10183,7 +10183,7 @@
         </is>
       </c>
       <c r="C465" t="n">
-        <v>1.720220600355917e-05</v>
+        <v>1.720547641326461e-05</v>
       </c>
       <c r="D465" t="inlineStr">
         <is>
@@ -10246,7 +10246,7 @@
         </is>
       </c>
       <c r="C468" t="n">
-        <v>4.029957332166645e-07</v>
+        <v>0</v>
       </c>
       <c r="D468" t="inlineStr">
         <is>
@@ -10330,7 +10330,7 @@
         </is>
       </c>
       <c r="C472" t="n">
-        <v>1.007504546556566e-07</v>
+        <v>1.007504546556567e-07</v>
       </c>
       <c r="D472" t="inlineStr">
         <is>
@@ -10372,7 +10372,7 @@
         </is>
       </c>
       <c r="C474" t="n">
-        <v>6.278904861846259e-07</v>
+        <v>6.278904861846264e-07</v>
       </c>
       <c r="D474" t="inlineStr">
         <is>
@@ -10393,7 +10393,7 @@
         </is>
       </c>
       <c r="C475" t="n">
-        <v>1.064699580000991e-08</v>
+        <v>1.064699579998028e-08</v>
       </c>
       <c r="D475" t="inlineStr">
         <is>
@@ -10414,7 +10414,7 @@
         </is>
       </c>
       <c r="C476" t="n">
-        <v>6.528428532533693e-07</v>
+        <v>6.528428532515527e-07</v>
       </c>
       <c r="D476" t="inlineStr">
         <is>
@@ -10435,7 +10435,7 @@
         </is>
       </c>
       <c r="C477" t="n">
-        <v>6.926304840006445e-09</v>
+        <v>6.926304839987173e-09</v>
       </c>
       <c r="D477" t="inlineStr">
         <is>
@@ -10540,7 +10540,7 @@
         </is>
       </c>
       <c r="C482" t="n">
-        <v>3.908024410663865e-06</v>
+        <v>3.908024410665979e-06</v>
       </c>
       <c r="D482" t="inlineStr">
         <is>
@@ -10582,7 +10582,7 @@
         </is>
       </c>
       <c r="C484" t="n">
-        <v>5.612518125604202e-05</v>
+        <v>5.612518125604157e-05</v>
       </c>
       <c r="D484" t="inlineStr">
         <is>
@@ -10624,7 +10624,7 @@
         </is>
       </c>
       <c r="C486" t="n">
-        <v>7.150912307296414e-05</v>
+        <v>6.765495931618091e-05</v>
       </c>
       <c r="D486" t="inlineStr">
         <is>
@@ -10729,7 +10729,7 @@
         </is>
       </c>
       <c r="C491" t="n">
-        <v>1.582560561313729e-05</v>
+        <v>1.583728620940058e-05</v>
       </c>
       <c r="D491" t="inlineStr">
         <is>
@@ -10771,7 +10771,7 @@
         </is>
       </c>
       <c r="C493" t="n">
-        <v>2.397027449505794e-05</v>
+        <v>2.325411106662185e-05</v>
       </c>
       <c r="D493" t="inlineStr">
         <is>
@@ -10834,7 +10834,7 @@
         </is>
       </c>
       <c r="C496" t="n">
-        <v>1.492065043198264e-06</v>
+        <v>1.492085273254263e-06</v>
       </c>
       <c r="D496" t="inlineStr">
         <is>
@@ -10855,7 +10855,7 @@
         </is>
       </c>
       <c r="C497" t="n">
-        <v>1.416511867987149e-07</v>
+        <v>1.416511867983208e-07</v>
       </c>
       <c r="D497" t="inlineStr">
         <is>
@@ -10876,7 +10876,7 @@
         </is>
       </c>
       <c r="C498" t="n">
-        <v>1.175454000001094e-09</v>
+        <v>1.175453999997823e-09</v>
       </c>
       <c r="D498" t="inlineStr">
         <is>
@@ -10960,7 +10960,7 @@
         </is>
       </c>
       <c r="C502" t="n">
-        <v>5.875392974472259e-07</v>
+        <v>5.875392974475436e-07</v>
       </c>
       <c r="D502" t="inlineStr">
         <is>
@@ -10981,7 +10981,7 @@
         </is>
       </c>
       <c r="C503" t="n">
-        <v>9.653352267070088e-06</v>
+        <v>9.653352267075309e-06</v>
       </c>
       <c r="D503" t="inlineStr">
         <is>
@@ -11002,7 +11002,7 @@
         </is>
       </c>
       <c r="C504" t="n">
-        <v>1.681996564325014e-07</v>
+        <v>1.68199656432517e-07</v>
       </c>
       <c r="D504" t="inlineStr">
         <is>
@@ -11023,7 +11023,7 @@
         </is>
       </c>
       <c r="C505" t="n">
-        <v>1.059344242318379e-05</v>
+        <v>1.059344242318952e-05</v>
       </c>
       <c r="D505" t="inlineStr">
         <is>
@@ -11065,7 +11065,7 @@
         </is>
       </c>
       <c r="C507" t="n">
-        <v>3.544771323958096e-07</v>
+        <v>3.544771323958859e-07</v>
       </c>
       <c r="D507" t="inlineStr">
         <is>
@@ -11107,7 +11107,7 @@
         </is>
       </c>
       <c r="C509" t="n">
-        <v>3.544771323958096e-07</v>
+        <v>3.544771323958859e-07</v>
       </c>
       <c r="D509" t="inlineStr">
         <is>
@@ -11149,7 +11149,7 @@
         </is>
       </c>
       <c r="C511" t="n">
-        <v>3.057955815939011e-06</v>
+        <v>3.060212838396801e-06</v>
       </c>
       <c r="D511" t="inlineStr">
         <is>
@@ -11170,7 +11170,7 @@
         </is>
       </c>
       <c r="C512" t="n">
-        <v>1.007174697103049e-05</v>
+        <v>1.007918074721009e-05</v>
       </c>
       <c r="D512" t="inlineStr">
         <is>
@@ -11317,7 +11317,7 @@
         </is>
       </c>
       <c r="C519" t="n">
-        <v>0</v>
+        <v>6.829346999999999e-12</v>
       </c>
       <c r="D519" t="inlineStr">
         <is>
@@ -11422,7 +11422,7 @@
         </is>
       </c>
       <c r="C524" t="n">
-        <v>1.743847977761864e-05</v>
+        <v>2.022956396657305e-05</v>
       </c>
       <c r="D524" t="inlineStr">
         <is>
@@ -11443,7 +11443,7 @@
         </is>
       </c>
       <c r="C525" t="n">
-        <v>1.66500352472282e-06</v>
+        <v>1.662893073619594e-06</v>
       </c>
       <c r="D525" t="inlineStr">
         <is>
@@ -11464,7 +11464,7 @@
         </is>
       </c>
       <c r="C526" t="n">
-        <v>1.66500352472282e-06</v>
+        <v>1.662893073619594e-06</v>
       </c>
       <c r="D526" t="inlineStr">
         <is>
@@ -11485,7 +11485,7 @@
         </is>
       </c>
       <c r="C527" t="n">
-        <v>1.66500352472282e-06</v>
+        <v>1.662893073619594e-06</v>
       </c>
       <c r="D527" t="inlineStr">
         <is>
@@ -11506,7 +11506,7 @@
         </is>
       </c>
       <c r="C528" t="n">
-        <v>1.66500352472282e-06</v>
+        <v>1.662893073619594e-06</v>
       </c>
       <c r="D528" t="inlineStr">
         <is>
@@ -11548,7 +11548,7 @@
         </is>
       </c>
       <c r="C530" t="n">
-        <v>8.070423186588362e-05</v>
+        <v>7.823076358556982e-05</v>
       </c>
       <c r="D530" t="inlineStr">
         <is>
@@ -11569,7 +11569,7 @@
         </is>
       </c>
       <c r="C531" t="n">
-        <v>2.070847799999997e-10</v>
+        <v>2.0708478e-10</v>
       </c>
       <c r="D531" t="inlineStr">
         <is>
@@ -11716,7 +11716,7 @@
         </is>
       </c>
       <c r="C538" t="n">
-        <v>5.600502645293783e-06</v>
+        <v>5.601355121791818e-06</v>
       </c>
       <c r="D538" t="inlineStr">
         <is>
@@ -11758,7 +11758,7 @@
         </is>
       </c>
       <c r="C540" t="n">
-        <v>6.071779770794277e-07</v>
+        <v>6.073328807716416e-07</v>
       </c>
       <c r="D540" t="inlineStr">
         <is>
@@ -11863,7 +11863,7 @@
         </is>
       </c>
       <c r="C545" t="n">
-        <v>0</v>
+        <v>1.482845398789235e-07</v>
       </c>
       <c r="D545" t="inlineStr">
         <is>
@@ -11884,7 +11884,7 @@
         </is>
       </c>
       <c r="C546" t="n">
-        <v>0</v>
+        <v>1.482845398789235e-07</v>
       </c>
       <c r="D546" t="inlineStr">
         <is>
@@ -12073,7 +12073,7 @@
         </is>
       </c>
       <c r="C555" t="n">
-        <v>1.071554400000997e-10</v>
+        <v>1.071554399998016e-10</v>
       </c>
       <c r="D555" t="inlineStr">
         <is>
@@ -12199,7 +12199,7 @@
         </is>
       </c>
       <c r="C561" t="n">
-        <v>5.051094701391905e-07</v>
+        <v>4.892948614608902e-07</v>
       </c>
       <c r="D561" t="inlineStr">
         <is>
@@ -12220,7 +12220,7 @@
         </is>
       </c>
       <c r="C562" t="n">
-        <v>5.051094701391905e-07</v>
+        <v>4.892948614608902e-07</v>
       </c>
       <c r="D562" t="inlineStr">
         <is>
@@ -12241,7 +12241,7 @@
         </is>
       </c>
       <c r="C563" t="n">
-        <v>5.051094701391905e-07</v>
+        <v>4.892948614608902e-07</v>
       </c>
       <c r="D563" t="inlineStr">
         <is>
@@ -12325,7 +12325,7 @@
         </is>
       </c>
       <c r="C567" t="n">
-        <v>4.121251366243663e-06</v>
+        <v>4.12125136624363e-06</v>
       </c>
       <c r="D567" t="inlineStr">
         <is>
@@ -12346,7 +12346,7 @@
         </is>
       </c>
       <c r="C568" t="n">
-        <v>1.007237251090195e-06</v>
+        <v>1.007237251090187e-06</v>
       </c>
       <c r="D568" t="inlineStr">
         <is>
@@ -12367,7 +12367,7 @@
         </is>
       </c>
       <c r="C569" t="n">
-        <v>1.007237251090195e-06</v>
+        <v>1.007237251090187e-06</v>
       </c>
       <c r="D569" t="inlineStr">
         <is>
@@ -12451,7 +12451,7 @@
         </is>
       </c>
       <c r="C573" t="n">
-        <v>5.001529765560731e-06</v>
+        <v>5.001529765560697e-06</v>
       </c>
       <c r="D573" t="inlineStr">
         <is>
@@ -12598,7 +12598,7 @@
         </is>
       </c>
       <c r="C580" t="n">
-        <v>1.937706215416395e-05</v>
+        <v>1.828837999151935e-05</v>
       </c>
       <c r="D580" t="inlineStr">
         <is>
@@ -12619,7 +12619,7 @@
         </is>
       </c>
       <c r="C581" t="n">
-        <v>2.664899708156437e-05</v>
+        <v>2.665518524973222e-05</v>
       </c>
       <c r="D581" t="inlineStr">
         <is>
@@ -12661,7 +12661,7 @@
         </is>
       </c>
       <c r="C583" t="n">
-        <v>3.50918139113354e-06</v>
+        <v>3.490816307458154e-06</v>
       </c>
       <c r="D583" t="inlineStr">
         <is>
@@ -12682,7 +12682,7 @@
         </is>
       </c>
       <c r="C584" t="n">
-        <v>9.515076596646934e-06</v>
+        <v>9.51507659664782e-06</v>
       </c>
       <c r="D584" t="inlineStr">
         <is>
@@ -12913,7 +12913,7 @@
         </is>
       </c>
       <c r="C595" t="n">
-        <v>0</v>
+        <v>5.996255999999999e-12</v>
       </c>
       <c r="D595" t="inlineStr">
         <is>
@@ -13144,7 +13144,7 @@
         </is>
       </c>
       <c r="C606" t="n">
-        <v>1.541795633422876e-05</v>
+        <v>0</v>
       </c>
       <c r="D606" t="inlineStr">
         <is>
@@ -13165,7 +13165,7 @@
         </is>
       </c>
       <c r="C607" t="n">
-        <v>9.506962317527592e-06</v>
+        <v>9.506962317527578e-06</v>
       </c>
       <c r="D607" t="inlineStr">
         <is>
@@ -13186,7 +13186,7 @@
         </is>
       </c>
       <c r="C608" t="n">
-        <v>9.506962317527592e-06</v>
+        <v>9.506962317527578e-06</v>
       </c>
       <c r="D608" t="inlineStr">
         <is>
@@ -13354,7 +13354,7 @@
         </is>
       </c>
       <c r="C616" t="n">
-        <v>2.980406935491901e-07</v>
+        <v>2.980406935491898e-07</v>
       </c>
       <c r="D616" t="inlineStr">
         <is>
@@ -13396,7 +13396,7 @@
         </is>
       </c>
       <c r="C618" t="n">
-        <v>3.330403817508616e-09</v>
+        <v>6.479099831243786e-09</v>
       </c>
       <c r="D618" t="inlineStr">
         <is>
@@ -13459,7 +13459,7 @@
         </is>
       </c>
       <c r="C621" t="n">
-        <v>1.644641527588539e-07</v>
+        <v>1.651996446181178e-07</v>
       </c>
       <c r="D621" t="inlineStr">
         <is>
@@ -13480,7 +13480,7 @@
         </is>
       </c>
       <c r="C622" t="n">
-        <v>1.204406279272527e-06</v>
+        <v>1.204406279272523e-06</v>
       </c>
       <c r="D622" t="inlineStr">
         <is>
@@ -13522,7 +13522,7 @@
         </is>
       </c>
       <c r="C624" t="n">
-        <v>2.460137982377647e-06</v>
+        <v>1.009829731392414e-06</v>
       </c>
       <c r="D624" t="inlineStr">
         <is>
@@ -13543,7 +13543,7 @@
         </is>
       </c>
       <c r="C625" t="n">
-        <v>4.948280078568954e-07</v>
+        <v>1.050154490315313e-06</v>
       </c>
       <c r="D625" t="inlineStr">
         <is>
@@ -13648,7 +13648,7 @@
         </is>
       </c>
       <c r="C630" t="n">
-        <v>5.431140932267017e-08</v>
+        <v>8.675034109564556e-08</v>
       </c>
       <c r="D630" t="inlineStr">
         <is>
@@ -13669,7 +13669,7 @@
         </is>
       </c>
       <c r="C631" t="n">
-        <v>1.263781464514028e-06</v>
+        <v>1.218672196655907e-06</v>
       </c>
       <c r="D631" t="inlineStr">
         <is>
@@ -13690,7 +13690,7 @@
         </is>
       </c>
       <c r="C632" t="n">
-        <v>5.039266493460528e-07</v>
+        <v>6.118208501905272e-07</v>
       </c>
       <c r="D632" t="inlineStr">
         <is>
@@ -13711,7 +13711,7 @@
         </is>
       </c>
       <c r="C633" t="n">
-        <v>9.305987680169555e-08</v>
+        <v>9.305987680169556e-08</v>
       </c>
       <c r="D633" t="inlineStr">
         <is>
@@ -13753,7 +13753,7 @@
         </is>
       </c>
       <c r="C635" t="n">
-        <v>4.271464610655413e-07</v>
+        <v>6.312478944201185e-07</v>
       </c>
       <c r="D635" t="inlineStr">
         <is>
@@ -13774,7 +13774,7 @@
         </is>
       </c>
       <c r="C636" t="n">
-        <v>2.47840202364158e-08</v>
+        <v>8.97059651436576e-08</v>
       </c>
       <c r="D636" t="inlineStr">
         <is>
@@ -13795,7 +13795,7 @@
         </is>
       </c>
       <c r="C637" t="n">
-        <v>3.824660392198851e-06</v>
+        <v>3.318377802769983e-06</v>
       </c>
       <c r="D637" t="inlineStr">
         <is>
@@ -14068,7 +14068,7 @@
         </is>
       </c>
       <c r="C650" t="n">
-        <v>1.297639553658393e-07</v>
+        <v>0</v>
       </c>
       <c r="D650" t="inlineStr">
         <is>
@@ -14824,7 +14824,7 @@
         </is>
       </c>
       <c r="C686" t="n">
-        <v>1.208511016474748e-05</v>
+        <v>1.382913232035101e-05</v>
       </c>
       <c r="D686" t="inlineStr">
         <is>
@@ -14887,7 +14887,7 @@
         </is>
       </c>
       <c r="C689" t="n">
-        <v>1.145385136341727e-05</v>
+        <v>1.20142523386676e-05</v>
       </c>
       <c r="D689" t="inlineStr">
         <is>
@@ -14992,7 +14992,7 @@
         </is>
       </c>
       <c r="C694" t="n">
-        <v>3.974428570793885e-06</v>
+        <v>3.974652039655661e-06</v>
       </c>
       <c r="D694" t="inlineStr">
         <is>
@@ -15034,7 +15034,7 @@
         </is>
       </c>
       <c r="C696" t="n">
-        <v>5.864097385130594e-05</v>
+        <v>6.730817351892377e-05</v>
       </c>
       <c r="D696" t="inlineStr">
         <is>
@@ -15265,7 +15265,7 @@
         </is>
       </c>
       <c r="C707" t="n">
-        <v>7.245530258039204e-05</v>
+        <v>6.89756799816749e-05</v>
       </c>
       <c r="D707" t="inlineStr">
         <is>
@@ -15412,7 +15412,7 @@
         </is>
       </c>
       <c r="C714" t="n">
-        <v>8.464855054655803e-06</v>
+        <v>8.529813552245564e-06</v>
       </c>
       <c r="D714" t="inlineStr">
         <is>
@@ -15496,7 +15496,7 @@
         </is>
       </c>
       <c r="C718" t="n">
-        <v>8.571183936e-10</v>
+        <v>8.853130776000001e-10</v>
       </c>
       <c r="D718" t="inlineStr">
         <is>
@@ -15559,7 +15559,7 @@
         </is>
       </c>
       <c r="C721" t="n">
-        <v>0</v>
+        <v>3.934874999999999e-10</v>
       </c>
       <c r="D721" t="inlineStr">
         <is>
@@ -15643,7 +15643,7 @@
         </is>
       </c>
       <c r="C725" t="n">
-        <v>5.176013422206758e-09</v>
+        <v>8.056258441125429e-09</v>
       </c>
       <c r="D725" t="inlineStr">
         <is>
@@ -15832,7 +15832,7 @@
         </is>
       </c>
       <c r="C734" t="n">
-        <v>4.921512027174269e-08</v>
+        <v>6.963030735643235e-06</v>
       </c>
       <c r="D734" t="inlineStr">
         <is>
@@ -15979,7 +15979,7 @@
         </is>
       </c>
       <c r="C741" t="n">
-        <v>0.0001720108659936563</v>
+        <v>0.0001846348662768155</v>
       </c>
       <c r="D741" t="inlineStr">
         <is>
@@ -16210,7 +16210,7 @@
         </is>
       </c>
       <c r="C752" t="n">
-        <v>2.427543057984982e-06</v>
+        <v>2.427543057984967e-06</v>
       </c>
       <c r="D752" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat: add function to calibrate the kcat value of a model
</commit_message>
<xml_diff>
--- a/data/data_check.xlsx
+++ b/data/data_check.xlsx
@@ -481,7 +481,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>2.649843398175449e-05</v>
+        <v>3.858702760649158e-05</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -502,7 +502,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1.482276902352393e-06</v>
+        <v>0</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -733,7 +733,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>2.752653119994902e-09</v>
+        <v>2.752653119990803e-09</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>2.752653119994902e-09</v>
+        <v>2.752653119990803e-09</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -838,7 +838,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>3.885749768074303e-06</v>
+        <v>3.885749768074301e-06</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -859,7 +859,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>5.982297078224262e-08</v>
+        <v>5.982297078222703e-08</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -901,7 +901,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>6.205356391217201e-06</v>
+        <v>6.205356391217212e-06</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -943,7 +943,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1.247665019997689e-09</v>
+        <v>1.247665019995831e-09</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -964,7 +964,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>6.062354394289476e-06</v>
+        <v>6.062354394289452e-06</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -1216,7 +1216,7 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>1.221345214330621e-05</v>
+        <v>1.221345214330625e-05</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -1258,7 +1258,7 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>8.184989591592579e-07</v>
+        <v>8.18498959159254e-07</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -1342,7 +1342,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>1.673044278148202e-05</v>
+        <v>1.673044278148195e-05</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -1426,7 +1426,7 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>4.943958551471168e-06</v>
+        <v>4.9439585514711e-06</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -1468,7 +1468,7 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>2.796073369360335e-07</v>
+        <v>2.796073369360297e-07</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -1573,7 +1573,7 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>6.935824979987155e-08</v>
+        <v>6.935824979976827e-08</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
@@ -1615,7 +1615,7 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>2.916005652000083e-09</v>
+        <v>2.916005651999324e-09</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
@@ -1636,7 +1636,7 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>6.613463220000188e-10</v>
+        <v>6.613463219998466e-10</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -1762,7 +1762,7 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>1.124529531910742e-08</v>
+        <v>1.124529531909067e-08</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
@@ -1825,7 +1825,7 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>2.500714733124178e-06</v>
+        <v>2.50071473312378e-06</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -1846,7 +1846,7 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>3.167705113852122e-07</v>
+        <v>3.157728388273484e-07</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
@@ -1888,7 +1888,7 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>0</v>
+        <v>5.776257884475657e-10</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
@@ -1930,7 +1930,7 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>1.375930054748013e-06</v>
+        <v>1.371596546394728e-06</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
@@ -1951,7 +1951,7 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>5.821585559989219e-11</v>
+        <v>5.82158555998055e-11</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -1972,7 +1972,7 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>2.077888259996152e-09</v>
+        <v>2.077888259993057e-09</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
@@ -2014,7 +2014,7 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>8.939387940576949e-06</v>
+        <v>8.937537328406136e-06</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -2056,7 +2056,7 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>3.504715355317637e-05</v>
+        <v>3.504715355317636e-05</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
@@ -2161,7 +2161,7 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>4.670169127491606e-05</v>
+        <v>1.62505245105974e-05</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
@@ -2350,7 +2350,7 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>3.619903559993297e-10</v>
+        <v>3.619903559987906e-10</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
@@ -2392,7 +2392,7 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>9.091859078054608e-06</v>
+        <v>9.051392149085006e-06</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
@@ -2434,7 +2434,7 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>1.093645671937287e-05</v>
+        <v>1.088777967615844e-05</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
@@ -2455,7 +2455,7 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>1.928925599996428e-09</v>
+        <v>1.928925599993556e-09</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
@@ -2497,7 +2497,7 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>0.0001699766665603495</v>
+        <v>0.0001696874844344086</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
@@ -2560,7 +2560,7 @@
         </is>
       </c>
       <c r="C102" t="n">
-        <v>3.564776883976501e-06</v>
+        <v>3.564776883975961e-06</v>
       </c>
       <c r="D102" t="inlineStr">
         <is>
@@ -2581,7 +2581,7 @@
         </is>
       </c>
       <c r="C103" t="n">
-        <v>5.051445635983571e-06</v>
+        <v>5.051445635982867e-06</v>
       </c>
       <c r="D103" t="inlineStr">
         <is>
@@ -2602,7 +2602,7 @@
         </is>
       </c>
       <c r="C104" t="n">
-        <v>1.40495500345564e-06</v>
+        <v>1.404955003455633e-06</v>
       </c>
       <c r="D104" t="inlineStr">
         <is>
@@ -2833,7 +2833,7 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>1.874382950969299e-05</v>
+        <v>1.518947536584058e-05</v>
       </c>
       <c r="D115" t="inlineStr">
         <is>
@@ -2875,7 +2875,7 @@
         </is>
       </c>
       <c r="C117" t="n">
-        <v>1.151426219997868e-09</v>
+        <v>1.151426219996153e-09</v>
       </c>
       <c r="D117" t="inlineStr">
         <is>
@@ -3379,7 +3379,7 @@
         </is>
       </c>
       <c r="C141" t="n">
-        <v>9.384927839054706e-06</v>
+        <v>9.384927839054606e-06</v>
       </c>
       <c r="D141" t="inlineStr">
         <is>
@@ -3400,7 +3400,7 @@
         </is>
       </c>
       <c r="C142" t="n">
-        <v>1.74744109508397e-06</v>
+        <v>1.747441095083951e-06</v>
       </c>
       <c r="D142" t="inlineStr">
         <is>
@@ -3421,7 +3421,7 @@
         </is>
       </c>
       <c r="C143" t="n">
-        <v>4.393683013560853e-06</v>
+        <v>4.393683013560806e-06</v>
       </c>
       <c r="D143" t="inlineStr">
         <is>
@@ -3631,7 +3631,7 @@
         </is>
       </c>
       <c r="C153" t="n">
-        <v>2.292547375478711e-06</v>
+        <v>2.292547375478712e-06</v>
       </c>
       <c r="D153" t="inlineStr">
         <is>
@@ -3652,7 +3652,7 @@
         </is>
       </c>
       <c r="C154" t="n">
-        <v>3.983907490299623e-07</v>
+        <v>3.983907490299624e-07</v>
       </c>
       <c r="D154" t="inlineStr">
         <is>
@@ -3673,7 +3673,7 @@
         </is>
       </c>
       <c r="C155" t="n">
-        <v>4.434805821719214e-06</v>
+        <v>5.668357701705465e-06</v>
       </c>
       <c r="D155" t="inlineStr">
         <is>
@@ -3694,7 +3694,7 @@
         </is>
       </c>
       <c r="C156" t="n">
-        <v>3.486454734573162e-05</v>
+        <v>4.293240657773285e-05</v>
       </c>
       <c r="D156" t="inlineStr">
         <is>
@@ -3820,7 +3820,7 @@
         </is>
       </c>
       <c r="C162" t="n">
-        <v>2.691099396024619e-06</v>
+        <v>3.797553160871518e-06</v>
       </c>
       <c r="D162" t="inlineStr">
         <is>
@@ -3841,7 +3841,7 @@
         </is>
       </c>
       <c r="C163" t="n">
-        <v>8.970304333606933e-07</v>
+        <v>1.26584724541913e-06</v>
       </c>
       <c r="D163" t="inlineStr">
         <is>
@@ -3862,7 +3862,7 @@
         </is>
       </c>
       <c r="C164" t="n">
-        <v>8.970304333606933e-07</v>
+        <v>1.26584724541913e-06</v>
       </c>
       <c r="D164" t="inlineStr">
         <is>
@@ -3883,7 +3883,7 @@
         </is>
       </c>
       <c r="C165" t="n">
-        <v>1.794060866721387e-06</v>
+        <v>2.53169449083826e-06</v>
       </c>
       <c r="D165" t="inlineStr">
         <is>
@@ -3925,7 +3925,7 @@
         </is>
       </c>
       <c r="C167" t="n">
-        <v>1.794060866721387e-06</v>
+        <v>2.53169449083826e-06</v>
       </c>
       <c r="D167" t="inlineStr">
         <is>
@@ -3946,7 +3946,7 @@
         </is>
       </c>
       <c r="C168" t="n">
-        <v>2.691099396024619e-06</v>
+        <v>3.797553160871518e-06</v>
       </c>
       <c r="D168" t="inlineStr">
         <is>
@@ -3967,7 +3967,7 @@
         </is>
       </c>
       <c r="C169" t="n">
-        <v>1.794060866721387e-06</v>
+        <v>2.53169449083826e-06</v>
       </c>
       <c r="D169" t="inlineStr">
         <is>
@@ -3988,7 +3988,7 @@
         </is>
       </c>
       <c r="C170" t="n">
-        <v>8.970304333606933e-07</v>
+        <v>1.26584724541913e-06</v>
       </c>
       <c r="D170" t="inlineStr">
         <is>
@@ -4009,7 +4009,7 @@
         </is>
       </c>
       <c r="C171" t="n">
-        <v>1.794060866721387e-06</v>
+        <v>2.53169449083826e-06</v>
       </c>
       <c r="D171" t="inlineStr">
         <is>
@@ -4030,7 +4030,7 @@
         </is>
       </c>
       <c r="C172" t="n">
-        <v>1.794060866721387e-06</v>
+        <v>2.53169449083826e-06</v>
       </c>
       <c r="D172" t="inlineStr">
         <is>
@@ -4051,7 +4051,7 @@
         </is>
       </c>
       <c r="C173" t="n">
-        <v>8.970304333606933e-07</v>
+        <v>1.26584724541913e-06</v>
       </c>
       <c r="D173" t="inlineStr">
         <is>
@@ -4072,7 +4072,7 @@
         </is>
       </c>
       <c r="C174" t="n">
-        <v>8.970304333606933e-07</v>
+        <v>1.26584724541913e-06</v>
       </c>
       <c r="D174" t="inlineStr">
         <is>
@@ -4345,7 +4345,7 @@
         </is>
       </c>
       <c r="C187" t="n">
-        <v>4.092129574456177e-05</v>
+        <v>3.785413262202465e-06</v>
       </c>
       <c r="D187" t="inlineStr">
         <is>
@@ -4765,7 +4765,7 @@
         </is>
       </c>
       <c r="C207" t="n">
-        <v>3.088147873660049e-05</v>
+        <v>3.088147873660037e-05</v>
       </c>
       <c r="D207" t="inlineStr">
         <is>
@@ -4786,7 +4786,7 @@
         </is>
       </c>
       <c r="C208" t="n">
-        <v>2.834381049774056e-07</v>
+        <v>4.937565777209873e-07</v>
       </c>
       <c r="D208" t="inlineStr">
         <is>
@@ -4912,7 +4912,7 @@
         </is>
       </c>
       <c r="C214" t="n">
-        <v>1.663221200699061e-07</v>
+        <v>1.663221200699064e-07</v>
       </c>
       <c r="D214" t="inlineStr">
         <is>
@@ -4954,7 +4954,7 @@
         </is>
       </c>
       <c r="C216" t="n">
-        <v>0</v>
+        <v>2.234009294435445e-07</v>
       </c>
       <c r="D216" t="inlineStr">
         <is>
@@ -5017,7 +5017,7 @@
         </is>
       </c>
       <c r="C219" t="n">
-        <v>1.707609041973026e-06</v>
+        <v>1.480056394777041e-06</v>
       </c>
       <c r="D219" t="inlineStr">
         <is>
@@ -5227,7 +5227,7 @@
         </is>
       </c>
       <c r="C229" t="n">
-        <v>0.0002458742248587892</v>
+        <v>0.0002086795659005535</v>
       </c>
       <c r="D229" t="inlineStr">
         <is>
@@ -5269,7 +5269,7 @@
         </is>
       </c>
       <c r="C231" t="n">
-        <v>1.234278812436112e-08</v>
+        <v>7.8573977883609e-09</v>
       </c>
       <c r="D231" t="inlineStr">
         <is>
@@ -5353,7 +5353,7 @@
         </is>
       </c>
       <c r="C235" t="n">
-        <v>1.266507790548001e-07</v>
+        <v>1.266507790547995e-07</v>
       </c>
       <c r="D235" t="inlineStr">
         <is>
@@ -5374,7 +5374,7 @@
         </is>
       </c>
       <c r="C236" t="n">
-        <v>8.514356256000243e-12</v>
+        <v>8.514356255998025e-12</v>
       </c>
       <c r="D236" t="inlineStr">
         <is>
@@ -5395,7 +5395,7 @@
         </is>
       </c>
       <c r="C237" t="n">
-        <v>5.014718100000143e-10</v>
+        <v>5.014718099998837e-10</v>
       </c>
       <c r="D237" t="inlineStr">
         <is>
@@ -5416,7 +5416,7 @@
         </is>
       </c>
       <c r="C238" t="n">
-        <v>2.623729654934093e-06</v>
+        <v>2.623729654934094e-06</v>
       </c>
       <c r="D238" t="inlineStr">
         <is>
@@ -5437,7 +5437,7 @@
         </is>
       </c>
       <c r="C239" t="n">
-        <v>1.944494344236873e-05</v>
+        <v>1.944494344236872e-05</v>
       </c>
       <c r="D239" t="inlineStr">
         <is>
@@ -5500,7 +5500,7 @@
         </is>
       </c>
       <c r="C242" t="n">
-        <v>2.47267668291286e-05</v>
+        <v>2.11643409829962e-05</v>
       </c>
       <c r="D242" t="inlineStr">
         <is>
@@ -5647,7 +5647,7 @@
         </is>
       </c>
       <c r="C249" t="n">
-        <v>3.998136239999999e-09</v>
+        <v>0</v>
       </c>
       <c r="D249" t="inlineStr">
         <is>
@@ -5941,7 +5941,7 @@
         </is>
       </c>
       <c r="C263" t="n">
-        <v>2.341720341564525e-07</v>
+        <v>3.288173851164888e-07</v>
       </c>
       <c r="D263" t="inlineStr">
         <is>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C264" t="n">
-        <v>4.683440683129051e-07</v>
+        <v>6.576347702329777e-07</v>
       </c>
       <c r="D264" t="inlineStr">
         <is>
@@ -5983,7 +5983,7 @@
         </is>
       </c>
       <c r="C265" t="n">
-        <v>2.341720341564525e-07</v>
+        <v>3.288173851164888e-07</v>
       </c>
       <c r="D265" t="inlineStr">
         <is>
@@ -6004,7 +6004,7 @@
         </is>
       </c>
       <c r="C266" t="n">
-        <v>2.341720341564525e-07</v>
+        <v>3.288173851164888e-07</v>
       </c>
       <c r="D266" t="inlineStr">
         <is>
@@ -6025,7 +6025,7 @@
         </is>
       </c>
       <c r="C267" t="n">
-        <v>2.341720341564525e-07</v>
+        <v>3.288173851164888e-07</v>
       </c>
       <c r="D267" t="inlineStr">
         <is>
@@ -6046,7 +6046,7 @@
         </is>
       </c>
       <c r="C268" t="n">
-        <v>2.341720341564525e-07</v>
+        <v>3.288173851164888e-07</v>
       </c>
       <c r="D268" t="inlineStr">
         <is>
@@ -6067,7 +6067,7 @@
         </is>
       </c>
       <c r="C269" t="n">
-        <v>2.341720341564525e-07</v>
+        <v>3.288173851164888e-07</v>
       </c>
       <c r="D269" t="inlineStr">
         <is>
@@ -6088,7 +6088,7 @@
         </is>
       </c>
       <c r="C270" t="n">
-        <v>2.341720341564525e-07</v>
+        <v>3.288173851164888e-07</v>
       </c>
       <c r="D270" t="inlineStr">
         <is>
@@ -6109,7 +6109,7 @@
         </is>
       </c>
       <c r="C271" t="n">
-        <v>2.341720341564525e-07</v>
+        <v>3.288173851164888e-07</v>
       </c>
       <c r="D271" t="inlineStr">
         <is>
@@ -6214,7 +6214,7 @@
         </is>
       </c>
       <c r="C276" t="n">
-        <v>2.603008991344158e-05</v>
+        <v>3.79293928362586e-05</v>
       </c>
       <c r="D276" t="inlineStr">
         <is>
@@ -6235,7 +6235,7 @@
         </is>
       </c>
       <c r="C277" t="n">
-        <v>2.603008991344158e-05</v>
+        <v>3.79293928362586e-05</v>
       </c>
       <c r="D277" t="inlineStr">
         <is>
@@ -6256,7 +6256,7 @@
         </is>
       </c>
       <c r="C278" t="n">
-        <v>2.603008991344158e-05</v>
+        <v>3.79293928362586e-05</v>
       </c>
       <c r="D278" t="inlineStr">
         <is>
@@ -6277,7 +6277,7 @@
         </is>
       </c>
       <c r="C279" t="n">
-        <v>2.603008991344158e-05</v>
+        <v>3.79293928362586e-05</v>
       </c>
       <c r="D279" t="inlineStr">
         <is>
@@ -6298,7 +6298,7 @@
         </is>
       </c>
       <c r="C280" t="n">
-        <v>2.603008991344158e-05</v>
+        <v>3.79293928362586e-05</v>
       </c>
       <c r="D280" t="inlineStr">
         <is>
@@ -6319,7 +6319,7 @@
         </is>
       </c>
       <c r="C281" t="n">
-        <v>2.603008991344158e-05</v>
+        <v>3.79293928362586e-05</v>
       </c>
       <c r="D281" t="inlineStr">
         <is>
@@ -6340,7 +6340,7 @@
         </is>
       </c>
       <c r="C282" t="n">
-        <v>2.603008991344158e-05</v>
+        <v>3.79293928362586e-05</v>
       </c>
       <c r="D282" t="inlineStr">
         <is>
@@ -6361,7 +6361,7 @@
         </is>
       </c>
       <c r="C283" t="n">
-        <v>2.603008991344158e-05</v>
+        <v>3.79293928362586e-05</v>
       </c>
       <c r="D283" t="inlineStr">
         <is>
@@ -6382,7 +6382,7 @@
         </is>
       </c>
       <c r="C284" t="n">
-        <v>2.603008991344158e-05</v>
+        <v>3.79293928362586e-05</v>
       </c>
       <c r="D284" t="inlineStr">
         <is>
@@ -6445,7 +6445,7 @@
         </is>
       </c>
       <c r="C287" t="n">
-        <v>7.664890881874985e-06</v>
+        <v>7.677334691740542e-06</v>
       </c>
       <c r="D287" t="inlineStr">
         <is>
@@ -6466,7 +6466,7 @@
         </is>
       </c>
       <c r="C288" t="n">
-        <v>1.312530472560445e-08</v>
+        <v>7.862972518720558e-09</v>
       </c>
       <c r="D288" t="inlineStr">
         <is>
@@ -6529,7 +6529,7 @@
         </is>
       </c>
       <c r="C291" t="n">
-        <v>6.022093703318908e-07</v>
+        <v>1.381831778078232e-06</v>
       </c>
       <c r="D291" t="inlineStr">
         <is>
@@ -6550,7 +6550,7 @@
         </is>
       </c>
       <c r="C292" t="n">
-        <v>3.116781911675664e-07</v>
+        <v>3.116781911675665e-07</v>
       </c>
       <c r="D292" t="inlineStr">
         <is>
@@ -6655,7 +6655,7 @@
         </is>
       </c>
       <c r="C297" t="n">
-        <v>5.97905953792724e-06</v>
+        <v>5.97782176634551e-06</v>
       </c>
       <c r="D297" t="inlineStr">
         <is>
@@ -6676,7 +6676,7 @@
         </is>
       </c>
       <c r="C298" t="n">
-        <v>7.462120906280369e-05</v>
+        <v>6.269720624189703e-05</v>
       </c>
       <c r="D298" t="inlineStr">
         <is>
@@ -6823,7 +6823,7 @@
         </is>
       </c>
       <c r="C305" t="n">
-        <v>2.906026837814722e-06</v>
+        <v>2.906026837814568e-06</v>
       </c>
       <c r="D305" t="inlineStr">
         <is>
@@ -7180,7 +7180,7 @@
         </is>
       </c>
       <c r="C322" t="n">
-        <v>7.625310897385459e-05</v>
+        <v>6.541725804581472e-05</v>
       </c>
       <c r="D322" t="inlineStr">
         <is>
@@ -7327,7 +7327,7 @@
         </is>
       </c>
       <c r="C329" t="n">
-        <v>1.932032168758395e-08</v>
+        <v>1.928312291417593e-08</v>
       </c>
       <c r="D329" t="inlineStr">
         <is>
@@ -7369,7 +7369,7 @@
         </is>
       </c>
       <c r="C331" t="n">
-        <v>1.4934068535189e-06</v>
+        <v>1.493406853518663e-06</v>
       </c>
       <c r="D331" t="inlineStr">
         <is>
@@ -7390,7 +7390,7 @@
         </is>
       </c>
       <c r="C332" t="n">
-        <v>2.831958989843268e-09</v>
+        <v>1.806575356339126e-09</v>
       </c>
       <c r="D332" t="inlineStr">
         <is>
@@ -7411,7 +7411,7 @@
         </is>
       </c>
       <c r="C333" t="n">
-        <v>2.831958989843268e-09</v>
+        <v>1.806575356339126e-09</v>
       </c>
       <c r="D333" t="inlineStr">
         <is>
@@ -7432,7 +7432,7 @@
         </is>
       </c>
       <c r="C334" t="n">
-        <v>3.331438606717563e-06</v>
+        <v>9.970477339385027e-06</v>
       </c>
       <c r="D334" t="inlineStr">
         <is>
@@ -7453,7 +7453,7 @@
         </is>
       </c>
       <c r="C335" t="n">
-        <v>2.831958989843268e-09</v>
+        <v>1.806575356339126e-09</v>
       </c>
       <c r="D335" t="inlineStr">
         <is>
@@ -7474,7 +7474,7 @@
         </is>
       </c>
       <c r="C336" t="n">
-        <v>8.053406921385313e-06</v>
+        <v>8.053406921384815e-06</v>
       </c>
       <c r="D336" t="inlineStr">
         <is>
@@ -7495,7 +7495,7 @@
         </is>
       </c>
       <c r="C337" t="n">
-        <v>1.206144979318767e-09</v>
+        <v>7.804274370887882e-10</v>
       </c>
       <c r="D337" t="inlineStr">
         <is>
@@ -7516,7 +7516,7 @@
         </is>
       </c>
       <c r="C338" t="n">
-        <v>0</v>
+        <v>2.690306701394838e-06</v>
       </c>
       <c r="D338" t="inlineStr">
         <is>
@@ -7537,7 +7537,7 @@
         </is>
       </c>
       <c r="C339" t="n">
-        <v>0</v>
+        <v>2.690306701394838e-06</v>
       </c>
       <c r="D339" t="inlineStr">
         <is>
@@ -7663,7 +7663,7 @@
         </is>
       </c>
       <c r="C345" t="n">
-        <v>2.115568481418958e-06</v>
+        <v>2.115568481418946e-06</v>
       </c>
       <c r="D345" t="inlineStr">
         <is>
@@ -7810,7 +7810,7 @@
         </is>
       </c>
       <c r="C352" t="n">
-        <v>1.269525482630874e-07</v>
+        <v>1.269525482630543e-07</v>
       </c>
       <c r="D352" t="inlineStr">
         <is>
@@ -7894,7 +7894,7 @@
         </is>
       </c>
       <c r="C356" t="n">
-        <v>3.988978407642667e-05</v>
+        <v>3.454495997955567e-05</v>
       </c>
       <c r="D356" t="inlineStr">
         <is>
@@ -8251,7 +8251,7 @@
         </is>
       </c>
       <c r="C373" t="n">
-        <v>1.39103703016237e-06</v>
+        <v>1.391037030162368e-06</v>
       </c>
       <c r="D373" t="inlineStr">
         <is>
@@ -8272,7 +8272,7 @@
         </is>
       </c>
       <c r="C374" t="n">
-        <v>6.112671102160227e-05</v>
+        <v>6.112671102160197e-05</v>
       </c>
       <c r="D374" t="inlineStr">
         <is>
@@ -8377,7 +8377,7 @@
         </is>
       </c>
       <c r="C379" t="n">
-        <v>7.408939649178085e-08</v>
+        <v>0</v>
       </c>
       <c r="D379" t="inlineStr">
         <is>
@@ -8461,7 +8461,7 @@
         </is>
       </c>
       <c r="C383" t="n">
-        <v>0</v>
+        <v>2.0603646e-11</v>
       </c>
       <c r="D383" t="inlineStr">
         <is>
@@ -8608,7 +8608,7 @@
         </is>
       </c>
       <c r="C390" t="n">
-        <v>9.168719945223369e-06</v>
+        <v>9.16871994522332e-06</v>
       </c>
       <c r="D390" t="inlineStr">
         <is>
@@ -8713,7 +8713,7 @@
         </is>
       </c>
       <c r="C395" t="n">
-        <v>7.672902048206029e-06</v>
+        <v>7.672902048205131e-06</v>
       </c>
       <c r="D395" t="inlineStr">
         <is>
@@ -8776,7 +8776,7 @@
         </is>
       </c>
       <c r="C398" t="n">
-        <v>1.399152629986029e-05</v>
+        <v>1.981115369914649e-05</v>
       </c>
       <c r="D398" t="inlineStr">
         <is>
@@ -8797,7 +8797,7 @@
         </is>
       </c>
       <c r="C399" t="n">
-        <v>1.399152629986029e-05</v>
+        <v>1.981115369914649e-05</v>
       </c>
       <c r="D399" t="inlineStr">
         <is>
@@ -8923,7 +8923,7 @@
         </is>
       </c>
       <c r="C405" t="n">
-        <v>0</v>
+        <v>2.628186359133498e-06</v>
       </c>
       <c r="D405" t="inlineStr">
         <is>
@@ -8944,7 +8944,7 @@
         </is>
       </c>
       <c r="C406" t="n">
-        <v>0</v>
+        <v>2.628186359133498e-06</v>
       </c>
       <c r="D406" t="inlineStr">
         <is>
@@ -8965,7 +8965,7 @@
         </is>
       </c>
       <c r="C407" t="n">
-        <v>1.412469141054455e-06</v>
+        <v>1.412469141054436e-06</v>
       </c>
       <c r="D407" t="inlineStr">
         <is>
@@ -9154,7 +9154,7 @@
         </is>
       </c>
       <c r="C416" t="n">
-        <v>3.142248853934328e-05</v>
+        <v>3.142248853934285e-05</v>
       </c>
       <c r="D416" t="inlineStr">
         <is>
@@ -9175,7 +9175,7 @@
         </is>
       </c>
       <c r="C417" t="n">
-        <v>6.952112981111937e-08</v>
+        <v>0</v>
       </c>
       <c r="D417" t="inlineStr">
         <is>
@@ -9322,7 +9322,7 @@
         </is>
       </c>
       <c r="C424" t="n">
-        <v>1.054576669368036e-05</v>
+        <v>1.371980198078469e-05</v>
       </c>
       <c r="D424" t="inlineStr">
         <is>
@@ -9406,7 +9406,7 @@
         </is>
       </c>
       <c r="C428" t="n">
-        <v>6.430857242503712e-06</v>
+        <v>3.652571499994113e-06</v>
       </c>
       <c r="D428" t="inlineStr">
         <is>
@@ -9490,7 +9490,7 @@
         </is>
       </c>
       <c r="C432" t="n">
-        <v>2.48996199183861e-06</v>
+        <v>2.478894347194044e-06</v>
       </c>
       <c r="D432" t="inlineStr">
         <is>
@@ -9805,7 +9805,7 @@
         </is>
       </c>
       <c r="C447" t="n">
-        <v>3.044358673364254e-07</v>
+        <v>3.044358673364213e-07</v>
       </c>
       <c r="D447" t="inlineStr">
         <is>
@@ -9952,7 +9952,7 @@
         </is>
       </c>
       <c r="C454" t="n">
-        <v>1.945389246930087e-06</v>
+        <v>1.945389246930061e-06</v>
       </c>
       <c r="D454" t="inlineStr">
         <is>
@@ -9994,7 +9994,7 @@
         </is>
       </c>
       <c r="C456" t="n">
-        <v>0.0001526247714053364</v>
+        <v>0.0002121548791333145</v>
       </c>
       <c r="D456" t="inlineStr">
         <is>
@@ -10120,7 +10120,7 @@
         </is>
       </c>
       <c r="C462" t="n">
-        <v>2.879673293259079e-07</v>
+        <v>2.879673293259039e-07</v>
       </c>
       <c r="D462" t="inlineStr">
         <is>
@@ -10141,7 +10141,7 @@
         </is>
       </c>
       <c r="C463" t="n">
-        <v>3.367245842451165e-05</v>
+        <v>3.367245842451119e-05</v>
       </c>
       <c r="D463" t="inlineStr">
         <is>
@@ -10183,7 +10183,7 @@
         </is>
       </c>
       <c r="C465" t="n">
-        <v>1.720547641326461e-05</v>
+        <v>1.720221609381652e-05</v>
       </c>
       <c r="D465" t="inlineStr">
         <is>
@@ -10246,7 +10246,7 @@
         </is>
       </c>
       <c r="C468" t="n">
-        <v>0</v>
+        <v>4.029957332166225e-07</v>
       </c>
       <c r="D468" t="inlineStr">
         <is>
@@ -10372,7 +10372,7 @@
         </is>
       </c>
       <c r="C474" t="n">
-        <v>6.278904861846264e-07</v>
+        <v>6.278904861846266e-07</v>
       </c>
       <c r="D474" t="inlineStr">
         <is>
@@ -10393,7 +10393,7 @@
         </is>
       </c>
       <c r="C475" t="n">
-        <v>1.064699579998028e-08</v>
+        <v>1.064699579996443e-08</v>
       </c>
       <c r="D475" t="inlineStr">
         <is>
@@ -10414,7 +10414,7 @@
         </is>
       </c>
       <c r="C476" t="n">
-        <v>6.528428532515527e-07</v>
+        <v>6.528428532505806e-07</v>
       </c>
       <c r="D476" t="inlineStr">
         <is>
@@ -10435,7 +10435,7 @@
         </is>
       </c>
       <c r="C477" t="n">
-        <v>6.926304839987173e-09</v>
+        <v>6.926304839976859e-09</v>
       </c>
       <c r="D477" t="inlineStr">
         <is>
@@ -10540,7 +10540,7 @@
         </is>
       </c>
       <c r="C482" t="n">
-        <v>3.908024410665979e-06</v>
+        <v>3.908024410665359e-06</v>
       </c>
       <c r="D482" t="inlineStr">
         <is>
@@ -10582,7 +10582,7 @@
         </is>
       </c>
       <c r="C484" t="n">
-        <v>5.612518125604157e-05</v>
+        <v>5.61251812560413e-05</v>
       </c>
       <c r="D484" t="inlineStr">
         <is>
@@ -10624,7 +10624,7 @@
         </is>
       </c>
       <c r="C486" t="n">
-        <v>6.765495931618091e-05</v>
+        <v>5.742044555190212e-05</v>
       </c>
       <c r="D486" t="inlineStr">
         <is>
@@ -10729,7 +10729,7 @@
         </is>
       </c>
       <c r="C491" t="n">
-        <v>1.583728620940058e-05</v>
+        <v>1.582567089894737e-05</v>
       </c>
       <c r="D491" t="inlineStr">
         <is>
@@ -10771,7 +10771,7 @@
         </is>
       </c>
       <c r="C493" t="n">
-        <v>2.325411106662185e-05</v>
+        <v>1.994961523198783e-05</v>
       </c>
       <c r="D493" t="inlineStr">
         <is>
@@ -10855,7 +10855,7 @@
         </is>
       </c>
       <c r="C497" t="n">
-        <v>1.416511867983208e-07</v>
+        <v>1.416511867981099e-07</v>
       </c>
       <c r="D497" t="inlineStr">
         <is>
@@ -10876,7 +10876,7 @@
         </is>
       </c>
       <c r="C498" t="n">
-        <v>1.175453999997823e-09</v>
+        <v>1.175453999996073e-09</v>
       </c>
       <c r="D498" t="inlineStr">
         <is>
@@ -10960,7 +10960,7 @@
         </is>
       </c>
       <c r="C502" t="n">
-        <v>5.875392974475436e-07</v>
+        <v>5.875392974474503e-07</v>
       </c>
       <c r="D502" t="inlineStr">
         <is>
@@ -10981,7 +10981,7 @@
         </is>
       </c>
       <c r="C503" t="n">
-        <v>9.653352267075309e-06</v>
+        <v>9.653352267073776e-06</v>
       </c>
       <c r="D503" t="inlineStr">
         <is>
@@ -11002,7 +11002,7 @@
         </is>
       </c>
       <c r="C504" t="n">
-        <v>1.68199656432517e-07</v>
+        <v>1.681996564325152e-07</v>
       </c>
       <c r="D504" t="inlineStr">
         <is>
@@ -11023,7 +11023,7 @@
         </is>
       </c>
       <c r="C505" t="n">
-        <v>1.059344242318952e-05</v>
+        <v>1.059344242318783e-05</v>
       </c>
       <c r="D505" t="inlineStr">
         <is>
@@ -11065,7 +11065,7 @@
         </is>
       </c>
       <c r="C507" t="n">
-        <v>3.544771323958859e-07</v>
+        <v>3.544771323958659e-07</v>
       </c>
       <c r="D507" t="inlineStr">
         <is>
@@ -11107,7 +11107,7 @@
         </is>
       </c>
       <c r="C509" t="n">
-        <v>3.544771323958859e-07</v>
+        <v>3.544771323958659e-07</v>
       </c>
       <c r="D509" t="inlineStr">
         <is>
@@ -11149,7 +11149,7 @@
         </is>
       </c>
       <c r="C511" t="n">
-        <v>3.060212838396801e-06</v>
+        <v>3.057968431009012e-06</v>
       </c>
       <c r="D511" t="inlineStr">
         <is>
@@ -11170,7 +11170,7 @@
         </is>
       </c>
       <c r="C512" t="n">
-        <v>1.007918074721009e-05</v>
+        <v>1.007178852028781e-05</v>
       </c>
       <c r="D512" t="inlineStr">
         <is>
@@ -11212,7 +11212,7 @@
         </is>
       </c>
       <c r="C514" t="n">
-        <v>0</v>
+        <v>3.812995199999999e-10</v>
       </c>
       <c r="D514" t="inlineStr">
         <is>
@@ -11254,7 +11254,7 @@
         </is>
       </c>
       <c r="C516" t="n">
-        <v>4.046773239311109e-06</v>
+        <v>4.046773239311108e-06</v>
       </c>
       <c r="D516" t="inlineStr">
         <is>
@@ -11422,7 +11422,7 @@
         </is>
       </c>
       <c r="C524" t="n">
-        <v>2.022956396657305e-05</v>
+        <v>1.743847977761865e-05</v>
       </c>
       <c r="D524" t="inlineStr">
         <is>
@@ -11443,7 +11443,7 @@
         </is>
       </c>
       <c r="C525" t="n">
-        <v>1.662893073619594e-06</v>
+        <v>2.293131119523641e-06</v>
       </c>
       <c r="D525" t="inlineStr">
         <is>
@@ -11464,7 +11464,7 @@
         </is>
       </c>
       <c r="C526" t="n">
-        <v>1.662893073619594e-06</v>
+        <v>2.293131119523641e-06</v>
       </c>
       <c r="D526" t="inlineStr">
         <is>
@@ -11485,7 +11485,7 @@
         </is>
       </c>
       <c r="C527" t="n">
-        <v>1.662893073619594e-06</v>
+        <v>2.293131119523641e-06</v>
       </c>
       <c r="D527" t="inlineStr">
         <is>
@@ -11506,7 +11506,7 @@
         </is>
       </c>
       <c r="C528" t="n">
-        <v>1.662893073619594e-06</v>
+        <v>2.293131119523641e-06</v>
       </c>
       <c r="D528" t="inlineStr">
         <is>
@@ -11548,7 +11548,7 @@
         </is>
       </c>
       <c r="C530" t="n">
-        <v>7.823076358556982e-05</v>
+        <v>6.682233382375788e-05</v>
       </c>
       <c r="D530" t="inlineStr">
         <is>
@@ -11716,7 +11716,7 @@
         </is>
       </c>
       <c r="C538" t="n">
-        <v>5.601355121791818e-06</v>
+        <v>5.600506958785072e-06</v>
       </c>
       <c r="D538" t="inlineStr">
         <is>
@@ -11758,7 +11758,7 @@
         </is>
       </c>
       <c r="C540" t="n">
-        <v>6.073328807716416e-07</v>
+        <v>6.071787608848265e-07</v>
       </c>
       <c r="D540" t="inlineStr">
         <is>
@@ -11863,7 +11863,7 @@
         </is>
       </c>
       <c r="C545" t="n">
-        <v>1.482845398789235e-07</v>
+        <v>0</v>
       </c>
       <c r="D545" t="inlineStr">
         <is>
@@ -11884,7 +11884,7 @@
         </is>
       </c>
       <c r="C546" t="n">
-        <v>1.482845398789235e-07</v>
+        <v>0</v>
       </c>
       <c r="D546" t="inlineStr">
         <is>
@@ -12073,7 +12073,7 @@
         </is>
       </c>
       <c r="C555" t="n">
-        <v>1.071554399998016e-10</v>
+        <v>1.07155439999642e-10</v>
       </c>
       <c r="D555" t="inlineStr">
         <is>
@@ -12199,7 +12199,7 @@
         </is>
       </c>
       <c r="C561" t="n">
-        <v>4.892948614608902e-07</v>
+        <v>5.199670797089505e-06</v>
       </c>
       <c r="D561" t="inlineStr">
         <is>
@@ -12220,7 +12220,7 @@
         </is>
       </c>
       <c r="C562" t="n">
-        <v>4.892948614608902e-07</v>
+        <v>5.199670797089505e-06</v>
       </c>
       <c r="D562" t="inlineStr">
         <is>
@@ -12241,7 +12241,7 @@
         </is>
       </c>
       <c r="C563" t="n">
-        <v>4.892948614608902e-07</v>
+        <v>5.199670797089505e-06</v>
       </c>
       <c r="D563" t="inlineStr">
         <is>
@@ -12325,7 +12325,7 @@
         </is>
       </c>
       <c r="C567" t="n">
-        <v>4.12125136624363e-06</v>
+        <v>4.121251366243611e-06</v>
       </c>
       <c r="D567" t="inlineStr">
         <is>
@@ -12346,7 +12346,7 @@
         </is>
       </c>
       <c r="C568" t="n">
-        <v>1.007237251090187e-06</v>
+        <v>1.007237251090182e-06</v>
       </c>
       <c r="D568" t="inlineStr">
         <is>
@@ -12367,7 +12367,7 @@
         </is>
       </c>
       <c r="C569" t="n">
-        <v>1.007237251090187e-06</v>
+        <v>1.007237251090182e-06</v>
       </c>
       <c r="D569" t="inlineStr">
         <is>
@@ -12451,7 +12451,7 @@
         </is>
       </c>
       <c r="C573" t="n">
-        <v>5.001529765560697e-06</v>
+        <v>5.001529765560677e-06</v>
       </c>
       <c r="D573" t="inlineStr">
         <is>
@@ -12598,7 +12598,7 @@
         </is>
       </c>
       <c r="C580" t="n">
-        <v>1.828837999151935e-05</v>
+        <v>1.539810183311682e-05</v>
       </c>
       <c r="D580" t="inlineStr">
         <is>
@@ -12619,7 +12619,7 @@
         </is>
       </c>
       <c r="C581" t="n">
-        <v>2.665518524973222e-05</v>
+        <v>2.664902839340443e-05</v>
       </c>
       <c r="D581" t="inlineStr">
         <is>
@@ -12661,7 +12661,7 @@
         </is>
       </c>
       <c r="C583" t="n">
-        <v>3.490816307458154e-06</v>
+        <v>3.009650337883544e-06</v>
       </c>
       <c r="D583" t="inlineStr">
         <is>
@@ -12682,7 +12682,7 @@
         </is>
       </c>
       <c r="C584" t="n">
-        <v>9.51507659664782e-06</v>
+        <v>9.515076596647718e-06</v>
       </c>
       <c r="D584" t="inlineStr">
         <is>
@@ -12955,7 +12955,7 @@
         </is>
       </c>
       <c r="C597" t="n">
-        <v>0</v>
+        <v>1.640923742711345e-10</v>
       </c>
       <c r="D597" t="inlineStr">
         <is>
@@ -13144,7 +13144,7 @@
         </is>
       </c>
       <c r="C606" t="n">
-        <v>0</v>
+        <v>1.541822813504235e-05</v>
       </c>
       <c r="D606" t="inlineStr">
         <is>
@@ -13354,7 +13354,7 @@
         </is>
       </c>
       <c r="C616" t="n">
-        <v>2.980406935491898e-07</v>
+        <v>2.980406935491899e-07</v>
       </c>
       <c r="D616" t="inlineStr">
         <is>
@@ -13396,7 +13396,7 @@
         </is>
       </c>
       <c r="C618" t="n">
-        <v>6.479099831243786e-09</v>
+        <v>3.330403817508616e-09</v>
       </c>
       <c r="D618" t="inlineStr">
         <is>
@@ -13459,7 +13459,7 @@
         </is>
       </c>
       <c r="C621" t="n">
-        <v>1.651996446181178e-07</v>
+        <v>1.644641527588539e-07</v>
       </c>
       <c r="D621" t="inlineStr">
         <is>
@@ -13522,7 +13522,7 @@
         </is>
       </c>
       <c r="C624" t="n">
-        <v>1.009829731392414e-06</v>
+        <v>2.460137982377643e-06</v>
       </c>
       <c r="D624" t="inlineStr">
         <is>
@@ -13543,7 +13543,7 @@
         </is>
       </c>
       <c r="C625" t="n">
-        <v>1.050154490315313e-06</v>
+        <v>4.948280078568954e-07</v>
       </c>
       <c r="D625" t="inlineStr">
         <is>
@@ -13648,7 +13648,7 @@
         </is>
       </c>
       <c r="C630" t="n">
-        <v>8.675034109564556e-08</v>
+        <v>5.431140932267016e-08</v>
       </c>
       <c r="D630" t="inlineStr">
         <is>
@@ -13669,7 +13669,7 @@
         </is>
       </c>
       <c r="C631" t="n">
-        <v>1.218672196655907e-06</v>
+        <v>1.263781464514027e-06</v>
       </c>
       <c r="D631" t="inlineStr">
         <is>
@@ -13690,7 +13690,7 @@
         </is>
       </c>
       <c r="C632" t="n">
-        <v>6.118208501905272e-07</v>
+        <v>5.039266493460497e-07</v>
       </c>
       <c r="D632" t="inlineStr">
         <is>
@@ -13711,7 +13711,7 @@
         </is>
       </c>
       <c r="C633" t="n">
-        <v>9.305987680169556e-08</v>
+        <v>9.305987680169555e-08</v>
       </c>
       <c r="D633" t="inlineStr">
         <is>
@@ -13753,7 +13753,7 @@
         </is>
       </c>
       <c r="C635" t="n">
-        <v>6.312478944201185e-07</v>
+        <v>4.271464610655406e-07</v>
       </c>
       <c r="D635" t="inlineStr">
         <is>
@@ -13774,7 +13774,7 @@
         </is>
       </c>
       <c r="C636" t="n">
-        <v>8.97059651436576e-08</v>
+        <v>2.478402023641416e-08</v>
       </c>
       <c r="D636" t="inlineStr">
         <is>
@@ -13795,7 +13795,7 @@
         </is>
       </c>
       <c r="C637" t="n">
-        <v>3.318377802769983e-06</v>
+        <v>3.82466039219886e-06</v>
       </c>
       <c r="D637" t="inlineStr">
         <is>
@@ -14068,7 +14068,7 @@
         </is>
       </c>
       <c r="C650" t="n">
-        <v>0</v>
+        <v>1.297639553658393e-07</v>
       </c>
       <c r="D650" t="inlineStr">
         <is>
@@ -14824,7 +14824,7 @@
         </is>
       </c>
       <c r="C686" t="n">
-        <v>1.382913232035101e-05</v>
+        <v>1.644774295975035e-05</v>
       </c>
       <c r="D686" t="inlineStr">
         <is>
@@ -14887,7 +14887,7 @@
         </is>
       </c>
       <c r="C689" t="n">
-        <v>1.20142523386676e-05</v>
+        <v>1.765070476483449e-05</v>
       </c>
       <c r="D689" t="inlineStr">
         <is>
@@ -14992,7 +14992,7 @@
         </is>
       </c>
       <c r="C694" t="n">
-        <v>3.974652039655661e-06</v>
+        <v>3.974430794374923e-06</v>
       </c>
       <c r="D694" t="inlineStr">
         <is>
@@ -15034,7 +15034,7 @@
         </is>
       </c>
       <c r="C696" t="n">
-        <v>6.730817351892377e-05</v>
+        <v>8.032178185554971e-05</v>
       </c>
       <c r="D696" t="inlineStr">
         <is>
@@ -15265,7 +15265,7 @@
         </is>
       </c>
       <c r="C707" t="n">
-        <v>6.89756799816749e-05</v>
+        <v>5.973364257786793e-05</v>
       </c>
       <c r="D707" t="inlineStr">
         <is>
@@ -15412,7 +15412,7 @@
         </is>
       </c>
       <c r="C714" t="n">
-        <v>8.529813552245564e-06</v>
+        <v>8.464855054655783e-06</v>
       </c>
       <c r="D714" t="inlineStr">
         <is>
@@ -15643,7 +15643,7 @@
         </is>
       </c>
       <c r="C725" t="n">
-        <v>8.056258441125429e-09</v>
+        <v>5.212744102523668e-09</v>
       </c>
       <c r="D725" t="inlineStr">
         <is>
@@ -15832,7 +15832,7 @@
         </is>
       </c>
       <c r="C734" t="n">
-        <v>6.963030735643235e-06</v>
+        <v>4.921512027174274e-08</v>
       </c>
       <c r="D734" t="inlineStr">
         <is>
@@ -15979,7 +15979,7 @@
         </is>
       </c>
       <c r="C741" t="n">
-        <v>0.0001846348662768155</v>
+        <v>0.0002645283349716769</v>
       </c>
       <c r="D741" t="inlineStr">
         <is>
@@ -16210,7 +16210,7 @@
         </is>
       </c>
       <c r="C752" t="n">
-        <v>2.427543057984967e-06</v>
+        <v>2.427543057984958e-06</v>
       </c>
       <c r="D752" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix: small update in code
</commit_message>
<xml_diff>
--- a/data/data_check.xlsx
+++ b/data/data_check.xlsx
@@ -481,7 +481,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>3.85870276190423e-05</v>
+        <v>3.858687999205868e-05</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -670,7 +670,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1.988557273623059e-07</v>
+        <v>1.988561485757594e-07</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>4.734219204423844e-06</v>
+        <v>4.734220341415089e-06</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -733,7 +733,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>2.752653119998463e-09</v>
+        <v>2.752651779357709e-09</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>2.752653119998463e-09</v>
+        <v>2.752651779357709e-09</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -775,7 +775,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>3.8905692e-08</v>
+        <v>3.890571073000501e-08</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -796,7 +796,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>4.053012599999999e-08</v>
+        <v>4.053011956303154e-08</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -817,7 +817,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>1.942872176729351e-06</v>
+        <v>1.942873181823992e-06</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -838,7 +838,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>3.885749768074303e-06</v>
+        <v>3.885746363647978e-06</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -859,7 +859,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>5.982297078224262e-08</v>
+        <v>5.982297318432829e-08</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -880,7 +880,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>9.853862004506921e-07</v>
+        <v>9.853859459389698e-07</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -901,7 +901,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>6.205356391217196e-06</v>
+        <v>6.205354246823452e-06</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -943,7 +943,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1.247665019999303e-09</v>
+        <v>1.247665817688355e-09</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -964,7 +964,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>6.062354394289486e-06</v>
+        <v>6.062352125347012e-06</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -1111,7 +1111,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>1.683584649599671e-05</v>
+        <v>1.683585472555498e-05</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -1132,7 +1132,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>3.516151473163842e-06</v>
+        <v>3.516145943180273e-06</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -1195,7 +1195,7 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2.892460908906534e-05</v>
+        <v>2.892460785081759e-05</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -1216,7 +1216,7 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>1.221345214330619e-05</v>
+        <v>1.22134586052908e-05</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -1237,7 +1237,7 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>1.116465328222518e-05</v>
+        <v>1.116465840616862e-05</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -1258,7 +1258,7 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>8.184989591592607e-07</v>
+        <v>8.185135392279869e-07</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -1321,7 +1321,7 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>2.214797855879776e-07</v>
+        <v>2.214797791871889e-07</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -1342,7 +1342,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>1.673044278148205e-05</v>
+        <v>1.673045007884725e-05</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -1384,7 +1384,7 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>6.330953999999999e-13</v>
+        <v>6.330945687873247e-13</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -1405,7 +1405,7 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>6.330953999999999e-13</v>
+        <v>6.330945687873247e-13</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -1426,7 +1426,7 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>4.943958551471196e-06</v>
+        <v>4.943958562762306e-06</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -1468,7 +1468,7 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>2.796073369360351e-07</v>
+        <v>2.79607329424925e-07</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -1510,7 +1510,7 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>7.900648262780398e-06</v>
+        <v>7.900648702644096e-06</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
@@ -1573,7 +1573,7 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>6.935824979996126e-08</v>
+        <v>6.935825956887501e-08</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
@@ -1615,7 +1615,7 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>2.916005652000083e-09</v>
+        <v>2.91600569335436e-09</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
@@ -1636,7 +1636,7 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>6.613463220000188e-10</v>
+        <v>6.61345883579656e-10</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -1657,7 +1657,7 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>0</v>
+        <v>3.12154524394814e-11</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -1678,7 +1678,7 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>6.611950580972941e-07</v>
+        <v>6.611948667903273e-07</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -1762,7 +1762,7 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>1.124529531912196e-08</v>
+        <v>1.124529568097847e-08</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
@@ -1825,7 +1825,7 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>2.500714733123582e-06</v>
+        <v>2.500731175390241e-06</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -1846,7 +1846,7 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>3.157728388273484e-07</v>
+        <v>3.157725618112419e-07</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
@@ -1888,7 +1888,7 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>5.776257884475657e-10</v>
+        <v>5.776257869892009e-10</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
@@ -1930,7 +1930,7 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>1.371596546394728e-06</v>
+        <v>1.371598053136376e-06</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
@@ -1951,7 +1951,7 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>5.821585559996749e-11</v>
+        <v>5.821585000119521e-11</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -1972,7 +1972,7 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>2.077888259998839e-09</v>
+        <v>2.077891873225852e-09</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
@@ -2014,7 +2014,7 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>8.937537328406102e-06</v>
+        <v>8.937537823581297e-06</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -2056,7 +2056,7 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>3.504715355317638e-05</v>
+        <v>3.504716000635247e-05</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
@@ -2098,7 +2098,7 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>4.467891904705558e-06</v>
+        <v>4.467888002003802e-06</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
@@ -2140,7 +2140,7 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>2.335084563745803e-05</v>
+        <v>2.335085058936934e-05</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
@@ -2161,7 +2161,7 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>1.62505245105974e-05</v>
+        <v>1.625054368623895e-05</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
@@ -2224,7 +2224,7 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>5.223997244649175e-06</v>
+        <v>5.223998422841062e-06</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
@@ -2266,7 +2266,7 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>3.14514615257323e-06</v>
+        <v>3.145147303525755e-06</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
@@ -2287,7 +2287,7 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>3.554149118667769e-07</v>
+        <v>3.554148110126372e-07</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
@@ -2350,7 +2350,7 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>3.619903559997978e-10</v>
+        <v>3.619905767801528e-10</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
@@ -2392,7 +2392,7 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>9.051392149085006e-06</v>
+        <v>9.051392159945317e-06</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
@@ -2434,7 +2434,7 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>1.088777967615844e-05</v>
+        <v>1.088777828673697e-05</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
@@ -2455,7 +2455,7 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>1.928925599998923e-09</v>
+        <v>1.928926411426127e-09</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
@@ -2497,7 +2497,7 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>0.0001696874844344081</v>
+        <v>0.0001696875729017192</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
@@ -2560,7 +2560,7 @@
         </is>
       </c>
       <c r="C102" t="n">
-        <v>3.56477688397569e-06</v>
+        <v>3.564770206342125e-06</v>
       </c>
       <c r="D102" t="inlineStr">
         <is>
@@ -2581,7 +2581,7 @@
         </is>
       </c>
       <c r="C103" t="n">
-        <v>5.051445635982511e-06</v>
+        <v>5.051443387797158e-06</v>
       </c>
       <c r="D103" t="inlineStr">
         <is>
@@ -2602,7 +2602,7 @@
         </is>
       </c>
       <c r="C104" t="n">
-        <v>1.404955003455644e-06</v>
+        <v>1.404981024708968e-06</v>
       </c>
       <c r="D104" t="inlineStr">
         <is>
@@ -2665,7 +2665,7 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>1.938410745217332e-05</v>
+        <v>1.938411005396029e-05</v>
       </c>
       <c r="D107" t="inlineStr">
         <is>
@@ -2833,7 +2833,7 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>1.518947536242022e-05</v>
+        <v>1.518952442121605e-05</v>
       </c>
       <c r="D115" t="inlineStr">
         <is>
@@ -2875,7 +2875,7 @@
         </is>
       </c>
       <c r="C117" t="n">
-        <v>1.151426219999357e-09</v>
+        <v>1.151426770677664e-09</v>
       </c>
       <c r="D117" t="inlineStr">
         <is>
@@ -2938,7 +2938,7 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>4.389623922317634e-06</v>
+        <v>4.389622612849125e-06</v>
       </c>
       <c r="D120" t="inlineStr">
         <is>
@@ -3232,7 +3232,7 @@
         </is>
       </c>
       <c r="C134" t="n">
-        <v>7.306655663744784e-07</v>
+        <v>7.306655319894739e-07</v>
       </c>
       <c r="D134" t="inlineStr">
         <is>
@@ -3253,7 +3253,7 @@
         </is>
       </c>
       <c r="C135" t="n">
-        <v>7.306655663744784e-07</v>
+        <v>7.306655319894739e-07</v>
       </c>
       <c r="D135" t="inlineStr">
         <is>
@@ -3295,7 +3295,7 @@
         </is>
       </c>
       <c r="C137" t="n">
-        <v>7.306655663744784e-07</v>
+        <v>7.306655319894739e-07</v>
       </c>
       <c r="D137" t="inlineStr">
         <is>
@@ -3379,7 +3379,7 @@
         </is>
       </c>
       <c r="C141" t="n">
-        <v>9.384927839054747e-06</v>
+        <v>9.38492785580574e-06</v>
       </c>
       <c r="D141" t="inlineStr">
         <is>
@@ -3400,7 +3400,7 @@
         </is>
       </c>
       <c r="C142" t="n">
-        <v>1.747441095083977e-06</v>
+        <v>1.747444202710669e-06</v>
       </c>
       <c r="D142" t="inlineStr">
         <is>
@@ -3421,7 +3421,7 @@
         </is>
       </c>
       <c r="C143" t="n">
-        <v>4.393683013560872e-06</v>
+        <v>4.39368314379435e-06</v>
       </c>
       <c r="D143" t="inlineStr">
         <is>
@@ -3484,7 +3484,7 @@
         </is>
       </c>
       <c r="C146" t="n">
-        <v>1.61072883345649e-06</v>
+        <v>1.610727032056713e-06</v>
       </c>
       <c r="D146" t="inlineStr">
         <is>
@@ -3505,7 +3505,7 @@
         </is>
       </c>
       <c r="C147" t="n">
-        <v>1.082804800392285e-06</v>
+        <v>1.082806301415691e-06</v>
       </c>
       <c r="D147" t="inlineStr">
         <is>
@@ -3526,7 +3526,7 @@
         </is>
       </c>
       <c r="C148" t="n">
-        <v>2.619423935019792e-06</v>
+        <v>2.619421745203339e-06</v>
       </c>
       <c r="D148" t="inlineStr">
         <is>
@@ -3610,7 +3610,7 @@
         </is>
       </c>
       <c r="C152" t="n">
-        <v>2.520979940585519e-06</v>
+        <v>2.520982311927279e-06</v>
       </c>
       <c r="D152" t="inlineStr">
         <is>
@@ -3631,7 +3631,7 @@
         </is>
       </c>
       <c r="C153" t="n">
-        <v>2.29254737547871e-06</v>
+        <v>2.292540790058935e-06</v>
       </c>
       <c r="D153" t="inlineStr">
         <is>
@@ -3652,7 +3652,7 @@
         </is>
       </c>
       <c r="C154" t="n">
-        <v>3.983907490299623e-07</v>
+        <v>3.983923529523328e-07</v>
       </c>
       <c r="D154" t="inlineStr">
         <is>
@@ -3673,7 +3673,7 @@
         </is>
       </c>
       <c r="C155" t="n">
-        <v>5.668357702410254e-06</v>
+        <v>5.668345323917242e-06</v>
       </c>
       <c r="D155" t="inlineStr">
         <is>
@@ -3694,7 +3694,7 @@
         </is>
       </c>
       <c r="C156" t="n">
-        <v>4.293240658234228e-05</v>
+        <v>4.293237776561915e-05</v>
       </c>
       <c r="D156" t="inlineStr">
         <is>
@@ -3715,7 +3715,7 @@
         </is>
       </c>
       <c r="C157" t="n">
-        <v>3.18686669702266e-06</v>
+        <v>3.186876134421072e-06</v>
       </c>
       <c r="D157" t="inlineStr">
         <is>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C158" t="n">
-        <v>7.454205833464618e-08</v>
+        <v>7.454208275282819e-08</v>
       </c>
       <c r="D158" t="inlineStr">
         <is>
@@ -3820,7 +3820,7 @@
         </is>
       </c>
       <c r="C162" t="n">
-        <v>3.797553162108554e-06</v>
+        <v>3.797533986940885e-06</v>
       </c>
       <c r="D162" t="inlineStr">
         <is>
@@ -3841,7 +3841,7 @@
         </is>
       </c>
       <c r="C163" t="n">
-        <v>1.265847245831474e-06</v>
+        <v>1.265844662313624e-06</v>
       </c>
       <c r="D163" t="inlineStr">
         <is>
@@ -3862,7 +3862,7 @@
         </is>
       </c>
       <c r="C164" t="n">
-        <v>1.265847245831474e-06</v>
+        <v>1.265844662313624e-06</v>
       </c>
       <c r="D164" t="inlineStr">
         <is>
@@ -3883,7 +3883,7 @@
         </is>
       </c>
       <c r="C165" t="n">
-        <v>2.531694491662948e-06</v>
+        <v>2.531689324627261e-06</v>
       </c>
       <c r="D165" t="inlineStr">
         <is>
@@ -3925,7 +3925,7 @@
         </is>
       </c>
       <c r="C167" t="n">
-        <v>2.531694491662948e-06</v>
+        <v>2.531689324627261e-06</v>
       </c>
       <c r="D167" t="inlineStr">
         <is>
@@ -3946,7 +3946,7 @@
         </is>
       </c>
       <c r="C168" t="n">
-        <v>3.797553162108554e-06</v>
+        <v>3.797533986940885e-06</v>
       </c>
       <c r="D168" t="inlineStr">
         <is>
@@ -3967,7 +3967,7 @@
         </is>
       </c>
       <c r="C169" t="n">
-        <v>2.531694491662948e-06</v>
+        <v>2.531689324627261e-06</v>
       </c>
       <c r="D169" t="inlineStr">
         <is>
@@ -3988,7 +3988,7 @@
         </is>
       </c>
       <c r="C170" t="n">
-        <v>1.265847245831474e-06</v>
+        <v>1.265844662313624e-06</v>
       </c>
       <c r="D170" t="inlineStr">
         <is>
@@ -4009,7 +4009,7 @@
         </is>
       </c>
       <c r="C171" t="n">
-        <v>2.531694491662948e-06</v>
+        <v>2.531689324627261e-06</v>
       </c>
       <c r="D171" t="inlineStr">
         <is>
@@ -4030,7 +4030,7 @@
         </is>
       </c>
       <c r="C172" t="n">
-        <v>2.531694491662948e-06</v>
+        <v>2.531689324627261e-06</v>
       </c>
       <c r="D172" t="inlineStr">
         <is>
@@ -4051,7 +4051,7 @@
         </is>
       </c>
       <c r="C173" t="n">
-        <v>1.265847245831474e-06</v>
+        <v>1.265844662313624e-06</v>
       </c>
       <c r="D173" t="inlineStr">
         <is>
@@ -4072,7 +4072,7 @@
         </is>
       </c>
       <c r="C174" t="n">
-        <v>1.265847245831474e-06</v>
+        <v>1.265844662313624e-06</v>
       </c>
       <c r="D174" t="inlineStr">
         <is>
@@ -4261,7 +4261,7 @@
         </is>
       </c>
       <c r="C183" t="n">
-        <v>2.337541243204578e-06</v>
+        <v>2.337541249385636e-06</v>
       </c>
       <c r="D183" t="inlineStr">
         <is>
@@ -4303,7 +4303,7 @@
         </is>
       </c>
       <c r="C185" t="n">
-        <v>2.795680185212714e-06</v>
+        <v>2.795679429655632e-06</v>
       </c>
       <c r="D185" t="inlineStr">
         <is>
@@ -4324,7 +4324,7 @@
         </is>
       </c>
       <c r="C186" t="n">
-        <v>2.272442872905617e-06</v>
+        <v>2.272442255889529e-06</v>
       </c>
       <c r="D186" t="inlineStr">
         <is>
@@ -4345,7 +4345,7 @@
         </is>
       </c>
       <c r="C187" t="n">
-        <v>3.785413000886372e-06</v>
+        <v>3.785412226947694e-06</v>
       </c>
       <c r="D187" t="inlineStr">
         <is>
@@ -4408,7 +4408,7 @@
         </is>
       </c>
       <c r="C190" t="n">
-        <v>1.326800969007848e-07</v>
+        <v>1.326800358059687e-07</v>
       </c>
       <c r="D190" t="inlineStr">
         <is>
@@ -4471,7 +4471,7 @@
         </is>
       </c>
       <c r="C193" t="n">
-        <v>1.370435718790287e-06</v>
+        <v>1.370430605954213e-06</v>
       </c>
       <c r="D193" t="inlineStr">
         <is>
@@ -4492,7 +4492,7 @@
         </is>
       </c>
       <c r="C194" t="n">
-        <v>1.370435718790287e-06</v>
+        <v>1.370430605954213e-06</v>
       </c>
       <c r="D194" t="inlineStr">
         <is>
@@ -4744,7 +4744,7 @@
         </is>
       </c>
       <c r="C206" t="n">
-        <v>6.936673102338296e-08</v>
+        <v>6.936677396866923e-08</v>
       </c>
       <c r="D206" t="inlineStr">
         <is>
@@ -4765,7 +4765,7 @@
         </is>
       </c>
       <c r="C207" t="n">
-        <v>3.088147873660054e-05</v>
+        <v>3.088147875636776e-05</v>
       </c>
       <c r="D207" t="inlineStr">
         <is>
@@ -4786,7 +4786,7 @@
         </is>
       </c>
       <c r="C208" t="n">
-        <v>4.937565779585677e-07</v>
+        <v>4.937534361500296e-07</v>
       </c>
       <c r="D208" t="inlineStr">
         <is>
@@ -4870,7 +4870,7 @@
         </is>
       </c>
       <c r="C212" t="n">
-        <v>1.6481346e-11</v>
+        <v>1.648135282722718e-11</v>
       </c>
       <c r="D212" t="inlineStr">
         <is>
@@ -4912,7 +4912,7 @@
         </is>
       </c>
       <c r="C214" t="n">
-        <v>1.663221200699061e-07</v>
+        <v>1.66322155849924e-07</v>
       </c>
       <c r="D214" t="inlineStr">
         <is>
@@ -4954,7 +4954,7 @@
         </is>
       </c>
       <c r="C216" t="n">
-        <v>2.234009294435597e-07</v>
+        <v>2.234355210740703e-07</v>
       </c>
       <c r="D216" t="inlineStr">
         <is>
@@ -5017,7 +5017,7 @@
         </is>
       </c>
       <c r="C219" t="n">
-        <v>1.480056394777043e-06</v>
+        <v>1.480056385549299e-06</v>
       </c>
       <c r="D219" t="inlineStr">
         <is>
@@ -5038,7 +5038,7 @@
         </is>
       </c>
       <c r="C220" t="n">
-        <v>1.446565748356897e-07</v>
+        <v>1.446565658338069e-07</v>
       </c>
       <c r="D220" t="inlineStr">
         <is>
@@ -5059,7 +5059,7 @@
         </is>
       </c>
       <c r="C221" t="n">
-        <v>2.97393768e-09</v>
+        <v>2.973937300261885e-09</v>
       </c>
       <c r="D221" t="inlineStr">
         <is>
@@ -5101,7 +5101,7 @@
         </is>
       </c>
       <c r="C223" t="n">
-        <v>1.95527096520164e-07</v>
+        <v>1.95526597686617e-07</v>
       </c>
       <c r="D223" t="inlineStr">
         <is>
@@ -5122,7 +5122,7 @@
         </is>
       </c>
       <c r="C224" t="n">
-        <v>1.95527096520164e-07</v>
+        <v>1.95526597686617e-07</v>
       </c>
       <c r="D224" t="inlineStr">
         <is>
@@ -5227,7 +5227,7 @@
         </is>
       </c>
       <c r="C229" t="n">
-        <v>0.0002086795658653689</v>
+        <v>0.0002086798371204448</v>
       </c>
       <c r="D229" t="inlineStr">
         <is>
@@ -5269,7 +5269,7 @@
         </is>
       </c>
       <c r="C231" t="n">
-        <v>7.857397788361011e-09</v>
+        <v>7.857398043154241e-09</v>
       </c>
       <c r="D231" t="inlineStr">
         <is>
@@ -5353,7 +5353,7 @@
         </is>
       </c>
       <c r="C235" t="n">
-        <v>1.266507790548001e-07</v>
+        <v>1.26650754200125e-07</v>
       </c>
       <c r="D235" t="inlineStr">
         <is>
@@ -5374,7 +5374,7 @@
         </is>
       </c>
       <c r="C236" t="n">
-        <v>8.514356256000243e-12</v>
+        <v>8.514353730554103e-12</v>
       </c>
       <c r="D236" t="inlineStr">
         <is>
@@ -5395,7 +5395,7 @@
         </is>
       </c>
       <c r="C237" t="n">
-        <v>5.014718100000143e-10</v>
+        <v>5.014722030256096e-10</v>
       </c>
       <c r="D237" t="inlineStr">
         <is>
@@ -5416,7 +5416,7 @@
         </is>
       </c>
       <c r="C238" t="n">
-        <v>2.62372965493409e-06</v>
+        <v>2.623729486590908e-06</v>
       </c>
       <c r="D238" t="inlineStr">
         <is>
@@ -5437,7 +5437,7 @@
         </is>
       </c>
       <c r="C239" t="n">
-        <v>1.944494344236873e-05</v>
+        <v>1.944493122343952e-05</v>
       </c>
       <c r="D239" t="inlineStr">
         <is>
@@ -5479,7 +5479,7 @@
         </is>
       </c>
       <c r="C241" t="n">
-        <v>5.74526003985476e-05</v>
+        <v>5.745260055046297e-05</v>
       </c>
       <c r="D241" t="inlineStr">
         <is>
@@ -5500,7 +5500,7 @@
         </is>
       </c>
       <c r="C242" t="n">
-        <v>2.11643409794392e-05</v>
+        <v>2.116439144751276e-05</v>
       </c>
       <c r="D242" t="inlineStr">
         <is>
@@ -5542,7 +5542,7 @@
         </is>
       </c>
       <c r="C244" t="n">
-        <v>4.083759489743285e-06</v>
+        <v>4.083747731110235e-06</v>
       </c>
       <c r="D244" t="inlineStr">
         <is>
@@ -5899,7 +5899,7 @@
         </is>
       </c>
       <c r="C261" t="n">
-        <v>2.388950068734915e-10</v>
+        <v>2.388950062703396e-10</v>
       </c>
       <c r="D261" t="inlineStr">
         <is>
@@ -5941,7 +5941,7 @@
         </is>
       </c>
       <c r="C263" t="n">
-        <v>3.288173852234391e-07</v>
+        <v>3.288163453343264e-07</v>
       </c>
       <c r="D263" t="inlineStr">
         <is>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C264" t="n">
-        <v>6.576347704468783e-07</v>
+        <v>6.576326906686528e-07</v>
       </c>
       <c r="D264" t="inlineStr">
         <is>
@@ -5983,7 +5983,7 @@
         </is>
       </c>
       <c r="C265" t="n">
-        <v>3.288173852234391e-07</v>
+        <v>3.288163453343264e-07</v>
       </c>
       <c r="D265" t="inlineStr">
         <is>
@@ -6004,7 +6004,7 @@
         </is>
       </c>
       <c r="C266" t="n">
-        <v>3.288173852234391e-07</v>
+        <v>3.288163453343264e-07</v>
       </c>
       <c r="D266" t="inlineStr">
         <is>
@@ -6025,7 +6025,7 @@
         </is>
       </c>
       <c r="C267" t="n">
-        <v>3.288173852234391e-07</v>
+        <v>3.288163453343264e-07</v>
       </c>
       <c r="D267" t="inlineStr">
         <is>
@@ -6046,7 +6046,7 @@
         </is>
       </c>
       <c r="C268" t="n">
-        <v>3.288173852234391e-07</v>
+        <v>3.288163453343264e-07</v>
       </c>
       <c r="D268" t="inlineStr">
         <is>
@@ -6067,7 +6067,7 @@
         </is>
       </c>
       <c r="C269" t="n">
-        <v>3.288173852234391e-07</v>
+        <v>3.288163453343264e-07</v>
       </c>
       <c r="D269" t="inlineStr">
         <is>
@@ -6088,7 +6088,7 @@
         </is>
       </c>
       <c r="C270" t="n">
-        <v>3.288173852234391e-07</v>
+        <v>3.288163453343264e-07</v>
       </c>
       <c r="D270" t="inlineStr">
         <is>
@@ -6109,7 +6109,7 @@
         </is>
       </c>
       <c r="C271" t="n">
-        <v>3.288173852234391e-07</v>
+        <v>3.288163453343264e-07</v>
       </c>
       <c r="D271" t="inlineStr">
         <is>
@@ -6214,7 +6214,7 @@
         </is>
       </c>
       <c r="C276" t="n">
-        <v>3.792939284859542e-05</v>
+        <v>3.792924730139003e-05</v>
       </c>
       <c r="D276" t="inlineStr">
         <is>
@@ -6235,7 +6235,7 @@
         </is>
       </c>
       <c r="C277" t="n">
-        <v>3.792939284859542e-05</v>
+        <v>3.792924730139003e-05</v>
       </c>
       <c r="D277" t="inlineStr">
         <is>
@@ -6256,7 +6256,7 @@
         </is>
       </c>
       <c r="C278" t="n">
-        <v>3.792939284859542e-05</v>
+        <v>3.792924730139003e-05</v>
       </c>
       <c r="D278" t="inlineStr">
         <is>
@@ -6277,7 +6277,7 @@
         </is>
       </c>
       <c r="C279" t="n">
-        <v>3.792939284859542e-05</v>
+        <v>3.792924730139003e-05</v>
       </c>
       <c r="D279" t="inlineStr">
         <is>
@@ -6298,7 +6298,7 @@
         </is>
       </c>
       <c r="C280" t="n">
-        <v>3.792939284859542e-05</v>
+        <v>3.792924730139003e-05</v>
       </c>
       <c r="D280" t="inlineStr">
         <is>
@@ -6319,7 +6319,7 @@
         </is>
       </c>
       <c r="C281" t="n">
-        <v>3.792939284859542e-05</v>
+        <v>3.792924730139003e-05</v>
       </c>
       <c r="D281" t="inlineStr">
         <is>
@@ -6340,7 +6340,7 @@
         </is>
       </c>
       <c r="C282" t="n">
-        <v>3.792939284859542e-05</v>
+        <v>3.792924730139003e-05</v>
       </c>
       <c r="D282" t="inlineStr">
         <is>
@@ -6361,7 +6361,7 @@
         </is>
       </c>
       <c r="C283" t="n">
-        <v>3.792939284859542e-05</v>
+        <v>3.792924730139003e-05</v>
       </c>
       <c r="D283" t="inlineStr">
         <is>
@@ -6382,7 +6382,7 @@
         </is>
       </c>
       <c r="C284" t="n">
-        <v>3.792939284859542e-05</v>
+        <v>3.792924730139003e-05</v>
       </c>
       <c r="D284" t="inlineStr">
         <is>
@@ -6403,7 +6403,7 @@
         </is>
       </c>
       <c r="C285" t="n">
-        <v>2.919125340126056e-09</v>
+        <v>2.919125266382746e-09</v>
       </c>
       <c r="D285" t="inlineStr">
         <is>
@@ -6445,7 +6445,7 @@
         </is>
       </c>
       <c r="C287" t="n">
-        <v>7.677334691740151e-06</v>
+        <v>7.677386672136504e-06</v>
       </c>
       <c r="D287" t="inlineStr">
         <is>
@@ -6466,7 +6466,7 @@
         </is>
       </c>
       <c r="C288" t="n">
-        <v>7.862972518555082e-09</v>
+        <v>7.852906978390975e-09</v>
       </c>
       <c r="D288" t="inlineStr">
         <is>
@@ -6529,7 +6529,7 @@
         </is>
       </c>
       <c r="C291" t="n">
-        <v>1.381831778958883e-06</v>
+        <v>1.381820561063441e-06</v>
       </c>
       <c r="D291" t="inlineStr">
         <is>
@@ -6550,7 +6550,7 @@
         </is>
       </c>
       <c r="C292" t="n">
-        <v>3.116781911675661e-07</v>
+        <v>3.116782951218094e-07</v>
       </c>
       <c r="D292" t="inlineStr">
         <is>
@@ -6655,7 +6655,7 @@
         </is>
       </c>
       <c r="C297" t="n">
-        <v>5.977821766345488e-06</v>
+        <v>5.977823322772781e-06</v>
       </c>
       <c r="D297" t="inlineStr">
         <is>
@@ -6676,7 +6676,7 @@
         </is>
       </c>
       <c r="C298" t="n">
-        <v>6.269720623061605e-05</v>
+        <v>6.269741142216417e-05</v>
       </c>
       <c r="D298" t="inlineStr">
         <is>
@@ -6697,7 +6697,7 @@
         </is>
       </c>
       <c r="C299" t="n">
-        <v>2.115026200515019e-06</v>
+        <v>2.115028559006806e-06</v>
       </c>
       <c r="D299" t="inlineStr">
         <is>
@@ -6802,7 +6802,7 @@
         </is>
       </c>
       <c r="C304" t="n">
-        <v>1.725449148951976e-06</v>
+        <v>1.725447523345389e-06</v>
       </c>
       <c r="D304" t="inlineStr">
         <is>
@@ -6823,7 +6823,7 @@
         </is>
       </c>
       <c r="C305" t="n">
-        <v>2.906026837814505e-06</v>
+        <v>2.906033327125302e-06</v>
       </c>
       <c r="D305" t="inlineStr">
         <is>
@@ -6886,7 +6886,7 @@
         </is>
       </c>
       <c r="C308" t="n">
-        <v>3.039505039292224e-06</v>
+        <v>3.039511045575845e-06</v>
       </c>
       <c r="D308" t="inlineStr">
         <is>
@@ -7180,7 +7180,7 @@
         </is>
       </c>
       <c r="C322" t="n">
-        <v>6.541725803499613e-05</v>
+        <v>6.541735562019884e-05</v>
       </c>
       <c r="D322" t="inlineStr">
         <is>
@@ -7327,7 +7327,7 @@
         </is>
       </c>
       <c r="C329" t="n">
-        <v>1.928312291417593e-08</v>
+        <v>1.928312997890255e-08</v>
       </c>
       <c r="D329" t="inlineStr">
         <is>
@@ -7369,7 +7369,7 @@
         </is>
       </c>
       <c r="C331" t="n">
-        <v>1.493406853518544e-06</v>
+        <v>1.493417539861265e-06</v>
       </c>
       <c r="D331" t="inlineStr">
         <is>
@@ -7390,7 +7390,7 @@
         </is>
       </c>
       <c r="C332" t="n">
-        <v>1.806575356308142e-09</v>
+        <v>1.804637564974597e-09</v>
       </c>
       <c r="D332" t="inlineStr">
         <is>
@@ -7411,7 +7411,7 @@
         </is>
       </c>
       <c r="C333" t="n">
-        <v>1.806575356308142e-09</v>
+        <v>1.804637564974597e-09</v>
       </c>
       <c r="D333" t="inlineStr">
         <is>
@@ -7432,7 +7432,7 @@
         </is>
       </c>
       <c r="C334" t="n">
-        <v>9.970477346886883e-06</v>
+        <v>9.970385666012544e-06</v>
       </c>
       <c r="D334" t="inlineStr">
         <is>
@@ -7453,7 +7453,7 @@
         </is>
       </c>
       <c r="C335" t="n">
-        <v>1.806575356308142e-09</v>
+        <v>1.804637564974597e-09</v>
       </c>
       <c r="D335" t="inlineStr">
         <is>
@@ -7474,7 +7474,7 @@
         </is>
       </c>
       <c r="C336" t="n">
-        <v>8.053406921384566e-06</v>
+        <v>8.053452524439171e-06</v>
       </c>
       <c r="D336" t="inlineStr">
         <is>
@@ -7495,7 +7495,7 @@
         </is>
       </c>
       <c r="C337" t="n">
-        <v>7.804274370755919e-10</v>
+        <v>7.796027918168833e-10</v>
       </c>
       <c r="D337" t="inlineStr">
         <is>
@@ -7516,7 +7516,7 @@
         </is>
       </c>
       <c r="C338" t="n">
-        <v>2.690306704433866e-06</v>
+        <v>2.690272098375816e-06</v>
       </c>
       <c r="D338" t="inlineStr">
         <is>
@@ -7537,7 +7537,7 @@
         </is>
       </c>
       <c r="C339" t="n">
-        <v>2.690306704433866e-06</v>
+        <v>2.690272098375816e-06</v>
       </c>
       <c r="D339" t="inlineStr">
         <is>
@@ -7558,7 +7558,7 @@
         </is>
       </c>
       <c r="C340" t="n">
-        <v>7.391978082366474e-06</v>
+        <v>7.391975308950212e-06</v>
       </c>
       <c r="D340" t="inlineStr">
         <is>
@@ -7579,7 +7579,7 @@
         </is>
       </c>
       <c r="C341" t="n">
-        <v>1.847986930886539e-06</v>
+        <v>1.847993827237557e-06</v>
       </c>
       <c r="D341" t="inlineStr">
         <is>
@@ -7642,7 +7642,7 @@
         </is>
       </c>
       <c r="C344" t="n">
-        <v>3.316865201561724e-06</v>
+        <v>3.316862934910667e-06</v>
       </c>
       <c r="D344" t="inlineStr">
         <is>
@@ -7663,7 +7663,7 @@
         </is>
       </c>
       <c r="C345" t="n">
-        <v>2.115568481418952e-06</v>
+        <v>2.115568480257355e-06</v>
       </c>
       <c r="D345" t="inlineStr">
         <is>
@@ -7810,7 +7810,7 @@
         </is>
       </c>
       <c r="C352" t="n">
-        <v>1.269525482630874e-07</v>
+        <v>1.269525533606426e-07</v>
       </c>
       <c r="D352" t="inlineStr">
         <is>
@@ -7831,7 +7831,7 @@
         </is>
       </c>
       <c r="C353" t="n">
-        <v>3.1273494e-09</v>
+        <v>3.12735067564937e-09</v>
       </c>
       <c r="D353" t="inlineStr">
         <is>
@@ -7894,7 +7894,7 @@
         </is>
       </c>
       <c r="C356" t="n">
-        <v>3.454495997449999e-05</v>
+        <v>3.454506800285953e-05</v>
       </c>
       <c r="D356" t="inlineStr">
         <is>
@@ -7978,7 +7978,7 @@
         </is>
       </c>
       <c r="C360" t="n">
-        <v>2.745737746368875e-06</v>
+        <v>2.745736694100143e-06</v>
       </c>
       <c r="D360" t="inlineStr">
         <is>
@@ -8020,7 +8020,7 @@
         </is>
       </c>
       <c r="C362" t="n">
-        <v>1.890405915860884e-07</v>
+        <v>1.890407360345822e-07</v>
       </c>
       <c r="D362" t="inlineStr">
         <is>
@@ -8041,7 +8041,7 @@
         </is>
       </c>
       <c r="C363" t="n">
-        <v>2.517805350023218e-07</v>
+        <v>2.517806170096031e-07</v>
       </c>
       <c r="D363" t="inlineStr">
         <is>
@@ -8083,7 +8083,7 @@
         </is>
       </c>
       <c r="C365" t="n">
-        <v>5.246451305600854e-08</v>
+        <v>5.246447953993108e-08</v>
       </c>
       <c r="D365" t="inlineStr">
         <is>
@@ -8104,7 +8104,7 @@
         </is>
       </c>
       <c r="C366" t="n">
-        <v>8.19750940135436e-05</v>
+        <v>8.197508862290608e-05</v>
       </c>
       <c r="D366" t="inlineStr">
         <is>
@@ -8188,7 +8188,7 @@
         </is>
       </c>
       <c r="C370" t="n">
-        <v>1.348890425249758e-05</v>
+        <v>1.34888997690315e-05</v>
       </c>
       <c r="D370" t="inlineStr">
         <is>
@@ -8209,7 +8209,7 @@
         </is>
       </c>
       <c r="C371" t="n">
-        <v>4.678923791647012e-07</v>
+        <v>4.678939392205732e-07</v>
       </c>
       <c r="D371" t="inlineStr">
         <is>
@@ -8230,7 +8230,7 @@
         </is>
       </c>
       <c r="C372" t="n">
-        <v>6.546675614480708e-06</v>
+        <v>6.546672027326384e-06</v>
       </c>
       <c r="D372" t="inlineStr">
         <is>
@@ -8251,7 +8251,7 @@
         </is>
       </c>
       <c r="C373" t="n">
-        <v>1.39103703016237e-06</v>
+        <v>1.391066280844674e-06</v>
       </c>
       <c r="D373" t="inlineStr">
         <is>
@@ -8272,7 +8272,7 @@
         </is>
       </c>
       <c r="C374" t="n">
-        <v>6.112671102160247e-05</v>
+        <v>6.112780848251965e-05</v>
       </c>
       <c r="D374" t="inlineStr">
         <is>
@@ -8440,7 +8440,7 @@
         </is>
       </c>
       <c r="C382" t="n">
-        <v>0</v>
+        <v>3.149916199579384e-12</v>
       </c>
       <c r="D382" t="inlineStr">
         <is>
@@ -8461,7 +8461,7 @@
         </is>
       </c>
       <c r="C383" t="n">
-        <v>2.0603646e-11</v>
+        <v>2.060364957137551e-11</v>
       </c>
       <c r="D383" t="inlineStr">
         <is>
@@ -8503,7 +8503,7 @@
         </is>
       </c>
       <c r="C385" t="n">
-        <v>5.823273632968851e-07</v>
+        <v>5.823274282110963e-07</v>
       </c>
       <c r="D385" t="inlineStr">
         <is>
@@ -8524,7 +8524,7 @@
         </is>
       </c>
       <c r="C386" t="n">
-        <v>1.561738099203095e-06</v>
+        <v>1.561736768471514e-06</v>
       </c>
       <c r="D386" t="inlineStr">
         <is>
@@ -8545,7 +8545,7 @@
         </is>
       </c>
       <c r="C387" t="n">
-        <v>0</v>
+        <v>7.107767925760749e-12</v>
       </c>
       <c r="D387" t="inlineStr">
         <is>
@@ -8566,7 +8566,7 @@
         </is>
       </c>
       <c r="C388" t="n">
-        <v>8.191076600250467e-06</v>
+        <v>8.191078197011901e-06</v>
       </c>
       <c r="D388" t="inlineStr">
         <is>
@@ -8587,7 +8587,7 @@
         </is>
       </c>
       <c r="C389" t="n">
-        <v>1.708168751260864e-06</v>
+        <v>1.708168454561987e-06</v>
       </c>
       <c r="D389" t="inlineStr">
         <is>
@@ -8608,7 +8608,7 @@
         </is>
       </c>
       <c r="C390" t="n">
-        <v>9.168719945223345e-06</v>
+        <v>9.168719940189064e-06</v>
       </c>
       <c r="D390" t="inlineStr">
         <is>
@@ -8713,7 +8713,7 @@
         </is>
       </c>
       <c r="C395" t="n">
-        <v>7.672902048204682e-06</v>
+        <v>7.672904036501626e-06</v>
       </c>
       <c r="D395" t="inlineStr">
         <is>
@@ -8776,7 +8776,7 @@
         </is>
       </c>
       <c r="C398" t="n">
-        <v>1.981115371087411e-05</v>
+        <v>1.981099649587891e-05</v>
       </c>
       <c r="D398" t="inlineStr">
         <is>
@@ -8797,7 +8797,7 @@
         </is>
       </c>
       <c r="C399" t="n">
-        <v>1.981115371087411e-05</v>
+        <v>1.981099649587891e-05</v>
       </c>
       <c r="D399" t="inlineStr">
         <is>
@@ -8860,7 +8860,7 @@
         </is>
       </c>
       <c r="C402" t="n">
-        <v>1.199561455642676e-06</v>
+        <v>1.19955892856983e-06</v>
       </c>
       <c r="D402" t="inlineStr">
         <is>
@@ -8902,7 +8902,7 @@
         </is>
       </c>
       <c r="C404" t="n">
-        <v>8.295600827569403e-06</v>
+        <v>8.295600849504516e-06</v>
       </c>
       <c r="D404" t="inlineStr">
         <is>
@@ -8923,7 +8923,7 @@
         </is>
       </c>
       <c r="C405" t="n">
-        <v>2.628186362102377e-06</v>
+        <v>2.628150004971435e-06</v>
       </c>
       <c r="D405" t="inlineStr">
         <is>
@@ -8944,7 +8944,7 @@
         </is>
       </c>
       <c r="C406" t="n">
-        <v>2.628186362102377e-06</v>
+        <v>2.628150004971435e-06</v>
       </c>
       <c r="D406" t="inlineStr">
         <is>
@@ -8965,7 +8965,7 @@
         </is>
       </c>
       <c r="C407" t="n">
-        <v>1.412469141054463e-06</v>
+        <v>1.412466751354739e-06</v>
       </c>
       <c r="D407" t="inlineStr">
         <is>
@@ -9049,7 +9049,7 @@
         </is>
       </c>
       <c r="C411" t="n">
-        <v>1.911640226357693e-06</v>
+        <v>1.91164504574945e-06</v>
       </c>
       <c r="D411" t="inlineStr">
         <is>
@@ -9091,7 +9091,7 @@
         </is>
       </c>
       <c r="C413" t="n">
-        <v>8.17198830183213e-06</v>
+        <v>8.171985612676672e-06</v>
       </c>
       <c r="D413" t="inlineStr">
         <is>
@@ -9154,7 +9154,7 @@
         </is>
       </c>
       <c r="C416" t="n">
-        <v>3.142248853934346e-05</v>
+        <v>3.142248861110676e-05</v>
       </c>
       <c r="D416" t="inlineStr">
         <is>
@@ -9196,7 +9196,7 @@
         </is>
       </c>
       <c r="C418" t="n">
-        <v>4.666443737957946e-07</v>
+        <v>4.666450801808998e-07</v>
       </c>
       <c r="D418" t="inlineStr">
         <is>
@@ -9217,7 +9217,7 @@
         </is>
       </c>
       <c r="C419" t="n">
-        <v>1.152215944432833e-06</v>
+        <v>1.152216424508941e-06</v>
       </c>
       <c r="D419" t="inlineStr">
         <is>
@@ -9280,7 +9280,7 @@
         </is>
       </c>
       <c r="C422" t="n">
-        <v>5.116605191229008e-06</v>
+        <v>5.116602962660499e-06</v>
       </c>
       <c r="D422" t="inlineStr">
         <is>
@@ -9322,7 +9322,7 @@
         </is>
       </c>
       <c r="C424" t="n">
-        <v>1.371980198319335e-05</v>
+        <v>1.371979000216175e-05</v>
       </c>
       <c r="D424" t="inlineStr">
         <is>
@@ -9406,7 +9406,7 @@
         </is>
       </c>
       <c r="C428" t="n">
-        <v>3.652571499994113e-06</v>
+        <v>3.652576715068682e-06</v>
       </c>
       <c r="D428" t="inlineStr">
         <is>
@@ -9448,7 +9448,7 @@
         </is>
       </c>
       <c r="C430" t="n">
-        <v>4.639593417046644e-07</v>
+        <v>4.639584590816327e-07</v>
       </c>
       <c r="D430" t="inlineStr">
         <is>
@@ -9469,7 +9469,7 @@
         </is>
       </c>
       <c r="C431" t="n">
-        <v>1.397569239003009e-05</v>
+        <v>1.397568202494603e-05</v>
       </c>
       <c r="D431" t="inlineStr">
         <is>
@@ -9490,7 +9490,7 @@
         </is>
       </c>
       <c r="C432" t="n">
-        <v>2.478894347194054e-06</v>
+        <v>2.478894565009502e-06</v>
       </c>
       <c r="D432" t="inlineStr">
         <is>
@@ -9595,7 +9595,7 @@
         </is>
       </c>
       <c r="C437" t="n">
-        <v>1.412804651750662e-06</v>
+        <v>1.412808256686351e-06</v>
       </c>
       <c r="D437" t="inlineStr">
         <is>
@@ -9616,7 +9616,7 @@
         </is>
       </c>
       <c r="C438" t="n">
-        <v>8.47561642600681e-05</v>
+        <v>8.475616448417918e-05</v>
       </c>
       <c r="D438" t="inlineStr">
         <is>
@@ -9700,7 +9700,7 @@
         </is>
       </c>
       <c r="C442" t="n">
-        <v>3.864980743307508e-08</v>
+        <v>3.864984418711379e-08</v>
       </c>
       <c r="D442" t="inlineStr">
         <is>
@@ -9721,7 +9721,7 @@
         </is>
       </c>
       <c r="C443" t="n">
-        <v>3.811420534189395e-08</v>
+        <v>3.811419451560395e-08</v>
       </c>
       <c r="D443" t="inlineStr">
         <is>
@@ -9784,7 +9784,7 @@
         </is>
       </c>
       <c r="C446" t="n">
-        <v>1.422830239375601e-07</v>
+        <v>1.422826683881053e-07</v>
       </c>
       <c r="D446" t="inlineStr">
         <is>
@@ -9805,7 +9805,7 @@
         </is>
       </c>
       <c r="C447" t="n">
-        <v>3.044358673364272e-07</v>
+        <v>3.044357246582948e-07</v>
       </c>
       <c r="D447" t="inlineStr">
         <is>
@@ -9952,7 +9952,7 @@
         </is>
       </c>
       <c r="C454" t="n">
-        <v>1.945389246930098e-06</v>
+        <v>1.945391474101507e-06</v>
       </c>
       <c r="D454" t="inlineStr">
         <is>
@@ -9994,7 +9994,7 @@
         </is>
       </c>
       <c r="C456" t="n">
-        <v>0.0002121548791940351</v>
+        <v>0.0002121544670339726</v>
       </c>
       <c r="D456" t="inlineStr">
         <is>
@@ -10120,7 +10120,7 @@
         </is>
       </c>
       <c r="C462" t="n">
-        <v>2.879673293259095e-07</v>
+        <v>2.879673296037115e-07</v>
       </c>
       <c r="D462" t="inlineStr">
         <is>
@@ -10141,7 +10141,7 @@
         </is>
       </c>
       <c r="C463" t="n">
-        <v>3.367245842451184e-05</v>
+        <v>3.367245850141367e-05</v>
       </c>
       <c r="D463" t="inlineStr">
         <is>
@@ -10183,7 +10183,7 @@
         </is>
       </c>
       <c r="C465" t="n">
-        <v>1.720221609381633e-05</v>
+        <v>1.720220235916246e-05</v>
       </c>
       <c r="D465" t="inlineStr">
         <is>
@@ -10246,7 +10246,7 @@
         </is>
       </c>
       <c r="C468" t="n">
-        <v>4.029957332166499e-07</v>
+        <v>4.030579621708958e-07</v>
       </c>
       <c r="D468" t="inlineStr">
         <is>
@@ -10267,7 +10267,7 @@
         </is>
       </c>
       <c r="C469" t="n">
-        <v>1.465269458058502e-07</v>
+        <v>1.465270040051596e-07</v>
       </c>
       <c r="D469" t="inlineStr">
         <is>
@@ -10330,7 +10330,7 @@
         </is>
       </c>
       <c r="C472" t="n">
-        <v>1.007504546556566e-07</v>
+        <v>1.007503624139611e-07</v>
       </c>
       <c r="D472" t="inlineStr">
         <is>
@@ -10372,7 +10372,7 @@
         </is>
       </c>
       <c r="C474" t="n">
-        <v>6.278904861846257e-07</v>
+        <v>6.278923955191283e-07</v>
       </c>
       <c r="D474" t="inlineStr">
         <is>
@@ -10393,7 +10393,7 @@
         </is>
       </c>
       <c r="C475" t="n">
-        <v>1.064699579999405e-08</v>
+        <v>1.064699871980877e-08</v>
       </c>
       <c r="D475" t="inlineStr">
         <is>
@@ -10414,7 +10414,7 @@
         </is>
       </c>
       <c r="C476" t="n">
-        <v>6.528428532523971e-07</v>
+        <v>6.528428742598873e-07</v>
       </c>
       <c r="D476" t="inlineStr">
         <is>
@@ -10435,7 +10435,7 @@
         </is>
       </c>
       <c r="C477" t="n">
-        <v>6.926304839996131e-09</v>
+        <v>6.926308160860092e-09</v>
       </c>
       <c r="D477" t="inlineStr">
         <is>
@@ -10477,7 +10477,7 @@
         </is>
       </c>
       <c r="C479" t="n">
-        <v>2.395345736579516e-06</v>
+        <v>2.395346690360567e-06</v>
       </c>
       <c r="D479" t="inlineStr">
         <is>
@@ -10498,7 +10498,7 @@
         </is>
       </c>
       <c r="C480" t="n">
-        <v>2.395345736579516e-06</v>
+        <v>2.395346690360567e-06</v>
       </c>
       <c r="D480" t="inlineStr">
         <is>
@@ -10540,7 +10540,7 @@
         </is>
       </c>
       <c r="C482" t="n">
-        <v>3.908024410665048e-06</v>
+        <v>3.908044896316404e-06</v>
       </c>
       <c r="D482" t="inlineStr">
         <is>
@@ -10582,7 +10582,7 @@
         </is>
       </c>
       <c r="C484" t="n">
-        <v>5.612518125604177e-05</v>
+        <v>5.612620157813168e-05</v>
       </c>
       <c r="D484" t="inlineStr">
         <is>
@@ -10624,7 +10624,7 @@
         </is>
       </c>
       <c r="C486" t="n">
-        <v>5.742044554222069e-05</v>
+        <v>5.742054796440197e-05</v>
       </c>
       <c r="D486" t="inlineStr">
         <is>
@@ -10666,7 +10666,7 @@
         </is>
       </c>
       <c r="C488" t="n">
-        <v>5.016487566594755e-06</v>
+        <v>5.01648838142386e-06</v>
       </c>
       <c r="D488" t="inlineStr">
         <is>
@@ -10729,7 +10729,7 @@
         </is>
       </c>
       <c r="C491" t="n">
-        <v>1.582567089894698e-05</v>
+        <v>1.582571588413967e-05</v>
       </c>
       <c r="D491" t="inlineStr">
         <is>
@@ -10771,7 +10771,7 @@
         </is>
       </c>
       <c r="C493" t="n">
-        <v>1.99496152286886e-05</v>
+        <v>1.994965778636271e-05</v>
       </c>
       <c r="D493" t="inlineStr">
         <is>
@@ -10813,7 +10813,7 @@
         </is>
       </c>
       <c r="C495" t="n">
-        <v>1.645441609710684e-05</v>
+        <v>1.645442219962944e-05</v>
       </c>
       <c r="D495" t="inlineStr">
         <is>
@@ -10834,7 +10834,7 @@
         </is>
       </c>
       <c r="C496" t="n">
-        <v>1.492085273254263e-06</v>
+        <v>1.492086334940044e-06</v>
       </c>
       <c r="D496" t="inlineStr">
         <is>
@@ -10855,7 +10855,7 @@
         </is>
       </c>
       <c r="C497" t="n">
-        <v>1.41651186798504e-07</v>
+        <v>1.416511913566238e-07</v>
       </c>
       <c r="D497" t="inlineStr">
         <is>
@@ -10876,7 +10876,7 @@
         </is>
       </c>
       <c r="C498" t="n">
-        <v>1.175453999999343e-09</v>
+        <v>1.175453998003097e-09</v>
       </c>
       <c r="D498" t="inlineStr">
         <is>
@@ -10960,7 +10960,7 @@
         </is>
       </c>
       <c r="C502" t="n">
-        <v>5.875392974474037e-07</v>
+        <v>5.875393733883862e-07</v>
       </c>
       <c r="D502" t="inlineStr">
         <is>
@@ -10981,7 +10981,7 @@
         </is>
       </c>
       <c r="C503" t="n">
-        <v>9.653352267073009e-06</v>
+        <v>9.653351113850163e-06</v>
       </c>
       <c r="D503" t="inlineStr">
         <is>
@@ -11002,7 +11002,7 @@
         </is>
       </c>
       <c r="C504" t="n">
-        <v>1.681996564325178e-07</v>
+        <v>1.6819955011567e-07</v>
       </c>
       <c r="D504" t="inlineStr">
         <is>
@@ -11023,7 +11023,7 @@
         </is>
       </c>
       <c r="C505" t="n">
-        <v>1.059344242318699e-05</v>
+        <v>1.059350210380923e-05</v>
       </c>
       <c r="D505" t="inlineStr">
         <is>
@@ -11065,7 +11065,7 @@
         </is>
       </c>
       <c r="C507" t="n">
-        <v>3.544771323958596e-07</v>
+        <v>3.544786688672783e-07</v>
       </c>
       <c r="D507" t="inlineStr">
         <is>
@@ -11107,7 +11107,7 @@
         </is>
       </c>
       <c r="C509" t="n">
-        <v>3.544771323958596e-07</v>
+        <v>3.544786688672783e-07</v>
       </c>
       <c r="D509" t="inlineStr">
         <is>
@@ -11149,7 +11149,7 @@
         </is>
       </c>
       <c r="C511" t="n">
-        <v>3.057968431008937e-06</v>
+        <v>3.057977541788223e-06</v>
       </c>
       <c r="D511" t="inlineStr">
         <is>
@@ -11170,7 +11170,7 @@
         </is>
       </c>
       <c r="C512" t="n">
-        <v>1.007178852028757e-05</v>
+        <v>1.007180190299907e-05</v>
       </c>
       <c r="D512" t="inlineStr">
         <is>
@@ -11212,7 +11212,7 @@
         </is>
       </c>
       <c r="C514" t="n">
-        <v>3.812995199999999e-10</v>
+        <v>3.812996820635818e-10</v>
       </c>
       <c r="D514" t="inlineStr">
         <is>
@@ -11254,7 +11254,7 @@
         </is>
       </c>
       <c r="C516" t="n">
-        <v>4.046773239311109e-06</v>
+        <v>4.046774681894313e-06</v>
       </c>
       <c r="D516" t="inlineStr">
         <is>
@@ -11296,7 +11296,7 @@
         </is>
       </c>
       <c r="C518" t="n">
-        <v>1.054302977088947e-06</v>
+        <v>1.054305208829647e-06</v>
       </c>
       <c r="D518" t="inlineStr">
         <is>
@@ -11317,7 +11317,7 @@
         </is>
       </c>
       <c r="C519" t="n">
-        <v>6.829346999999999e-12</v>
+        <v>6.829355544077037e-12</v>
       </c>
       <c r="D519" t="inlineStr">
         <is>
@@ -11422,7 +11422,7 @@
         </is>
       </c>
       <c r="C524" t="n">
-        <v>1.743847977761864e-05</v>
+        <v>1.743843642877246e-05</v>
       </c>
       <c r="D524" t="inlineStr">
         <is>
@@ -11443,7 +11443,7 @@
         </is>
       </c>
       <c r="C525" t="n">
-        <v>2.293131120235572e-06</v>
+        <v>2.293116097065482e-06</v>
       </c>
       <c r="D525" t="inlineStr">
         <is>
@@ -11464,7 +11464,7 @@
         </is>
       </c>
       <c r="C526" t="n">
-        <v>2.293131120235572e-06</v>
+        <v>2.293116097065482e-06</v>
       </c>
       <c r="D526" t="inlineStr">
         <is>
@@ -11485,7 +11485,7 @@
         </is>
       </c>
       <c r="C527" t="n">
-        <v>2.293131120235572e-06</v>
+        <v>2.293116097065482e-06</v>
       </c>
       <c r="D527" t="inlineStr">
         <is>
@@ -11506,7 +11506,7 @@
         </is>
       </c>
       <c r="C528" t="n">
-        <v>2.293131120235572e-06</v>
+        <v>2.293116097065482e-06</v>
       </c>
       <c r="D528" t="inlineStr">
         <is>
@@ -11548,7 +11548,7 @@
         </is>
       </c>
       <c r="C530" t="n">
-        <v>6.682233381236685e-05</v>
+        <v>6.682238039869929e-05</v>
       </c>
       <c r="D530" t="inlineStr">
         <is>
@@ -11569,7 +11569,7 @@
         </is>
       </c>
       <c r="C531" t="n">
-        <v>2.070847799999997e-10</v>
+        <v>2.070847483017488e-10</v>
       </c>
       <c r="D531" t="inlineStr">
         <is>
@@ -11590,7 +11590,7 @@
         </is>
       </c>
       <c r="C532" t="n">
-        <v>9.031667536242791e-07</v>
+        <v>9.031667275226668e-07</v>
       </c>
       <c r="D532" t="inlineStr">
         <is>
@@ -11611,7 +11611,7 @@
         </is>
       </c>
       <c r="C533" t="n">
-        <v>2.6674452e-09</v>
+        <v>2.667446193005024e-09</v>
       </c>
       <c r="D533" t="inlineStr">
         <is>
@@ -11632,7 +11632,7 @@
         </is>
       </c>
       <c r="C534" t="n">
-        <v>1.5844248e-08</v>
+        <v>1.584428432912243e-08</v>
       </c>
       <c r="D534" t="inlineStr">
         <is>
@@ -11653,7 +11653,7 @@
         </is>
       </c>
       <c r="C535" t="n">
-        <v>3.798658207251888e-08</v>
+        <v>3.798658193017692e-08</v>
       </c>
       <c r="D535" t="inlineStr">
         <is>
@@ -11716,7 +11716,7 @@
         </is>
       </c>
       <c r="C538" t="n">
-        <v>5.600506958785019e-06</v>
+        <v>5.600512441503721e-06</v>
       </c>
       <c r="D538" t="inlineStr">
         <is>
@@ -11758,7 +11758,7 @@
         </is>
       </c>
       <c r="C540" t="n">
-        <v>6.071787608848234e-07</v>
+        <v>6.071791338604164e-07</v>
       </c>
       <c r="D540" t="inlineStr">
         <is>
@@ -11821,7 +11821,7 @@
         </is>
       </c>
       <c r="C543" t="n">
-        <v>8.587724313972687e-06</v>
+        <v>8.58772141220754e-06</v>
       </c>
       <c r="D543" t="inlineStr">
         <is>
@@ -11842,7 +11842,7 @@
         </is>
       </c>
       <c r="C544" t="n">
-        <v>1.469688458087377e-06</v>
+        <v>1.469693422639303e-06</v>
       </c>
       <c r="D544" t="inlineStr">
         <is>
@@ -12073,7 +12073,7 @@
         </is>
       </c>
       <c r="C555" t="n">
-        <v>1.071554399999402e-10</v>
+        <v>1.071552271751719e-10</v>
       </c>
       <c r="D555" t="inlineStr">
         <is>
@@ -12157,7 +12157,7 @@
         </is>
       </c>
       <c r="C559" t="n">
-        <v>2.155568526370744e-08</v>
+        <v>2.155572732806756e-08</v>
       </c>
       <c r="D559" t="inlineStr">
         <is>
@@ -12178,7 +12178,7 @@
         </is>
       </c>
       <c r="C560" t="n">
-        <v>1.741157642776518e-07</v>
+        <v>1.741155341770887e-07</v>
       </c>
       <c r="D560" t="inlineStr">
         <is>
@@ -12199,7 +12199,7 @@
         </is>
       </c>
       <c r="C561" t="n">
-        <v>5.199670802410487e-06</v>
+        <v>5.199632191641318e-06</v>
       </c>
       <c r="D561" t="inlineStr">
         <is>
@@ -12220,7 +12220,7 @@
         </is>
       </c>
       <c r="C562" t="n">
-        <v>5.199670802410487e-06</v>
+        <v>5.199632191641318e-06</v>
       </c>
       <c r="D562" t="inlineStr">
         <is>
@@ -12241,7 +12241,7 @@
         </is>
       </c>
       <c r="C563" t="n">
-        <v>5.199670802410487e-06</v>
+        <v>5.199632191641318e-06</v>
       </c>
       <c r="D563" t="inlineStr">
         <is>
@@ -12283,7 +12283,7 @@
         </is>
       </c>
       <c r="C565" t="n">
-        <v>0</v>
+        <v>4.053861620850435e-12</v>
       </c>
       <c r="D565" t="inlineStr">
         <is>
@@ -12325,7 +12325,7 @@
         </is>
       </c>
       <c r="C567" t="n">
-        <v>4.121251366243645e-06</v>
+        <v>4.121326288118514e-06</v>
       </c>
       <c r="D567" t="inlineStr">
         <is>
@@ -12346,7 +12346,7 @@
         </is>
       </c>
       <c r="C568" t="n">
-        <v>1.007237251090191e-06</v>
+        <v>1.007255193646406e-06</v>
       </c>
       <c r="D568" t="inlineStr">
         <is>
@@ -12367,7 +12367,7 @@
         </is>
       </c>
       <c r="C569" t="n">
-        <v>1.007237251090191e-06</v>
+        <v>1.007255193646406e-06</v>
       </c>
       <c r="D569" t="inlineStr">
         <is>
@@ -12451,7 +12451,7 @@
         </is>
       </c>
       <c r="C573" t="n">
-        <v>5.001529765560712e-06</v>
+        <v>5.001606904387972e-06</v>
       </c>
       <c r="D573" t="inlineStr">
         <is>
@@ -12493,7 +12493,7 @@
         </is>
       </c>
       <c r="C575" t="n">
-        <v>3.015539087193188e-06</v>
+        <v>3.015536740923836e-06</v>
       </c>
       <c r="D575" t="inlineStr">
         <is>
@@ -12535,7 +12535,7 @@
         </is>
       </c>
       <c r="C577" t="n">
-        <v>3.87059904e-08</v>
+        <v>3.870599739681104e-08</v>
       </c>
       <c r="D577" t="inlineStr">
         <is>
@@ -12598,7 +12598,7 @@
         </is>
       </c>
       <c r="C580" t="n">
-        <v>1.539810183038258e-05</v>
+        <v>1.539813263562332e-05</v>
       </c>
       <c r="D580" t="inlineStr">
         <is>
@@ -12619,7 +12619,7 @@
         </is>
       </c>
       <c r="C581" t="n">
-        <v>2.664902839340428e-05</v>
+        <v>2.66490474239534e-05</v>
       </c>
       <c r="D581" t="inlineStr">
         <is>
@@ -12661,7 +12661,7 @@
         </is>
       </c>
       <c r="C583" t="n">
-        <v>3.009650337374911e-06</v>
+        <v>3.009663569317357e-06</v>
       </c>
       <c r="D583" t="inlineStr">
         <is>
@@ -12682,7 +12682,7 @@
         </is>
       </c>
       <c r="C584" t="n">
-        <v>9.515076596647862e-06</v>
+        <v>9.515074822337265e-06</v>
       </c>
       <c r="D584" t="inlineStr">
         <is>
@@ -12703,7 +12703,7 @@
         </is>
       </c>
       <c r="C585" t="n">
-        <v>2.664991576676624e-07</v>
+        <v>2.664987757340847e-07</v>
       </c>
       <c r="D585" t="inlineStr">
         <is>
@@ -12745,7 +12745,7 @@
         </is>
       </c>
       <c r="C587" t="n">
-        <v>3.398293525467515e-06</v>
+        <v>3.398292387844769e-06</v>
       </c>
       <c r="D587" t="inlineStr">
         <is>
@@ -12829,7 +12829,7 @@
         </is>
       </c>
       <c r="C591" t="n">
-        <v>1.186261502105196e-05</v>
+        <v>1.186261500616483e-05</v>
       </c>
       <c r="D591" t="inlineStr">
         <is>
@@ -12913,7 +12913,7 @@
         </is>
       </c>
       <c r="C595" t="n">
-        <v>5.996255999999999e-12</v>
+        <v>5.996244358676762e-12</v>
       </c>
       <c r="D595" t="inlineStr">
         <is>
@@ -12955,7 +12955,7 @@
         </is>
       </c>
       <c r="C597" t="n">
-        <v>1.640923742711345e-10</v>
+        <v>1.640923738568411e-10</v>
       </c>
       <c r="D597" t="inlineStr">
         <is>
@@ -12997,7 +12997,7 @@
         </is>
       </c>
       <c r="C599" t="n">
-        <v>5.563316569708118e-06</v>
+        <v>5.56332144833331e-06</v>
       </c>
       <c r="D599" t="inlineStr">
         <is>
@@ -13144,7 +13144,7 @@
         </is>
       </c>
       <c r="C606" t="n">
-        <v>1.541822813504304e-05</v>
+        <v>1.541822496358217e-05</v>
       </c>
       <c r="D606" t="inlineStr">
         <is>
@@ -13165,7 +13165,7 @@
         </is>
       </c>
       <c r="C607" t="n">
-        <v>9.506962317527578e-06</v>
+        <v>9.506961725251421e-06</v>
       </c>
       <c r="D607" t="inlineStr">
         <is>
@@ -13186,7 +13186,7 @@
         </is>
       </c>
       <c r="C608" t="n">
-        <v>9.506962317527578e-06</v>
+        <v>9.506961725251421e-06</v>
       </c>
       <c r="D608" t="inlineStr">
         <is>
@@ -13354,7 +13354,7 @@
         </is>
       </c>
       <c r="C616" t="n">
-        <v>2.980406935491899e-07</v>
+        <v>2.980410953077939e-07</v>
       </c>
       <c r="D616" t="inlineStr">
         <is>
@@ -13396,7 +13396,7 @@
         </is>
       </c>
       <c r="C618" t="n">
-        <v>3.330403817508616e-09</v>
+        <v>3.330410466950117e-09</v>
       </c>
       <c r="D618" t="inlineStr">
         <is>
@@ -13459,7 +13459,7 @@
         </is>
       </c>
       <c r="C621" t="n">
-        <v>1.64464152758854e-07</v>
+        <v>1.64463764180639e-07</v>
       </c>
       <c r="D621" t="inlineStr">
         <is>
@@ -13480,7 +13480,7 @@
         </is>
       </c>
       <c r="C622" t="n">
-        <v>1.204406279272523e-06</v>
+        <v>1.204406888012912e-06</v>
       </c>
       <c r="D622" t="inlineStr">
         <is>
@@ -13522,7 +13522,7 @@
         </is>
       </c>
       <c r="C624" t="n">
-        <v>2.460137982377643e-06</v>
+        <v>2.460137869865208e-06</v>
       </c>
       <c r="D624" t="inlineStr">
         <is>
@@ -13543,7 +13543,7 @@
         </is>
       </c>
       <c r="C625" t="n">
-        <v>4.948280078568954e-07</v>
+        <v>4.948281890454237e-07</v>
       </c>
       <c r="D625" t="inlineStr">
         <is>
@@ -13648,7 +13648,7 @@
         </is>
       </c>
       <c r="C630" t="n">
-        <v>5.431140932267016e-08</v>
+        <v>5.431154021550703e-08</v>
       </c>
       <c r="D630" t="inlineStr">
         <is>
@@ -13669,7 +13669,7 @@
         </is>
       </c>
       <c r="C631" t="n">
-        <v>1.263781464514027e-06</v>
+        <v>1.263781510951516e-06</v>
       </c>
       <c r="D631" t="inlineStr">
         <is>
@@ -13690,7 +13690,7 @@
         </is>
       </c>
       <c r="C632" t="n">
-        <v>5.039266493460497e-07</v>
+        <v>5.039267506412859e-07</v>
       </c>
       <c r="D632" t="inlineStr">
         <is>
@@ -13711,7 +13711,7 @@
         </is>
       </c>
       <c r="C633" t="n">
-        <v>9.305987680169555e-08</v>
+        <v>9.305980203279636e-08</v>
       </c>
       <c r="D633" t="inlineStr">
         <is>
@@ -13753,7 +13753,7 @@
         </is>
       </c>
       <c r="C635" t="n">
-        <v>4.271464610655406e-07</v>
+        <v>4.271464009363537e-07</v>
       </c>
       <c r="D635" t="inlineStr">
         <is>
@@ -13774,7 +13774,7 @@
         </is>
       </c>
       <c r="C636" t="n">
-        <v>2.478402023641762e-08</v>
+        <v>2.478397225738281e-08</v>
       </c>
       <c r="D636" t="inlineStr">
         <is>
@@ -13795,7 +13795,7 @@
         </is>
       </c>
       <c r="C637" t="n">
-        <v>3.824660392198842e-06</v>
+        <v>3.824661005826951e-06</v>
       </c>
       <c r="D637" t="inlineStr">
         <is>
@@ -14068,7 +14068,7 @@
         </is>
       </c>
       <c r="C650" t="n">
-        <v>1.297639553658393e-07</v>
+        <v>1.297639856315199e-07</v>
       </c>
       <c r="D650" t="inlineStr">
         <is>
@@ -14824,7 +14824,7 @@
         </is>
       </c>
       <c r="C686" t="n">
-        <v>1.644774296124644e-05</v>
+        <v>1.644774417094031e-05</v>
       </c>
       <c r="D686" t="inlineStr">
         <is>
@@ -14887,7 +14887,7 @@
         </is>
       </c>
       <c r="C689" t="n">
-        <v>1.765070477114412e-05</v>
+        <v>1.765058582630066e-05</v>
       </c>
       <c r="D689" t="inlineStr">
         <is>
@@ -14992,7 +14992,7 @@
         </is>
       </c>
       <c r="C694" t="n">
-        <v>3.97443079437488e-06</v>
+        <v>3.974436774809531e-06</v>
       </c>
       <c r="D694" t="inlineStr">
         <is>
@@ -15034,7 +15034,7 @@
         </is>
       </c>
       <c r="C696" t="n">
-        <v>8.032178186298482e-05</v>
+        <v>8.032157081072058e-05</v>
       </c>
       <c r="D696" t="inlineStr">
         <is>
@@ -15265,7 +15265,7 @@
         </is>
       </c>
       <c r="C707" t="n">
-        <v>5.973364256912587e-05</v>
+        <v>5.973376052435517e-05</v>
       </c>
       <c r="D707" t="inlineStr">
         <is>
@@ -15412,7 +15412,7 @@
         </is>
       </c>
       <c r="C714" t="n">
-        <v>8.464855054655785e-06</v>
+        <v>8.46485505117639e-06</v>
       </c>
       <c r="D714" t="inlineStr">
         <is>
@@ -15496,7 +15496,7 @@
         </is>
       </c>
       <c r="C718" t="n">
-        <v>8.853130776000001e-10</v>
+        <v>8.853128628454521e-10</v>
       </c>
       <c r="D718" t="inlineStr">
         <is>
@@ -15559,7 +15559,7 @@
         </is>
       </c>
       <c r="C721" t="n">
-        <v>3.934874999999999e-10</v>
+        <v>3.934875373017703e-10</v>
       </c>
       <c r="D721" t="inlineStr">
         <is>
@@ -15643,7 +15643,7 @@
         </is>
       </c>
       <c r="C725" t="n">
-        <v>5.212744102435525e-09</v>
+        <v>5.207236690180368e-09</v>
       </c>
       <c r="D725" t="inlineStr">
         <is>
@@ -15748,7 +15748,7 @@
         </is>
       </c>
       <c r="C730" t="n">
-        <v>3.985716113724323e-08</v>
+        <v>3.985710209236246e-08</v>
       </c>
       <c r="D730" t="inlineStr">
         <is>
@@ -15832,7 +15832,7 @@
         </is>
       </c>
       <c r="C734" t="n">
-        <v>4.921512027174268e-08</v>
+        <v>4.921556117187967e-08</v>
       </c>
       <c r="D734" t="inlineStr">
         <is>
@@ -15874,7 +15874,7 @@
         </is>
       </c>
       <c r="C736" t="n">
-        <v>3.38985003625763e-08</v>
+        <v>3.389848512980349e-08</v>
       </c>
       <c r="D736" t="inlineStr">
         <is>
@@ -15895,7 +15895,7 @@
         </is>
       </c>
       <c r="C737" t="n">
-        <v>2.343595728350238e-05</v>
+        <v>2.343596848879036e-05</v>
       </c>
       <c r="D737" t="inlineStr">
         <is>
@@ -15979,7 +15979,7 @@
         </is>
       </c>
       <c r="C741" t="n">
-        <v>0.0002645283350658781</v>
+        <v>0.0002645272296063229</v>
       </c>
       <c r="D741" t="inlineStr">
         <is>
@@ -16105,7 +16105,7 @@
         </is>
       </c>
       <c r="C747" t="n">
-        <v>3.54547599e-08</v>
+        <v>3.545468167733681e-08</v>
       </c>
       <c r="D747" t="inlineStr">
         <is>
@@ -16210,7 +16210,7 @@
         </is>
       </c>
       <c r="C752" t="n">
-        <v>2.427543057984973e-06</v>
+        <v>2.427577559709353e-06</v>
       </c>
       <c r="D752" t="inlineStr">
         <is>
@@ -17239,7 +17239,7 @@
         </is>
       </c>
       <c r="C801" t="n">
-        <v>1.708840842484271e-07</v>
+        <v>1.708843101827301e-07</v>
       </c>
       <c r="D801" t="inlineStr">
         <is>
@@ -18709,7 +18709,7 @@
         </is>
       </c>
       <c r="C871" t="n">
-        <v>3.709818583790847e-08</v>
+        <v>3.709818471414543e-08</v>
       </c>
       <c r="D871" t="inlineStr">
         <is>
@@ -18730,7 +18730,7 @@
         </is>
       </c>
       <c r="C872" t="n">
-        <v>5.139594767999999e-09</v>
+        <v>5.13958778242029e-09</v>
       </c>
       <c r="D872" t="inlineStr">
         <is>

</xml_diff>